<commit_message>
Atualiza dashboards Aura - 2026-06-09 10:54:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5776,7 +5776,7 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5884,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-09 14:29:03
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -4927,7 +4927,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 09:00</t>
         </is>
       </c>
     </row>
@@ -9623,7 +9623,7 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 12:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-09 15:46:32
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$404</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$405</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F404"/>
+  <dimension ref="A1:F405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -975,7 +975,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 11:40</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,11 @@
           <t>BA</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>A8210</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
           <t>00019200000012729507</t>
@@ -2010,7 +2014,11 @@
           <t>ES</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>TA0575</t>
+        </is>
+      </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
           <t>00019200000012720992</t>
@@ -2774,7 +2782,11 @@
           <t>GO</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>TA0218</t>
+        </is>
+      </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
           <t>00019200000012719986</t>
@@ -3075,7 +3087,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3119,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5067,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:14</t>
         </is>
       </c>
     </row>
@@ -5230,10 +5242,14 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr"/>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>A5580</t>
+        </is>
+      </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714585</t>
+          <t>00019200000012714577</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
@@ -5250,39 +5266,39 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>555906</t>
+          <t>556173</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>TA1064</t>
+          <t>A4423</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718556</t>
+          <t>00019200000012714585</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:51</t>
+          <t>06/06/2026 09:17</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>556105</t>
+          <t>555906</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -5292,17 +5308,17 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>A0431</t>
+          <t>TA1064</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>00019200000012717614</t>
+          <t>00019200000012718556</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 22:37</t>
+          <t>07/06/2026 22:51</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -5314,7 +5330,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>556187</t>
+          <t>556105</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -5324,54 +5340,54 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>A8822</t>
+          <t>A0431</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864242</t>
+          <t>00019200000012717614</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 21:57</t>
+          <t>08/06/2026 22:37</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 13:07</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>556113</t>
+          <t>556187</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>A9365</t>
+          <t>A8822</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714593</t>
+          <t>00019200000012864242</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:53</t>
+          <t>02/06/2026 21:57</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>04/06/2026 13:07</t>
         </is>
       </c>
     </row>
@@ -5388,12 +5404,12 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>A7132</t>
+          <t>A9365</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714607</t>
+          <t>00019200000012714593</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -5420,12 +5436,12 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>A6834</t>
+          <t>A7132</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714615</t>
+          <t>00019200000012714607</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
@@ -5452,12 +5468,12 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>A8249</t>
+          <t>A6834</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714623</t>
+          <t>00019200000012714615</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
@@ -5484,12 +5500,12 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>A8816</t>
+          <t>A8249</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714640</t>
+          <t>00019200000012714623</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -5506,7 +5522,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>556339</t>
+          <t>556113</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -5516,17 +5532,17 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>A7748</t>
+          <t>A8816</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729124</t>
+          <t>00019200000012714640</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 03:51</t>
+          <t>08/06/2026 10:53</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -5538,7 +5554,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>556549</t>
+          <t>556339</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -5548,17 +5564,17 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>A7654</t>
+          <t>A7748</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730505</t>
+          <t>00019200000012729124</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:31</t>
+          <t>09/06/2026 03:51</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -5570,39 +5586,39 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>20260717</t>
+          <t>556549</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>A5970</t>
+          <t>A7654</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721034</t>
+          <t>00019200000012730505</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:14</t>
+          <t>08/06/2026 05:31</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 13:12</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>556743</t>
+          <t>20260717</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -5612,54 +5628,54 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>A7321</t>
+          <t>A5970</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723487</t>
+          <t>00019200000012721034</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:50</t>
+          <t>02/06/2026 01:14</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:50</t>
+          <t>03/06/2026 13:12</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>556083</t>
+          <t>556743</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>A5844</t>
+          <t>A7321</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721867</t>
+          <t>00019200000012723487</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:05</t>
+          <t>07/06/2026 22:50</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 17:29</t>
+          <t>09/06/2026 10:50</t>
         </is>
       </c>
     </row>
@@ -5676,12 +5692,12 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>A4723</t>
+          <t>A5844</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721891</t>
+          <t>00019200000012721867</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
@@ -5698,7 +5714,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>556294</t>
+          <t>556083</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -5708,22 +5724,22 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>A3519</t>
+          <t>A4723</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714704</t>
+          <t>00019200000012721891</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 13:37</t>
+          <t>01/06/2026 22:05</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 16:38</t>
+          <t>03/06/2026 17:29</t>
         </is>
       </c>
     </row>
@@ -5740,12 +5756,12 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>A9135</t>
+          <t>A3519</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714712</t>
+          <t>00019200000012714704</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
@@ -5772,12 +5788,12 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>TA0487</t>
+          <t>A9135</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714720</t>
+          <t>00019200000012714712</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
@@ -5804,12 +5820,12 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>TA1114</t>
+          <t>TA0487</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714739</t>
+          <t>00019200000012714720</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
@@ -5836,12 +5852,12 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>A8445</t>
+          <t>TA1114</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714747</t>
+          <t>00019200000012714739</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
@@ -5868,12 +5884,12 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>A6194</t>
+          <t>A8445</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714763</t>
+          <t>00019200000012714747</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
@@ -5900,12 +5916,12 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>A9186</t>
+          <t>A6194</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714771</t>
+          <t>00019200000012714763</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -5930,10 +5946,14 @@
           <t>RN</t>
         </is>
       </c>
-      <c r="C173" s="2" t="inlineStr"/>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>A9186</t>
+        </is>
+      </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714780</t>
+          <t>00019200000012714771</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -5960,12 +5980,12 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>A0774</t>
+          <t>A8034</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714798</t>
+          <t>00019200000012714780</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -5992,12 +6012,12 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>A8373</t>
+          <t>A0774</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714801</t>
+          <t>00019200000012714798</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -6024,12 +6044,12 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>A8792</t>
+          <t>A8373</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714810</t>
+          <t>00019200000012714801</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
@@ -6056,12 +6076,12 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>A0162</t>
+          <t>A8792</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714828</t>
+          <t>00019200000012714810</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -6078,39 +6098,39 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>555911</t>
+          <t>556294</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>A4881</t>
+          <t>A0162</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715298</t>
+          <t>00019200000012714828</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:02</t>
+          <t>02/06/2026 13:37</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>03/06/2026 16:38</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>556157</t>
+          <t>555911</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -6120,12 +6140,12 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>TA0188</t>
+          <t>A4881</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730203</t>
+          <t>00019200000012715298</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
@@ -6152,12 +6172,12 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>TA0670</t>
+          <t>TA0188</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730211</t>
+          <t>00019200000012730203</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -6184,12 +6204,12 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>A3810</t>
+          <t>TA0670</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730220</t>
+          <t>00019200000012730211</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
@@ -6216,12 +6236,12 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>A0800</t>
+          <t>A3810</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730238</t>
+          <t>00019200000012730220</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -6248,12 +6268,12 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>A5751</t>
+          <t>A0800</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730246</t>
+          <t>00019200000012730238</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -6280,12 +6300,12 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>A3830</t>
+          <t>A5751</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730254</t>
+          <t>00019200000012730246</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -6312,12 +6332,12 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>A2419</t>
+          <t>A3830</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730262</t>
+          <t>00019200000012730254</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -6344,12 +6364,12 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>A7535</t>
+          <t>A2419</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730270</t>
+          <t>00019200000012730262</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
@@ -6376,12 +6396,12 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>A5563</t>
+          <t>A7535</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730289</t>
+          <t>00019200000012730270</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -6408,12 +6428,12 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>A9066</t>
+          <t>A5563</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730297</t>
+          <t>00019200000012730289</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
@@ -6440,12 +6460,12 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>A5828</t>
+          <t>A9066</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730300</t>
+          <t>00019200000012730297</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
@@ -6472,12 +6492,12 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>A4055</t>
+          <t>A5828</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730319</t>
+          <t>00019200000012730300</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
@@ -6504,12 +6524,12 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>A0130</t>
+          <t>A4055</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730327</t>
+          <t>00019200000012730319</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
@@ -6536,12 +6556,12 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>A7797</t>
+          <t>A0130</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730335</t>
+          <t>00019200000012730327</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
@@ -6568,12 +6588,12 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>A9654</t>
+          <t>A7797</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730343</t>
+          <t>00019200000012730335</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
@@ -6600,12 +6620,12 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>A7482</t>
+          <t>A9654</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730351</t>
+          <t>00019200000012730343</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
@@ -6632,12 +6652,12 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>A7723</t>
+          <t>A7482</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730360</t>
+          <t>00019200000012730351</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -6664,12 +6684,12 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>A7997</t>
+          <t>A7723</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730378</t>
+          <t>00019200000012730360</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -6686,7 +6706,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>556258</t>
+          <t>556157</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -6696,17 +6716,17 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>A6961</t>
+          <t>A7997</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729159</t>
+          <t>00019200000012730378</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>06/06/2026 05:02</t>
         </is>
       </c>
       <c r="F197" s="2" t="inlineStr">
@@ -6718,22 +6738,22 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>556158</t>
+          <t>556258</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>A8351</t>
+          <t>A6961</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715344</t>
+          <t>00019200000012729159</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -6743,7 +6763,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6760,12 +6780,12 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>A6522</t>
+          <t>A8351</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715352</t>
+          <t>00019200000012715344</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
@@ -6792,12 +6812,12 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>A7263</t>
+          <t>A6522</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715360</t>
+          <t>00019200000012715352</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
@@ -6824,12 +6844,12 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>A9019</t>
+          <t>A7263</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715379</t>
+          <t>00019200000012715360</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
@@ -6856,12 +6876,12 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>A4823</t>
+          <t>A9019</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715387</t>
+          <t>00019200000012715379</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
@@ -6888,12 +6908,12 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>A5775</t>
+          <t>A4823</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715395</t>
+          <t>00019200000012715387</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
@@ -6920,12 +6940,12 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>A6931</t>
+          <t>A5775</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715409</t>
+          <t>00019200000012715395</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
@@ -6942,32 +6962,32 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>556159</t>
+          <t>556158</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>TA1119</t>
+          <t>A6931</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753440</t>
+          <t>00019200000012715409</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:08</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -6984,12 +7004,12 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>A6893</t>
+          <t>TA1119</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753459</t>
+          <t>00019200000012753440</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
@@ -7016,12 +7036,12 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>A8127</t>
+          <t>A6893</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753467</t>
+          <t>00019200000012753459</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
@@ -7048,12 +7068,12 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>A6189</t>
+          <t>A8127</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753475</t>
+          <t>00019200000012753467</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
@@ -7080,12 +7100,12 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>TA0776</t>
+          <t>A6189</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753483</t>
+          <t>00019200000012753475</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
@@ -7112,12 +7132,12 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>A8534</t>
+          <t>TA0776</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753491</t>
+          <t>00019200000012753483</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
@@ -7144,12 +7164,12 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>A7575</t>
+          <t>A8534</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753505</t>
+          <t>00019200000012753491</t>
         </is>
       </c>
       <c r="E211" s="2" t="inlineStr">
@@ -7176,12 +7196,12 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>A0609</t>
+          <t>A7575</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753513</t>
+          <t>00019200000012753505</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
@@ -7208,12 +7228,12 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>A9499</t>
+          <t>A0609</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753521</t>
+          <t>00019200000012753513</t>
         </is>
       </c>
       <c r="E213" s="2" t="inlineStr">
@@ -7240,12 +7260,12 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>A6581</t>
+          <t>A9499</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753530</t>
+          <t>00019200000012753521</t>
         </is>
       </c>
       <c r="E214" s="2" t="inlineStr">
@@ -7272,12 +7292,12 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>A8536</t>
+          <t>A6581</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753548</t>
+          <t>00019200000012753530</t>
         </is>
       </c>
       <c r="E215" s="2" t="inlineStr">
@@ -7304,12 +7324,12 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>A9316</t>
+          <t>A8536</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753556</t>
+          <t>00019200000012753548</t>
         </is>
       </c>
       <c r="E216" s="2" t="inlineStr">
@@ -7336,12 +7356,12 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>TA0880</t>
+          <t>A9316</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753564</t>
+          <t>00019200000012753556</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
@@ -7368,12 +7388,12 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>A1933</t>
+          <t>TA0880</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753572</t>
+          <t>00019200000012753564</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
@@ -7400,12 +7420,12 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>A0504</t>
+          <t>A1933</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753882</t>
+          <t>00019200000012753572</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
@@ -7432,12 +7452,12 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>TA0704</t>
+          <t>A0504</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753890</t>
+          <t>00019200000012753882</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
@@ -7464,12 +7484,12 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>A8967</t>
+          <t>TA0704</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753904</t>
+          <t>00019200000012753890</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -7496,12 +7516,12 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>A4337</t>
+          <t>A8967</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753912</t>
+          <t>00019200000012753904</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -7528,12 +7548,12 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>A5175</t>
+          <t>A4337</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753920</t>
+          <t>00019200000012753912</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -7560,12 +7580,12 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>TA0974</t>
+          <t>A5175</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753939</t>
+          <t>00019200000012753920</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -7592,12 +7612,12 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>A6700</t>
+          <t>TA0974</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753947</t>
+          <t>00019200000012753939</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -7624,12 +7644,12 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>A8361</t>
+          <t>A6700</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753955</t>
+          <t>00019200000012753947</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -7656,12 +7676,12 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>A3121</t>
+          <t>A8361</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753963</t>
+          <t>00019200000012753955</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -7688,12 +7708,12 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>A8154</t>
+          <t>A3121</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753971</t>
+          <t>00019200000012753963</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -7720,12 +7740,12 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>TA0597</t>
+          <t>A8154</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753980</t>
+          <t>00019200000012753971</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -7752,12 +7772,12 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>A6883</t>
+          <t>TA0597</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753998</t>
+          <t>00019200000012753980</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -7784,12 +7804,12 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>A9704</t>
+          <t>A6883</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754005</t>
+          <t>00019200000012753998</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -7816,12 +7836,12 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>A9302</t>
+          <t>A9704</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754013</t>
+          <t>00019200000012754005</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
@@ -7848,12 +7868,12 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>A0119</t>
+          <t>A9302</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754021</t>
+          <t>00019200000012754013</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
@@ -7880,12 +7900,12 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>A9040</t>
+          <t>A0119</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754048</t>
+          <t>00019200000012754021</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -7912,12 +7932,12 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>A7876</t>
+          <t>A9040</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754056</t>
+          <t>00019200000012754048</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
@@ -7944,12 +7964,12 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>A8919</t>
+          <t>A7876</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754064</t>
+          <t>00019200000012754056</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -7976,12 +7996,12 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>A6393</t>
+          <t>A8919</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754072</t>
+          <t>00019200000012754064</t>
         </is>
       </c>
       <c r="E237" s="2" t="inlineStr">
@@ -8008,12 +8028,12 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>A4317</t>
+          <t>A6393</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754080</t>
+          <t>00019200000012754072</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
@@ -8040,12 +8060,12 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>A8657</t>
+          <t>A4317</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754099</t>
+          <t>00019200000012754080</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
@@ -8072,12 +8092,12 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>A8940</t>
+          <t>A8657</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754102</t>
+          <t>00019200000012754099</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
@@ -8104,12 +8124,12 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>A6261</t>
+          <t>A8940</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754110</t>
+          <t>00019200000012754102</t>
         </is>
       </c>
       <c r="E241" s="2" t="inlineStr">
@@ -8136,12 +8156,12 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>A5569</t>
+          <t>A6261</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754129</t>
+          <t>00019200000012754110</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
@@ -8168,12 +8188,12 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>A8748</t>
+          <t>A5569</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754137</t>
+          <t>00019200000012754129</t>
         </is>
       </c>
       <c r="E243" s="2" t="inlineStr">
@@ -8200,12 +8220,12 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>A9213</t>
+          <t>A8748</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754145</t>
+          <t>00019200000012754137</t>
         </is>
       </c>
       <c r="E244" s="2" t="inlineStr">
@@ -8232,12 +8252,12 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>TA0226</t>
+          <t>A9213</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754153</t>
+          <t>00019200000012754145</t>
         </is>
       </c>
       <c r="E245" s="2" t="inlineStr">
@@ -8264,12 +8284,12 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>A8485</t>
+          <t>TA0226</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754161</t>
+          <t>00019200000012754153</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
@@ -8296,12 +8316,12 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>A8095</t>
+          <t>A8485</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754170</t>
+          <t>00019200000012754161</t>
         </is>
       </c>
       <c r="E247" s="2" t="inlineStr">
@@ -8328,12 +8348,12 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>A9152</t>
+          <t>A8095</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754188</t>
+          <t>00019200000012754170</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
@@ -8360,12 +8380,12 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>A7849</t>
+          <t>A9152</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754196</t>
+          <t>00019200000012754188</t>
         </is>
       </c>
       <c r="E249" s="2" t="inlineStr">
@@ -8392,12 +8412,12 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>A6854</t>
+          <t>A7849</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754200</t>
+          <t>00019200000012754196</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
@@ -8424,12 +8444,12 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>A8670</t>
+          <t>A6854</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754218</t>
+          <t>00019200000012754200</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
@@ -8456,12 +8476,12 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>A8352</t>
+          <t>A8670</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754226</t>
+          <t>00019200000012754218</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
@@ -8488,12 +8508,12 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>A6584</t>
+          <t>A8352</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754234</t>
+          <t>00019200000012754226</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
@@ -8520,12 +8540,12 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>A5394</t>
+          <t>A6584</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754242</t>
+          <t>00019200000012754234</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
@@ -8552,12 +8572,12 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>A9258</t>
+          <t>A5394</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754250</t>
+          <t>00019200000012754242</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
@@ -8584,12 +8604,12 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>A2475</t>
+          <t>A9258</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754269</t>
+          <t>00019200000012754250</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
@@ -8616,12 +8636,12 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>A8952</t>
+          <t>A2475</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754277</t>
+          <t>00019200000012754269</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
@@ -8648,12 +8668,12 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>A6781</t>
+          <t>A8952</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754285</t>
+          <t>00019200000012754277</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
@@ -8680,12 +8700,12 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>A8379</t>
+          <t>A6781</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754293</t>
+          <t>00019200000012754285</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
@@ -8712,12 +8732,12 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>A8243</t>
+          <t>A8379</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754307</t>
+          <t>00019200000012754293</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
@@ -8744,12 +8764,12 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>A7097</t>
+          <t>A8243</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754315</t>
+          <t>00019200000012754307</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
@@ -8776,12 +8796,12 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>TA0235</t>
+          <t>A7097</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754323</t>
+          <t>00019200000012754315</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
@@ -8808,12 +8828,12 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>A8222</t>
+          <t>TA0235</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754331</t>
+          <t>00019200000012754323</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
@@ -8840,12 +8860,12 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>A1510</t>
+          <t>A8222</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754340</t>
+          <t>00019200000012754331</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
@@ -8872,12 +8892,12 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>A0773</t>
+          <t>A1510</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754358</t>
+          <t>00019200000012754340</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
@@ -8904,12 +8924,12 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>A8448</t>
+          <t>A0773</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754366</t>
+          <t>00019200000012754358</t>
         </is>
       </c>
       <c r="E266" s="2" t="inlineStr">
@@ -8936,12 +8956,12 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>A7767</t>
+          <t>A8448</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754374</t>
+          <t>00019200000012754366</t>
         </is>
       </c>
       <c r="E267" s="2" t="inlineStr">
@@ -8968,12 +8988,12 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>A8254</t>
+          <t>A7767</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754382</t>
+          <t>00019200000012754374</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
@@ -9000,12 +9020,12 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>A9361</t>
+          <t>A8254</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754390</t>
+          <t>00019200000012754382</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
@@ -9032,12 +9052,12 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>A5087</t>
+          <t>A9361</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754404</t>
+          <t>00019200000012754390</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
@@ -9064,12 +9084,12 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>A0387</t>
+          <t>A5087</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754412</t>
+          <t>00019200000012754404</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
@@ -9096,12 +9116,12 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>A6996</t>
+          <t>A0387</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754420</t>
+          <t>00019200000012754412</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
@@ -9128,12 +9148,12 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>A7094</t>
+          <t>A6996</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754439</t>
+          <t>00019200000012754420</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
@@ -9160,12 +9180,12 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>A7194</t>
+          <t>A7094</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754447</t>
+          <t>00019200000012754439</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
@@ -9192,12 +9212,12 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>A6941</t>
+          <t>A7194</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754455</t>
+          <t>00019200000012754447</t>
         </is>
       </c>
       <c r="E275" s="2" t="inlineStr">
@@ -9224,12 +9244,12 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>A6571</t>
+          <t>A6941</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754463</t>
+          <t>00019200000012754455</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
@@ -9256,12 +9276,12 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>A5633</t>
+          <t>A6571</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754471</t>
+          <t>00019200000012754463</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
@@ -9288,12 +9308,12 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>A9483</t>
+          <t>A5633</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754480</t>
+          <t>00019200000012754471</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
@@ -9320,12 +9340,12 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>A9277</t>
+          <t>A9483</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754498</t>
+          <t>00019200000012754480</t>
         </is>
       </c>
       <c r="E279" s="2" t="inlineStr">
@@ -9352,12 +9372,12 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>A6305</t>
+          <t>A9277</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754501</t>
+          <t>00019200000012754498</t>
         </is>
       </c>
       <c r="E280" s="2" t="inlineStr">
@@ -9384,12 +9404,12 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>A0745</t>
+          <t>A6305</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754510</t>
+          <t>00019200000012754501</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
@@ -9416,12 +9436,12 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>A7451</t>
+          <t>A0745</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755958</t>
+          <t>00019200000012754510</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
@@ -9448,12 +9468,12 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>A9324</t>
+          <t>A7451</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755966</t>
+          <t>00019200000012755958</t>
         </is>
       </c>
       <c r="E283" s="2" t="inlineStr">
@@ -9480,12 +9500,12 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>A8491</t>
+          <t>A9324</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755974</t>
+          <t>00019200000012755966</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
@@ -9512,12 +9532,12 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>A9490</t>
+          <t>A8491</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755982</t>
+          <t>00019200000012755974</t>
         </is>
       </c>
       <c r="E285" s="2" t="inlineStr">
@@ -9544,12 +9564,12 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>A9202</t>
+          <t>A9490</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755990</t>
+          <t>00019200000012755982</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
@@ -9576,12 +9596,12 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>A5679</t>
+          <t>A9202</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>00019200000012756008</t>
+          <t>00019200000012755990</t>
         </is>
       </c>
       <c r="E287" s="2" t="inlineStr">
@@ -9598,7 +9618,7 @@
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>556744</t>
+          <t>556159</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
@@ -9608,54 +9628,54 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>A6519</t>
+          <t>A5679</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723479</t>
+          <t>00019200000012756008</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:33</t>
+          <t>09/06/2026 09:08</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 12:15</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>556160</t>
+          <t>556744</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>A9538</t>
+          <t>A6519</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730009</t>
+          <t>00019200000012723479</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 11:33</t>
+          <t>08/06/2026 05:33</t>
         </is>
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 11:46</t>
+          <t>09/06/2026 12:15</t>
         </is>
       </c>
     </row>
@@ -9672,12 +9692,12 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>TA0617</t>
+          <t>A9538</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730882</t>
+          <t>00019200000012730009</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
@@ -9704,12 +9724,12 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>A5841</t>
+          <t>TA0617</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730890</t>
+          <t>00019200000012730882</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
@@ -9736,12 +9756,12 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>A7704</t>
+          <t>A5841</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730904</t>
+          <t>00019200000012730890</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -9768,12 +9788,12 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>A6707</t>
+          <t>A7704</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730912</t>
+          <t>00019200000012730904</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -9798,10 +9818,14 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C294" s="2" t="inlineStr"/>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>A6707</t>
+        </is>
+      </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730920</t>
+          <t>00019200000012730912</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
@@ -9826,14 +9850,10 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C295" s="2" t="inlineStr">
-        <is>
-          <t>A5971</t>
-        </is>
-      </c>
+      <c r="C295" s="2" t="inlineStr"/>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730939</t>
+          <t>00019200000012730920</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
@@ -9860,12 +9880,12 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A5971</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731005</t>
+          <t>00019200000012730939</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
@@ -9892,12 +9912,12 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>A7331</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731560</t>
+          <t>00019200000012731005</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
@@ -9924,12 +9944,12 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>A2361</t>
+          <t>A7331</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731579</t>
+          <t>00019200000012731560</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
@@ -9956,12 +9976,12 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>A9716</t>
+          <t>A2361</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731587</t>
+          <t>00019200000012731579</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
@@ -9988,12 +10008,12 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>A9274</t>
+          <t>A9716</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731595</t>
+          <t>00019200000012731587</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
@@ -10020,12 +10040,12 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>A7020</t>
+          <t>A9274</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731609</t>
+          <t>00019200000012731595</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
@@ -10052,12 +10072,12 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>A8090</t>
+          <t>A7020</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731617</t>
+          <t>00019200000012731609</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
@@ -10084,12 +10104,12 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>A2173</t>
+          <t>A8090</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731625</t>
+          <t>00019200000012731617</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
@@ -10116,12 +10136,12 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>A5456</t>
+          <t>A2173</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731633</t>
+          <t>00019200000012731625</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
@@ -10148,12 +10168,12 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>A8993</t>
+          <t>A5456</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731641</t>
+          <t>00019200000012731633</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
@@ -10180,12 +10200,12 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>A7043</t>
+          <t>A8993</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731650</t>
+          <t>00019200000012731641</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
@@ -10212,12 +10232,12 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>A6600</t>
+          <t>A7043</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731668</t>
+          <t>00019200000012731650</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
@@ -10244,12 +10264,12 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>A6518</t>
+          <t>A6600</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731676</t>
+          <t>00019200000012731668</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
@@ -10276,12 +10296,12 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>A6804</t>
+          <t>A6518</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731684</t>
+          <t>00019200000012731676</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
@@ -10308,12 +10328,12 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>A1679</t>
+          <t>A6804</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731692</t>
+          <t>00019200000012731684</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
@@ -10340,12 +10360,12 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>A6311</t>
+          <t>A1679</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731803</t>
+          <t>00019200000012731692</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
@@ -10372,12 +10392,12 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>TA0484</t>
+          <t>A6311</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731900</t>
+          <t>00019200000012731803</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
@@ -10404,12 +10424,12 @@
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>A9205</t>
+          <t>TA0484</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731919</t>
+          <t>00019200000012731900</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
@@ -10436,12 +10456,12 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>A1019</t>
+          <t>A9205</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731927</t>
+          <t>00019200000012731919</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
@@ -10468,12 +10488,12 @@
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>A6694</t>
+          <t>A1019</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731935</t>
+          <t>00019200000012731927</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
@@ -10500,12 +10520,12 @@
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>A4625</t>
+          <t>A6694</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731943</t>
+          <t>00019200000012731935</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
@@ -10532,12 +10552,12 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>A7288</t>
+          <t>A4625</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731951</t>
+          <t>00019200000012731943</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
@@ -10564,12 +10584,12 @@
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>A7878</t>
+          <t>A7288</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731960</t>
+          <t>00019200000012731951</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
@@ -10596,12 +10616,12 @@
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>A0974</t>
+          <t>A7878</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731978</t>
+          <t>00019200000012731960</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
@@ -10628,12 +10648,12 @@
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>A8869</t>
+          <t>A0974</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731986</t>
+          <t>00019200000012731978</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
@@ -10660,12 +10680,12 @@
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>A7491</t>
+          <t>A8869</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731994</t>
+          <t>00019200000012731986</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
@@ -10692,12 +10712,12 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>A6871</t>
+          <t>A7491</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732001</t>
+          <t>00019200000012731994</t>
         </is>
       </c>
       <c r="E322" s="2" t="inlineStr">
@@ -10724,12 +10744,12 @@
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>A1824</t>
+          <t>A6871</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732010</t>
+          <t>00019200000012732001</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
@@ -10756,12 +10776,12 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A1824</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732028</t>
+          <t>00019200000012732010</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
@@ -10788,12 +10808,12 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>A9638</t>
+          <t>A9207</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732036</t>
+          <t>00019200000012732028</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
@@ -10820,12 +10840,12 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>TA1173</t>
+          <t>A9638</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732044</t>
+          <t>00019200000012732036</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -10852,12 +10872,12 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>A9280</t>
+          <t>TA1173</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732052</t>
+          <t>00019200000012732044</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
@@ -10884,12 +10904,12 @@
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>A6843</t>
+          <t>A9280</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732060</t>
+          <t>00019200000012732052</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -10916,12 +10936,12 @@
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>A8045</t>
+          <t>A6843</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732079</t>
+          <t>00019200000012732060</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
@@ -10948,12 +10968,12 @@
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A8045</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732087</t>
+          <t>00019200000012732079</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
@@ -10980,12 +11000,12 @@
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>A1989</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732095</t>
+          <t>00019200000012732087</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
@@ -11012,12 +11032,12 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>TA0654</t>
+          <t>A1989</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732109</t>
+          <t>00019200000012732095</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
@@ -11044,12 +11064,12 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>A4447</t>
+          <t>TA0654</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732117</t>
+          <t>00019200000012732109</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -11076,12 +11096,12 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>A8046</t>
+          <t>A4447</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732125</t>
+          <t>00019200000012732117</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -11108,12 +11128,12 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>A3920</t>
+          <t>A8046</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732133</t>
+          <t>00019200000012732125</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -11140,12 +11160,12 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>A7425</t>
+          <t>A3920</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732141</t>
+          <t>00019200000012732133</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -11172,12 +11192,12 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>A3679</t>
+          <t>A7425</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732150</t>
+          <t>00019200000012732141</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -11204,12 +11224,12 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>A7985</t>
+          <t>A3679</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732168</t>
+          <t>00019200000012732150</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
@@ -11236,12 +11256,12 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>A6562</t>
+          <t>A7985</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732176</t>
+          <t>00019200000012732168</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
@@ -11268,12 +11288,12 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>A4360</t>
+          <t>A6562</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732184</t>
+          <t>00019200000012732176</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -11300,12 +11320,12 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>A9173</t>
+          <t>A4360</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732192</t>
+          <t>00019200000012732184</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
@@ -11332,12 +11352,12 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>A2809</t>
+          <t>A9173</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732206</t>
+          <t>00019200000012732192</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
@@ -11364,12 +11384,12 @@
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>TA0960</t>
+          <t>A2809</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732214</t>
+          <t>00019200000012732206</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
@@ -11396,12 +11416,12 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>TA0960</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732222</t>
+          <t>00019200000012732214</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -11428,12 +11448,12 @@
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>A9307</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732230</t>
+          <t>00019200000012732222</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
@@ -11460,12 +11480,12 @@
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>A7068</t>
+          <t>A9307</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732249</t>
+          <t>00019200000012732230</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
@@ -11492,12 +11512,12 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>A3376</t>
+          <t>A7068</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732257</t>
+          <t>00019200000012732249</t>
         </is>
       </c>
       <c r="E347" s="2" t="inlineStr">
@@ -11524,12 +11544,12 @@
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>A3287</t>
+          <t>A3376</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732265</t>
+          <t>00019200000012732257</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -11556,12 +11576,12 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>A9200</t>
+          <t>A3287</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732273</t>
+          <t>00019200000012732265</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
@@ -11588,12 +11608,12 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>A5037</t>
+          <t>A9200</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732281</t>
+          <t>00019200000012732273</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
@@ -11620,12 +11640,12 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>A9610</t>
+          <t>A5037</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732290</t>
+          <t>00019200000012732281</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
@@ -11652,12 +11672,12 @@
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>A1420</t>
+          <t>A9610</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>00019200000012857750</t>
+          <t>00019200000012732290</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -11674,32 +11694,32 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>555932</t>
+          <t>556160</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>A4257</t>
+          <t>A1420</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721840</t>
+          <t>00019200000012857750</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:18</t>
+          <t>06/06/2026 11:33</t>
         </is>
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:33</t>
+          <t>08/06/2026 11:46</t>
         </is>
       </c>
     </row>
@@ -11716,12 +11736,12 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>A9287</t>
+          <t>A4257</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723061</t>
+          <t>00019200000012721840</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
@@ -11738,7 +11758,7 @@
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>556161</t>
+          <t>555932</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
@@ -11748,22 +11768,22 @@
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>A7008</t>
+          <t>A9287</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730491</t>
+          <t>00019200000012723061</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:18</t>
         </is>
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:51</t>
+          <t>03/06/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -11780,12 +11800,12 @@
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>A7785</t>
+          <t>A7008</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730670</t>
+          <t>00019200000012730491</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
@@ -11812,12 +11832,12 @@
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>A6386</t>
+          <t>A7785</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730688</t>
+          <t>00019200000012730670</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
@@ -11844,12 +11864,12 @@
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>A8302</t>
+          <t>A6386</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730696</t>
+          <t>00019200000012730688</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -11876,12 +11896,12 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>A6870</t>
+          <t>A8302</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730700</t>
+          <t>00019200000012730696</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
@@ -11908,12 +11928,12 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>A8192</t>
+          <t>A6870</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731331</t>
+          <t>00019200000012730700</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
@@ -11940,12 +11960,12 @@
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>A1045</t>
+          <t>A8192</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731340</t>
+          <t>00019200000012731331</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
@@ -11972,12 +11992,12 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>A3603</t>
+          <t>A1045</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731358</t>
+          <t>00019200000012731340</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
@@ -12004,12 +12024,12 @@
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>A9427</t>
+          <t>A3603</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731366</t>
+          <t>00019200000012731358</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
@@ -12036,12 +12056,12 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>A4068</t>
+          <t>A9427</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731374</t>
+          <t>00019200000012731366</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -12068,12 +12088,12 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>A2753</t>
+          <t>A4068</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731382</t>
+          <t>00019200000012731374</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
@@ -12100,12 +12120,12 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>TA0353</t>
+          <t>A2753</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731390</t>
+          <t>00019200000012731382</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
@@ -12132,12 +12152,12 @@
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>A7155</t>
+          <t>TA0353</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731404</t>
+          <t>00019200000012731390</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
@@ -12164,12 +12184,12 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>A6665</t>
+          <t>A7155</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731412</t>
+          <t>00019200000012731404</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
@@ -12196,12 +12216,12 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>TA0675</t>
+          <t>A6665</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731420</t>
+          <t>00019200000012731412</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
@@ -12228,12 +12248,12 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>A7142</t>
+          <t>TA0675</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731439</t>
+          <t>00019200000012731420</t>
         </is>
       </c>
       <c r="E370" s="2" t="inlineStr">
@@ -12260,12 +12280,12 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>TA0136</t>
+          <t>A7142</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731447</t>
+          <t>00019200000012731439</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
@@ -12292,12 +12312,12 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>TA0818</t>
+          <t>TA0136</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731455</t>
+          <t>00019200000012731447</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
@@ -12324,12 +12344,12 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>A6147</t>
+          <t>TA0818</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731463</t>
+          <t>00019200000012731455</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
@@ -12356,12 +12376,12 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>A4999</t>
+          <t>A6147</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731471</t>
+          <t>00019200000012731463</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr">
@@ -12388,12 +12408,12 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>A5847</t>
+          <t>A4999</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731498</t>
+          <t>00019200000012731471</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
@@ -12420,12 +12440,12 @@
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>A2981</t>
+          <t>A5847</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731501</t>
+          <t>00019200000012731498</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
@@ -12452,12 +12472,12 @@
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>A7462</t>
+          <t>A2981</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731510</t>
+          <t>00019200000012731501</t>
         </is>
       </c>
       <c r="E377" s="2" t="inlineStr">
@@ -12484,12 +12504,12 @@
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>A4340</t>
+          <t>A7462</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731528</t>
+          <t>00019200000012731510</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
@@ -12516,12 +12536,12 @@
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>A8938</t>
+          <t>A4340</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731536</t>
+          <t>00019200000012731528</t>
         </is>
       </c>
       <c r="E379" s="2" t="inlineStr">
@@ -12538,7 +12558,7 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>556300</t>
+          <t>556161</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
@@ -12548,54 +12568,54 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>TA0506</t>
+          <t>A8938</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728918</t>
+          <t>00019200000012731536</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 10:36</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F380" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:54</t>
+          <t>08/06/2026 14:51</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>556300</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>TA0506</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000012728918</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>06/06/2026 10:36</t>
         </is>
       </c>
       <c r="F381" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>08/06/2026 10:54</t>
         </is>
       </c>
     </row>
@@ -12612,12 +12632,12 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
@@ -12644,12 +12664,12 @@
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E383" s="2" t="inlineStr">
@@ -12666,39 +12686,39 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B385" s="2" t="inlineStr">
@@ -12708,22 +12728,22 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E385" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F385" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -12740,12 +12760,12 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
@@ -12772,12 +12792,12 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E387" s="2" t="inlineStr">
@@ -12804,12 +12824,12 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
@@ -12836,12 +12856,12 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr">
@@ -12868,12 +12888,12 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
@@ -12900,12 +12920,12 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
@@ -12932,12 +12952,12 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
@@ -12964,12 +12984,12 @@
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
@@ -12996,12 +13016,12 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
@@ -13028,12 +13048,12 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
@@ -13060,12 +13080,12 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
@@ -13092,12 +13112,12 @@
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E397" s="2" t="inlineStr">
@@ -13124,12 +13144,12 @@
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E398" s="2" t="inlineStr">
@@ -13156,12 +13176,12 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E399" s="2" t="inlineStr">
@@ -13178,7 +13198,7 @@
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B400" s="2" t="inlineStr">
@@ -13188,17 +13208,17 @@
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E400" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F400" s="2" t="inlineStr">
@@ -13220,12 +13240,12 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E401" s="2" t="inlineStr">
@@ -13252,12 +13272,12 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E402" s="2" t="inlineStr">
@@ -13284,12 +13304,12 @@
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E403" s="2" t="inlineStr">
@@ -13316,27 +13336,59 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B405" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
           <t>A8196</t>
         </is>
       </c>
-      <c r="D404" s="2" t="inlineStr">
+      <c r="D405" s="2" t="inlineStr">
         <is>
           <t>00019200000012728802</t>
         </is>
       </c>
-      <c r="E404" s="2" t="inlineStr">
+      <c r="E405" s="2" t="inlineStr">
         <is>
           <t>09/06/2026 02:06</t>
         </is>
       </c>
-      <c r="F404" s="2" t="inlineStr">
+      <c r="F405" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F404"/>
+  <autoFilter ref="A1:F405"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-09 17:34:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5003,7 +5003,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 09:30</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 09:53</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 17:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-10 10:56:54
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -2187,7 +2187,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-10 16:51:04
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -14851,7 +14851,7 @@
       </c>
       <c r="F451" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -14883,7 +14883,7 @@
       </c>
       <c r="F452" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="F453" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -14947,7 +14947,7 @@
       </c>
       <c r="F454" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -14979,7 +14979,7 @@
       </c>
       <c r="F455" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-10 18:32:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -14371,7 +14371,7 @@
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14403,7 +14403,7 @@
       </c>
       <c r="F437" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="F438" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14467,7 +14467,7 @@
       </c>
       <c r="F439" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14499,7 +14499,7 @@
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14531,7 +14531,7 @@
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14563,7 +14563,7 @@
       </c>
       <c r="F442" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14595,7 +14595,7 @@
       </c>
       <c r="F443" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14627,7 +14627,7 @@
       </c>
       <c r="F444" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14659,7 +14659,7 @@
       </c>
       <c r="F445" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14691,7 @@
       </c>
       <c r="F446" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14723,7 +14723,7 @@
       </c>
       <c r="F447" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14755,7 +14755,7 @@
       </c>
       <c r="F448" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14787,7 +14787,7 @@
       </c>
       <c r="F449" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -14819,7 +14819,7 @@
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-10 19:15:46
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -4299,7 +4299,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4395,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4747,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4939,7 +4939,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5163,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5543,7 +5543,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5575,7 +5575,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5895,7 +5895,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6023,7 +6023,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6247,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6311,7 +6311,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6407,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 11:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-11 12:24:19
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 12:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-11 13:07:40
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -4847,7 +4847,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5167,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5359,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 12:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-11 17:38:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -15207,7 +15207,7 @@
       </c>
       <c r="F462" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -15239,7 +15239,7 @@
       </c>
       <c r="F463" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="F464" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-11 19:35:42
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10443,7 +10443,7 @@
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10475,7 +10475,7 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10507,7 +10507,7 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10571,7 +10571,7 @@
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10635,7 +10635,7 @@
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10667,7 +10667,7 @@
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10731,7 +10731,7 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10763,7 +10763,7 @@
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10795,7 +10795,7 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10827,7 +10827,7 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -10987,7 +10987,7 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11051,7 +11051,7 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11083,7 +11083,7 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11115,7 +11115,7 @@
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11243,7 +11243,7 @@
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11275,7 +11275,7 @@
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11339,7 +11339,7 @@
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11371,7 +11371,7 @@
       </c>
       <c r="F342" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11435,7 +11435,7 @@
       </c>
       <c r="F344" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11467,7 +11467,7 @@
       </c>
       <c r="F345" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11499,7 +11499,7 @@
       </c>
       <c r="F346" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11531,7 +11531,7 @@
       </c>
       <c r="F347" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F348" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11595,7 +11595,7 @@
       </c>
       <c r="F349" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11627,7 +11627,7 @@
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="F351" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11691,7 +11691,7 @@
       </c>
       <c r="F352" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11755,7 +11755,7 @@
       </c>
       <c r="F354" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11787,7 +11787,7 @@
       </c>
       <c r="F355" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11819,7 +11819,7 @@
       </c>
       <c r="F356" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11851,7 +11851,7 @@
       </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="F358" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11915,7 +11915,7 @@
       </c>
       <c r="F359" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11947,7 +11947,7 @@
       </c>
       <c r="F360" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11979,7 @@
       </c>
       <c r="F361" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12011,7 +12011,7 @@
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12075,7 +12075,7 @@
       </c>
       <c r="F364" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12107,7 @@
       </c>
       <c r="F365" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12139,7 +12139,7 @@
       </c>
       <c r="F366" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12171,7 +12171,7 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12203,7 +12203,7 @@
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12235,7 +12235,7 @@
       </c>
       <c r="F369" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12267,7 +12267,7 @@
       </c>
       <c r="F370" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12299,7 +12299,7 @@
       </c>
       <c r="F371" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="F372" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12363,7 +12363,7 @@
       </c>
       <c r="F373" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12395,7 +12395,7 @@
       </c>
       <c r="F374" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12427,7 +12427,7 @@
       </c>
       <c r="F375" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="F376" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12491,7 +12491,7 @@
       </c>
       <c r="F377" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12523,7 +12523,7 @@
       </c>
       <c r="F378" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12555,7 +12555,7 @@
       </c>
       <c r="F379" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12587,7 +12587,7 @@
       </c>
       <c r="F380" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12619,7 +12619,7 @@
       </c>
       <c r="F381" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12651,7 +12651,7 @@
       </c>
       <c r="F382" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12683,7 +12683,7 @@
       </c>
       <c r="F383" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12715,7 +12715,7 @@
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12747,7 +12747,7 @@
       </c>
       <c r="F385" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="F386" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12811,7 +12811,7 @@
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12843,7 +12843,7 @@
       </c>
       <c r="F388" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12875,7 +12875,7 @@
       </c>
       <c r="F389" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12907,7 +12907,7 @@
       </c>
       <c r="F390" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12939,7 @@
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -12971,7 +12971,7 @@
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -13003,7 +13003,7 @@
       </c>
       <c r="F393" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="F394" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -13067,7 +13067,7 @@
       </c>
       <c r="F395" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 08:56:32
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -2767,7 +2767,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 16:55</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 16:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 10:25:41
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9611,7 +9611,7 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9643,7 +9643,7 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9675,7 +9675,7 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9707,7 +9707,7 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9739,7 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9771,7 +9771,7 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9899,7 +9899,7 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9931,7 +9931,7 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9963,7 +9963,7 @@
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10027,7 +10027,7 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10059,7 +10059,7 @@
       </c>
       <c r="F301" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10091,7 +10091,7 @@
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10123,7 +10123,7 @@
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10155,7 @@
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10187,7 +10187,7 @@
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 10:56:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -1743,7 +1743,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 11:11:48
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -815,7 +815,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 12:26:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 12:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 15:39:16
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:25</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 15:54:15
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5455,7 +5455,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:31</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:31</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 17:22:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -7787,7 +7787,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7947,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8011,7 +8011,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8043,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8075,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8139,7 +8139,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8171,7 +8171,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8203,7 +8203,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8267,7 +8267,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8299,7 +8299,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>
@@ -8331,7 +8331,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 17:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 20:04:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -1871,7 +1871,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12/06/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-12 21:45:02
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -8843,7 +8843,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
@@ -8939,7 +8939,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
@@ -8971,7 +8971,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-13 13:08:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$516</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$517</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F516"/>
+  <dimension ref="A1:F517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8402,39 +8402,39 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>555905</t>
+          <t>556651</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>TA1127</t>
+          <t>TA0400</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>00019200000012720607</t>
+          <t>00019200000013212958</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:04</t>
+          <t>13/06/2026 12:56</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:30</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>556204</t>
+          <t>555905</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -8444,61 +8444,61 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>A9236</t>
+          <t>TA1127</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715247</t>
+          <t>00019200000012720607</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 00:11</t>
+          <t>06/06/2026 05:04</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:53</t>
+          <t>09/06/2026 09:30</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>555984</t>
+          <t>556204</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>A2586</t>
+          <t>A9236</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718378</t>
+          <t>00019200000012715247</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:09</t>
+          <t>08/06/2026 00:11</t>
         </is>
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 15:14</t>
+          <t>09/06/2026 09:53</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>556084</t>
+          <t>555984</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
@@ -8508,29 +8508,29 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>A7594</t>
+          <t>A2586</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721921</t>
+          <t>00019200000012718378</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:17</t>
+          <t>06/06/2026 05:09</t>
         </is>
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 16:30</t>
+          <t>09/06/2026 15:14</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>556170</t>
+          <t>556084</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -8540,12 +8540,12 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>A6367</t>
+          <t>A7594</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718521</t>
+          <t>00019200000012721921</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr">
@@ -8555,7 +8555,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 17:00</t>
+          <t>03/06/2026 16:30</t>
         </is>
       </c>
     </row>
@@ -8572,12 +8572,12 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>TA0161</t>
+          <t>A6367</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718530</t>
+          <t>00019200000012718521</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
@@ -8604,12 +8604,12 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>TA0713</t>
+          <t>TA0161</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718548</t>
+          <t>00019200000012718530</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr">
@@ -8626,7 +8626,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>556330</t>
+          <t>556170</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -8636,54 +8636,54 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>A8235</t>
+          <t>TA0713</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728926</t>
+          <t>00019200000012718548</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 22:37</t>
+          <t>01/06/2026 22:17</t>
         </is>
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 16:07</t>
+          <t>08/06/2026 17:00</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>556173</t>
+          <t>556330</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>A5580</t>
+          <t>A8235</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714577</t>
+          <t>00019200000012728926</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 09:17</t>
+          <t>08/06/2026 22:37</t>
         </is>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:00</t>
+          <t>10/06/2026 16:07</t>
         </is>
       </c>
     </row>
@@ -8700,12 +8700,12 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>A4423</t>
+          <t>A5580</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714585</t>
+          <t>00019200000012714577</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
@@ -8722,39 +8722,39 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>555906</t>
+          <t>556173</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>TA1064</t>
+          <t>A4423</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718556</t>
+          <t>00019200000012714585</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:51</t>
+          <t>06/06/2026 09:17</t>
         </is>
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 17:20</t>
+          <t>08/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>556105</t>
+          <t>555906</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
@@ -8764,29 +8764,29 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>A0431</t>
+          <t>TA1064</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>00019200000012717614</t>
+          <t>00019200000012718556</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 22:37</t>
+          <t>07/06/2026 22:51</t>
         </is>
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30</t>
+          <t>09/06/2026 17:20</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>556187</t>
+          <t>556105</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -8796,54 +8796,54 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>A8822</t>
+          <t>A0431</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864242</t>
+          <t>00019200000012717614</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 21:57</t>
+          <t>08/06/2026 22:37</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 13:07</t>
+          <t>10/06/2026 10:30</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>556113</t>
+          <t>556187</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>A9365</t>
+          <t>A8822</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714593</t>
+          <t>00019200000012864242</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:53</t>
+          <t>02/06/2026 21:57</t>
         </is>
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 19:47</t>
+          <t>04/06/2026 13:07</t>
         </is>
       </c>
     </row>
@@ -8860,12 +8860,12 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>A7132</t>
+          <t>A9365</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714607</t>
+          <t>00019200000012714593</t>
         </is>
       </c>
       <c r="E264" s="2" t="inlineStr">
@@ -8892,12 +8892,12 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>A6834</t>
+          <t>A7132</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714615</t>
+          <t>00019200000012714607</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
@@ -8924,12 +8924,12 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>A8249</t>
+          <t>A6834</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714623</t>
+          <t>00019200000012714615</t>
         </is>
       </c>
       <c r="E266" s="2" t="inlineStr">
@@ -8956,12 +8956,12 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>A8816</t>
+          <t>A8249</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714640</t>
+          <t>00019200000012714623</t>
         </is>
       </c>
       <c r="E267" s="2" t="inlineStr">
@@ -8978,7 +8978,7 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>556339</t>
+          <t>556113</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
@@ -8988,29 +8988,29 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>A7748</t>
+          <t>A8816</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729124</t>
+          <t>00019200000012714640</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 03:51</t>
+          <t>08/06/2026 10:53</t>
         </is>
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 17:19</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>556549</t>
+          <t>556339</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
@@ -9020,61 +9020,61 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>A7654</t>
+          <t>A7748</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730505</t>
+          <t>00019200000012729124</t>
         </is>
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:31</t>
+          <t>09/06/2026 03:51</t>
         </is>
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 17:00</t>
+          <t>10/06/2026 17:19</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>20260717</t>
+          <t>556549</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>A5970</t>
+          <t>A7654</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721034</t>
+          <t>00019200000012730505</t>
         </is>
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:14</t>
+          <t>08/06/2026 05:31</t>
         </is>
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 13:12</t>
+          <t>09/06/2026 17:00</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>556743</t>
+          <t>20260717</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
@@ -9084,54 +9084,54 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>A7321</t>
+          <t>A5970</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723487</t>
+          <t>00019200000012721034</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:50</t>
+          <t>02/06/2026 01:14</t>
         </is>
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:50</t>
+          <t>03/06/2026 13:12</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>556083</t>
+          <t>556743</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>A5844</t>
+          <t>A7321</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721867</t>
+          <t>00019200000012723487</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:05</t>
+          <t>07/06/2026 22:50</t>
         </is>
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 17:29</t>
+          <t>09/06/2026 10:50</t>
         </is>
       </c>
     </row>
@@ -9148,12 +9148,12 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>A4723</t>
+          <t>A5844</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721891</t>
+          <t>00019200000012721867</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr">
@@ -9170,7 +9170,7 @@
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>556294</t>
+          <t>556083</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
@@ -9180,22 +9180,22 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>A3519</t>
+          <t>A4723</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714704</t>
+          <t>00019200000012721891</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 13:37</t>
+          <t>01/06/2026 22:05</t>
         </is>
       </c>
       <c r="F274" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 16:38</t>
+          <t>03/06/2026 17:29</t>
         </is>
       </c>
     </row>
@@ -9212,12 +9212,12 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>A9135</t>
+          <t>A3519</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714712</t>
+          <t>00019200000012714704</t>
         </is>
       </c>
       <c r="E275" s="2" t="inlineStr">
@@ -9244,12 +9244,12 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>TA0487</t>
+          <t>A9135</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714720</t>
+          <t>00019200000012714712</t>
         </is>
       </c>
       <c r="E276" s="2" t="inlineStr">
@@ -9276,12 +9276,12 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>TA1114</t>
+          <t>TA0487</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714739</t>
+          <t>00019200000012714720</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
@@ -9308,12 +9308,12 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>A8445</t>
+          <t>TA1114</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714747</t>
+          <t>00019200000012714739</t>
         </is>
       </c>
       <c r="E278" s="2" t="inlineStr">
@@ -9340,12 +9340,12 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>A6194</t>
+          <t>A8445</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714763</t>
+          <t>00019200000012714747</t>
         </is>
       </c>
       <c r="E279" s="2" t="inlineStr">
@@ -9372,12 +9372,12 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>A9186</t>
+          <t>A6194</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714771</t>
+          <t>00019200000012714763</t>
         </is>
       </c>
       <c r="E280" s="2" t="inlineStr">
@@ -9404,12 +9404,12 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>A8034</t>
+          <t>A9186</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714780</t>
+          <t>00019200000012714771</t>
         </is>
       </c>
       <c r="E281" s="2" t="inlineStr">
@@ -9436,12 +9436,12 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>A0774</t>
+          <t>A8034</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714798</t>
+          <t>00019200000012714780</t>
         </is>
       </c>
       <c r="E282" s="2" t="inlineStr">
@@ -9468,12 +9468,12 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>A8373</t>
+          <t>A0774</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714801</t>
+          <t>00019200000012714798</t>
         </is>
       </c>
       <c r="E283" s="2" t="inlineStr">
@@ -9500,12 +9500,12 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>A8792</t>
+          <t>A8373</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714810</t>
+          <t>00019200000012714801</t>
         </is>
       </c>
       <c r="E284" s="2" t="inlineStr">
@@ -9532,12 +9532,12 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>A0162</t>
+          <t>A8792</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714828</t>
+          <t>00019200000012714810</t>
         </is>
       </c>
       <c r="E285" s="2" t="inlineStr">
@@ -9554,39 +9554,39 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>555911</t>
+          <t>556294</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>A4881</t>
+          <t>A0162</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715298</t>
+          <t>00019200000012714828</t>
         </is>
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:02</t>
+          <t>02/06/2026 13:37</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>03/06/2026 16:38</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>556157</t>
+          <t>555911</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
@@ -9596,12 +9596,12 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>TA0188</t>
+          <t>A4881</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730203</t>
+          <t>00019200000012715298</t>
         </is>
       </c>
       <c r="E287" s="2" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:00</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -9628,12 +9628,12 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>TA0670</t>
+          <t>TA0188</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730211</t>
+          <t>00019200000012730203</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
@@ -9660,12 +9660,12 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>A3810</t>
+          <t>TA0670</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730220</t>
+          <t>00019200000012730211</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr">
@@ -9692,12 +9692,12 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>A0800</t>
+          <t>A3810</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730238</t>
+          <t>00019200000012730220</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
@@ -9724,12 +9724,12 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>A5751</t>
+          <t>A0800</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730246</t>
+          <t>00019200000012730238</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
@@ -9756,12 +9756,12 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>A3830</t>
+          <t>A5751</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730254</t>
+          <t>00019200000012730246</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
@@ -9788,12 +9788,12 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>A2419</t>
+          <t>A3830</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730262</t>
+          <t>00019200000012730254</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
@@ -9820,12 +9820,12 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>A7535</t>
+          <t>A2419</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730270</t>
+          <t>00019200000012730262</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
@@ -9852,12 +9852,12 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>A5563</t>
+          <t>A7535</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730289</t>
+          <t>00019200000012730270</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
@@ -9884,12 +9884,12 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>A9066</t>
+          <t>A5563</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730297</t>
+          <t>00019200000012730289</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
@@ -9916,12 +9916,12 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>A5828</t>
+          <t>A9066</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730300</t>
+          <t>00019200000012730297</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
@@ -9948,12 +9948,12 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>A4055</t>
+          <t>A5828</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730319</t>
+          <t>00019200000012730300</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
@@ -9980,12 +9980,12 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>A0130</t>
+          <t>A4055</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730327</t>
+          <t>00019200000012730319</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
@@ -10012,12 +10012,12 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>A7797</t>
+          <t>A0130</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730335</t>
+          <t>00019200000012730327</t>
         </is>
       </c>
       <c r="E300" s="2" t="inlineStr">
@@ -10044,12 +10044,12 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>A9654</t>
+          <t>A7797</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730343</t>
+          <t>00019200000012730335</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
@@ -10076,12 +10076,12 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>A7482</t>
+          <t>A9654</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730351</t>
+          <t>00019200000012730343</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
@@ -10108,12 +10108,12 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>A7723</t>
+          <t>A7482</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730360</t>
+          <t>00019200000012730351</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
@@ -10140,12 +10140,12 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>A7997</t>
+          <t>A7723</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730378</t>
+          <t>00019200000012730360</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
@@ -10162,7 +10162,7 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>556258</t>
+          <t>556157</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
@@ -10172,17 +10172,17 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>A6961</t>
+          <t>A7997</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729159</t>
+          <t>00019200000012730378</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>06/06/2026 05:02</t>
         </is>
       </c>
       <c r="F305" s="2" t="inlineStr">
@@ -10194,22 +10194,22 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>556158</t>
+          <t>556258</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>A8351</t>
+          <t>A6961</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715344</t>
+          <t>00019200000012729159</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
@@ -10219,7 +10219,7 @@
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:00</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -10236,12 +10236,12 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>A6522</t>
+          <t>A8351</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715352</t>
+          <t>00019200000012715344</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
@@ -10268,12 +10268,12 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>A7263</t>
+          <t>A6522</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715360</t>
+          <t>00019200000012715352</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
@@ -10300,12 +10300,12 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>A9019</t>
+          <t>A7263</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715379</t>
+          <t>00019200000012715360</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
@@ -10332,12 +10332,12 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>A4823</t>
+          <t>A9019</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715387</t>
+          <t>00019200000012715379</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
@@ -10364,12 +10364,12 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>A5775</t>
+          <t>A4823</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715395</t>
+          <t>00019200000012715387</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
@@ -10396,12 +10396,12 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>A6931</t>
+          <t>A5775</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715409</t>
+          <t>00019200000012715395</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
@@ -10418,32 +10418,32 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>556159</t>
+          <t>556158</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>TA1119</t>
+          <t>A6931</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753440</t>
+          <t>00019200000012715409</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:08</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 13:30</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -10460,12 +10460,12 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>A6893</t>
+          <t>TA1119</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753459</t>
+          <t>00019200000012753440</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
@@ -10492,12 +10492,12 @@
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>A8127</t>
+          <t>A6893</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753467</t>
+          <t>00019200000012753459</t>
         </is>
       </c>
       <c r="E315" s="2" t="inlineStr">
@@ -10524,12 +10524,12 @@
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>A6189</t>
+          <t>A8127</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753475</t>
+          <t>00019200000012753467</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
@@ -10556,12 +10556,12 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>TA0776</t>
+          <t>A6189</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753483</t>
+          <t>00019200000012753475</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
@@ -10588,12 +10588,12 @@
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>A8534</t>
+          <t>TA0776</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753491</t>
+          <t>00019200000012753483</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
@@ -10620,12 +10620,12 @@
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>A7575</t>
+          <t>A8534</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753505</t>
+          <t>00019200000012753491</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
@@ -10652,12 +10652,12 @@
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>A0609</t>
+          <t>A7575</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753513</t>
+          <t>00019200000012753505</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
@@ -10684,12 +10684,12 @@
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>A9499</t>
+          <t>A0609</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753521</t>
+          <t>00019200000012753513</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
@@ -10716,12 +10716,12 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>A6581</t>
+          <t>A9499</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753530</t>
+          <t>00019200000012753521</t>
         </is>
       </c>
       <c r="E322" s="2" t="inlineStr">
@@ -10748,12 +10748,12 @@
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>A8536</t>
+          <t>A6581</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753548</t>
+          <t>00019200000012753530</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
@@ -10780,12 +10780,12 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>A9316</t>
+          <t>A8536</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753556</t>
+          <t>00019200000012753548</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
@@ -10812,12 +10812,12 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>TA0880</t>
+          <t>A9316</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753564</t>
+          <t>00019200000012753556</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
@@ -10844,12 +10844,12 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>A1933</t>
+          <t>TA0880</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753572</t>
+          <t>00019200000012753564</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -10876,12 +10876,12 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>A0504</t>
+          <t>A1933</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753882</t>
+          <t>00019200000012753572</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
@@ -10908,12 +10908,12 @@
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>TA0704</t>
+          <t>A0504</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753890</t>
+          <t>00019200000012753882</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -10940,12 +10940,12 @@
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>A8967</t>
+          <t>TA0704</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753904</t>
+          <t>00019200000012753890</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
@@ -10972,12 +10972,12 @@
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>A4337</t>
+          <t>A8967</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753912</t>
+          <t>00019200000012753904</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
@@ -11004,12 +11004,12 @@
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>A5175</t>
+          <t>A4337</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753920</t>
+          <t>00019200000012753912</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
@@ -11036,12 +11036,12 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>TA0974</t>
+          <t>A5175</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753939</t>
+          <t>00019200000012753920</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
@@ -11068,12 +11068,12 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>A6700</t>
+          <t>TA0974</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753947</t>
+          <t>00019200000012753939</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -11100,12 +11100,12 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>A8361</t>
+          <t>A6700</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753955</t>
+          <t>00019200000012753947</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -11132,12 +11132,12 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>A3121</t>
+          <t>A8361</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753963</t>
+          <t>00019200000012753955</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -11164,12 +11164,12 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>A8154</t>
+          <t>A3121</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753971</t>
+          <t>00019200000012753963</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -11196,12 +11196,12 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>TA0597</t>
+          <t>A8154</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753980</t>
+          <t>00019200000012753971</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -11228,12 +11228,12 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>A6883</t>
+          <t>TA0597</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753998</t>
+          <t>00019200000012753980</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
@@ -11260,12 +11260,12 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>A9704</t>
+          <t>A6883</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754005</t>
+          <t>00019200000012753998</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
@@ -11292,12 +11292,12 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>A9302</t>
+          <t>A9704</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754013</t>
+          <t>00019200000012754005</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -11324,12 +11324,12 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>A0119</t>
+          <t>A9302</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754021</t>
+          <t>00019200000012754013</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
@@ -11356,12 +11356,12 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>A9040</t>
+          <t>A0119</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754048</t>
+          <t>00019200000012754021</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
@@ -11388,12 +11388,12 @@
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>A7876</t>
+          <t>A9040</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754056</t>
+          <t>00019200000012754048</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
@@ -11420,12 +11420,12 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>A8919</t>
+          <t>A7876</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754064</t>
+          <t>00019200000012754056</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -11452,12 +11452,12 @@
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>A6393</t>
+          <t>A8919</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754072</t>
+          <t>00019200000012754064</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
@@ -11484,12 +11484,12 @@
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>A4317</t>
+          <t>A6393</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754080</t>
+          <t>00019200000012754072</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
@@ -11516,12 +11516,12 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>A8657</t>
+          <t>A4317</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754099</t>
+          <t>00019200000012754080</t>
         </is>
       </c>
       <c r="E347" s="2" t="inlineStr">
@@ -11548,12 +11548,12 @@
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>A8940</t>
+          <t>A8657</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754102</t>
+          <t>00019200000012754099</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -11580,12 +11580,12 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>A6261</t>
+          <t>A8940</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754110</t>
+          <t>00019200000012754102</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
@@ -11612,12 +11612,12 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>A5569</t>
+          <t>A6261</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754129</t>
+          <t>00019200000012754110</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
@@ -11644,12 +11644,12 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>A8748</t>
+          <t>A5569</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754137</t>
+          <t>00019200000012754129</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
@@ -11676,12 +11676,12 @@
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>A9213</t>
+          <t>A8748</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754145</t>
+          <t>00019200000012754137</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -11708,12 +11708,12 @@
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>TA0226</t>
+          <t>A9213</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754153</t>
+          <t>00019200000012754145</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
@@ -11740,12 +11740,12 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>A8485</t>
+          <t>TA0226</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754161</t>
+          <t>00019200000012754153</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
@@ -11772,12 +11772,12 @@
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>A8095</t>
+          <t>A8485</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754170</t>
+          <t>00019200000012754161</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
@@ -11804,12 +11804,12 @@
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>A9152</t>
+          <t>A8095</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754188</t>
+          <t>00019200000012754170</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
@@ -11836,12 +11836,12 @@
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>A7849</t>
+          <t>A9152</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754196</t>
+          <t>00019200000012754188</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
@@ -11868,12 +11868,12 @@
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>A6854</t>
+          <t>A7849</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754200</t>
+          <t>00019200000012754196</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -11900,12 +11900,12 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>A8670</t>
+          <t>A6854</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754218</t>
+          <t>00019200000012754200</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
@@ -11932,12 +11932,12 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>A8352</t>
+          <t>A8670</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754226</t>
+          <t>00019200000012754218</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
@@ -11964,12 +11964,12 @@
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>A6584</t>
+          <t>A8352</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754234</t>
+          <t>00019200000012754226</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
@@ -11996,12 +11996,12 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>A5394</t>
+          <t>A6584</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754242</t>
+          <t>00019200000012754234</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
@@ -12028,12 +12028,12 @@
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>A9258</t>
+          <t>A5394</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754250</t>
+          <t>00019200000012754242</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
@@ -12060,12 +12060,12 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>A2475</t>
+          <t>A9258</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754269</t>
+          <t>00019200000012754250</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -12092,12 +12092,12 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>A8952</t>
+          <t>A2475</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754277</t>
+          <t>00019200000012754269</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
@@ -12124,12 +12124,12 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>A6781</t>
+          <t>A8952</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754285</t>
+          <t>00019200000012754277</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
@@ -12156,12 +12156,12 @@
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>A8379</t>
+          <t>A6781</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754293</t>
+          <t>00019200000012754285</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
@@ -12188,12 +12188,12 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>A8243</t>
+          <t>A8379</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754307</t>
+          <t>00019200000012754293</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
@@ -12220,12 +12220,12 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>A7097</t>
+          <t>A8243</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754315</t>
+          <t>00019200000012754307</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
@@ -12252,12 +12252,12 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>TA0235</t>
+          <t>A7097</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754323</t>
+          <t>00019200000012754315</t>
         </is>
       </c>
       <c r="E370" s="2" t="inlineStr">
@@ -12284,12 +12284,12 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>A8222</t>
+          <t>TA0235</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754331</t>
+          <t>00019200000012754323</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
@@ -12316,12 +12316,12 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>A1510</t>
+          <t>A8222</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754340</t>
+          <t>00019200000012754331</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
@@ -12348,12 +12348,12 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>A0773</t>
+          <t>A1510</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754358</t>
+          <t>00019200000012754340</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
@@ -12380,12 +12380,12 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>A8448</t>
+          <t>A0773</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754366</t>
+          <t>00019200000012754358</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr">
@@ -12412,12 +12412,12 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>A7767</t>
+          <t>A8448</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754374</t>
+          <t>00019200000012754366</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
@@ -12444,12 +12444,12 @@
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>A8254</t>
+          <t>A7767</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754382</t>
+          <t>00019200000012754374</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
@@ -12476,12 +12476,12 @@
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>A9361</t>
+          <t>A8254</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754390</t>
+          <t>00019200000012754382</t>
         </is>
       </c>
       <c r="E377" s="2" t="inlineStr">
@@ -12508,12 +12508,12 @@
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>A5087</t>
+          <t>A9361</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754404</t>
+          <t>00019200000012754390</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
@@ -12540,12 +12540,12 @@
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>A0387</t>
+          <t>A5087</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754412</t>
+          <t>00019200000012754404</t>
         </is>
       </c>
       <c r="E379" s="2" t="inlineStr">
@@ -12572,12 +12572,12 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>A6996</t>
+          <t>A0387</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754420</t>
+          <t>00019200000012754412</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
@@ -12604,12 +12604,12 @@
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>A7094</t>
+          <t>A6996</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754439</t>
+          <t>00019200000012754420</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
@@ -12636,12 +12636,12 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>A7194</t>
+          <t>A7094</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754447</t>
+          <t>00019200000012754439</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
@@ -12668,12 +12668,12 @@
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>A6941</t>
+          <t>A7194</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754455</t>
+          <t>00019200000012754447</t>
         </is>
       </c>
       <c r="E383" s="2" t="inlineStr">
@@ -12700,12 +12700,12 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>A6571</t>
+          <t>A6941</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754463</t>
+          <t>00019200000012754455</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
@@ -12732,12 +12732,12 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>A5633</t>
+          <t>A6571</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754471</t>
+          <t>00019200000012754463</t>
         </is>
       </c>
       <c r="E385" s="2" t="inlineStr">
@@ -12764,12 +12764,12 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>A9483</t>
+          <t>A5633</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754480</t>
+          <t>00019200000012754471</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
@@ -12796,12 +12796,12 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>A9277</t>
+          <t>A9483</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754498</t>
+          <t>00019200000012754480</t>
         </is>
       </c>
       <c r="E387" s="2" t="inlineStr">
@@ -12828,12 +12828,12 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>A6305</t>
+          <t>A9277</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754501</t>
+          <t>00019200000012754498</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
@@ -12860,12 +12860,12 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>A0745</t>
+          <t>A6305</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754510</t>
+          <t>00019200000012754501</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr">
@@ -12892,12 +12892,12 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>A7451</t>
+          <t>A0745</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755958</t>
+          <t>00019200000012754510</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
@@ -12924,12 +12924,12 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>A9324</t>
+          <t>A7451</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755966</t>
+          <t>00019200000012755958</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
@@ -12956,12 +12956,12 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>A8491</t>
+          <t>A9324</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755974</t>
+          <t>00019200000012755966</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
@@ -12988,12 +12988,12 @@
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>A9490</t>
+          <t>A8491</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755982</t>
+          <t>00019200000012755974</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
@@ -13020,12 +13020,12 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>A9202</t>
+          <t>A9490</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755990</t>
+          <t>00019200000012755982</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
@@ -13052,12 +13052,12 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>A5679</t>
+          <t>A9202</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>00019200000012756008</t>
+          <t>00019200000012755990</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
@@ -13074,7 +13074,7 @@
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>556744</t>
+          <t>556159</t>
         </is>
       </c>
       <c r="B396" s="2" t="inlineStr">
@@ -13084,54 +13084,54 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>A6519</t>
+          <t>A5679</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723479</t>
+          <t>00019200000012756008</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:33</t>
+          <t>09/06/2026 09:08</t>
         </is>
       </c>
       <c r="F396" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 12:15</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>556160</t>
+          <t>556744</t>
         </is>
       </c>
       <c r="B397" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>A9538</t>
+          <t>A6519</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730009</t>
+          <t>00019200000012723479</t>
         </is>
       </c>
       <c r="E397" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 11:33</t>
+          <t>08/06/2026 05:33</t>
         </is>
       </c>
       <c r="F397" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 11:46</t>
+          <t>09/06/2026 12:15</t>
         </is>
       </c>
     </row>
@@ -13148,12 +13148,12 @@
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>TA0617</t>
+          <t>A9538</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730882</t>
+          <t>00019200000012730009</t>
         </is>
       </c>
       <c r="E398" s="2" t="inlineStr">
@@ -13180,12 +13180,12 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>A5841</t>
+          <t>TA0617</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730890</t>
+          <t>00019200000012730882</t>
         </is>
       </c>
       <c r="E399" s="2" t="inlineStr">
@@ -13212,12 +13212,12 @@
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>A7704</t>
+          <t>A5841</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730904</t>
+          <t>00019200000012730890</t>
         </is>
       </c>
       <c r="E400" s="2" t="inlineStr">
@@ -13244,12 +13244,12 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>A6707</t>
+          <t>A7704</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730912</t>
+          <t>00019200000012730904</t>
         </is>
       </c>
       <c r="E401" s="2" t="inlineStr">
@@ -13274,10 +13274,14 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C402" s="2" t="inlineStr"/>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>A6707</t>
+        </is>
+      </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730920</t>
+          <t>00019200000012730912</t>
         </is>
       </c>
       <c r="E402" s="2" t="inlineStr">
@@ -13302,14 +13306,10 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C403" s="2" t="inlineStr">
-        <is>
-          <t>A5971</t>
-        </is>
-      </c>
+      <c r="C403" s="2" t="inlineStr"/>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730939</t>
+          <t>00019200000012730920</t>
         </is>
       </c>
       <c r="E403" s="2" t="inlineStr">
@@ -13336,12 +13336,12 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A5971</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731005</t>
+          <t>00019200000012730939</t>
         </is>
       </c>
       <c r="E404" s="2" t="inlineStr">
@@ -13368,12 +13368,12 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>A7331</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731560</t>
+          <t>00019200000012731005</t>
         </is>
       </c>
       <c r="E405" s="2" t="inlineStr">
@@ -13400,12 +13400,12 @@
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>A2361</t>
+          <t>A7331</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731579</t>
+          <t>00019200000012731560</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr">
@@ -13432,12 +13432,12 @@
       </c>
       <c r="C407" s="2" t="inlineStr">
         <is>
-          <t>A9716</t>
+          <t>A2361</t>
         </is>
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731587</t>
+          <t>00019200000012731579</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr">
@@ -13464,12 +13464,12 @@
       </c>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>A9274</t>
+          <t>A9716</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731595</t>
+          <t>00019200000012731587</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr">
@@ -13496,12 +13496,12 @@
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
-          <t>A7020</t>
+          <t>A9274</t>
         </is>
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731609</t>
+          <t>00019200000012731595</t>
         </is>
       </c>
       <c r="E409" s="2" t="inlineStr">
@@ -13528,12 +13528,12 @@
       </c>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>A8090</t>
+          <t>A7020</t>
         </is>
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731617</t>
+          <t>00019200000012731609</t>
         </is>
       </c>
       <c r="E410" s="2" t="inlineStr">
@@ -13560,12 +13560,12 @@
       </c>
       <c r="C411" s="2" t="inlineStr">
         <is>
-          <t>A2173</t>
+          <t>A8090</t>
         </is>
       </c>
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731625</t>
+          <t>00019200000012731617</t>
         </is>
       </c>
       <c r="E411" s="2" t="inlineStr">
@@ -13592,12 +13592,12 @@
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>A5456</t>
+          <t>A2173</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731633</t>
+          <t>00019200000012731625</t>
         </is>
       </c>
       <c r="E412" s="2" t="inlineStr">
@@ -13624,12 +13624,12 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>A8993</t>
+          <t>A5456</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731641</t>
+          <t>00019200000012731633</t>
         </is>
       </c>
       <c r="E413" s="2" t="inlineStr">
@@ -13656,12 +13656,12 @@
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>A7043</t>
+          <t>A8993</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731650</t>
+          <t>00019200000012731641</t>
         </is>
       </c>
       <c r="E414" s="2" t="inlineStr">
@@ -13688,12 +13688,12 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>A6600</t>
+          <t>A7043</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731668</t>
+          <t>00019200000012731650</t>
         </is>
       </c>
       <c r="E415" s="2" t="inlineStr">
@@ -13720,12 +13720,12 @@
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>A6518</t>
+          <t>A6600</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731676</t>
+          <t>00019200000012731668</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr">
@@ -13752,12 +13752,12 @@
       </c>
       <c r="C417" s="2" t="inlineStr">
         <is>
-          <t>A6804</t>
+          <t>A6518</t>
         </is>
       </c>
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731684</t>
+          <t>00019200000012731676</t>
         </is>
       </c>
       <c r="E417" s="2" t="inlineStr">
@@ -13784,12 +13784,12 @@
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>A1679</t>
+          <t>A6804</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731692</t>
+          <t>00019200000012731684</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
@@ -13816,12 +13816,12 @@
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>A6311</t>
+          <t>A1679</t>
         </is>
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731803</t>
+          <t>00019200000012731692</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
@@ -13848,12 +13848,12 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>TA0484</t>
+          <t>A6311</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731900</t>
+          <t>00019200000012731803</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
@@ -13880,12 +13880,12 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>A9205</t>
+          <t>TA0484</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731919</t>
+          <t>00019200000012731900</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
@@ -13912,12 +13912,12 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>A1019</t>
+          <t>A9205</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731927</t>
+          <t>00019200000012731919</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
@@ -13944,12 +13944,12 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>A6694</t>
+          <t>A1019</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731935</t>
+          <t>00019200000012731927</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
@@ -13976,12 +13976,12 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>A4625</t>
+          <t>A6694</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731943</t>
+          <t>00019200000012731935</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr">
@@ -14008,12 +14008,12 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>A7288</t>
+          <t>A4625</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731951</t>
+          <t>00019200000012731943</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
@@ -14040,12 +14040,12 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>A7878</t>
+          <t>A7288</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731960</t>
+          <t>00019200000012731951</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
@@ -14072,12 +14072,12 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>A0974</t>
+          <t>A7878</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731978</t>
+          <t>00019200000012731960</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
@@ -14104,12 +14104,12 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>A8869</t>
+          <t>A0974</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731986</t>
+          <t>00019200000012731978</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
@@ -14136,12 +14136,12 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>A7491</t>
+          <t>A8869</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731994</t>
+          <t>00019200000012731986</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
@@ -14168,12 +14168,12 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>A6871</t>
+          <t>A7491</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732001</t>
+          <t>00019200000012731994</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
@@ -14200,12 +14200,12 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>A1824</t>
+          <t>A6871</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732010</t>
+          <t>00019200000012732001</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
@@ -14232,12 +14232,12 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A1824</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732028</t>
+          <t>00019200000012732010</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
@@ -14264,12 +14264,12 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>A9638</t>
+          <t>A9207</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732036</t>
+          <t>00019200000012732028</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
@@ -14296,12 +14296,12 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>TA1173</t>
+          <t>A9638</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732044</t>
+          <t>00019200000012732036</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
@@ -14328,12 +14328,12 @@
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>A9280</t>
+          <t>TA1173</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732052</t>
+          <t>00019200000012732044</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
@@ -14360,12 +14360,12 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>A6843</t>
+          <t>A9280</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732060</t>
+          <t>00019200000012732052</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -14392,12 +14392,12 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>A8045</t>
+          <t>A6843</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732079</t>
+          <t>00019200000012732060</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
@@ -14424,12 +14424,12 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A8045</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732087</t>
+          <t>00019200000012732079</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
@@ -14456,12 +14456,12 @@
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>A1989</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732095</t>
+          <t>00019200000012732087</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
@@ -14488,12 +14488,12 @@
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>TA0654</t>
+          <t>A1989</t>
         </is>
       </c>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732109</t>
+          <t>00019200000012732095</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr">
@@ -14520,12 +14520,12 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>A4447</t>
+          <t>TA0654</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732117</t>
+          <t>00019200000012732109</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
@@ -14552,12 +14552,12 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>A8046</t>
+          <t>A4447</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732125</t>
+          <t>00019200000012732117</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
@@ -14584,12 +14584,12 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>A3920</t>
+          <t>A8046</t>
         </is>
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732133</t>
+          <t>00019200000012732125</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr">
@@ -14616,12 +14616,12 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>A7425</t>
+          <t>A3920</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732141</t>
+          <t>00019200000012732133</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
@@ -14648,12 +14648,12 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>A3679</t>
+          <t>A7425</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732150</t>
+          <t>00019200000012732141</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
@@ -14680,12 +14680,12 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>A7985</t>
+          <t>A3679</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732168</t>
+          <t>00019200000012732150</t>
         </is>
       </c>
       <c r="E446" s="2" t="inlineStr">
@@ -14712,12 +14712,12 @@
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>A6562</t>
+          <t>A7985</t>
         </is>
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732176</t>
+          <t>00019200000012732168</t>
         </is>
       </c>
       <c r="E447" s="2" t="inlineStr">
@@ -14744,12 +14744,12 @@
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>A4360</t>
+          <t>A6562</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732184</t>
+          <t>00019200000012732176</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
@@ -14776,12 +14776,12 @@
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>A9173</t>
+          <t>A4360</t>
         </is>
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732192</t>
+          <t>00019200000012732184</t>
         </is>
       </c>
       <c r="E449" s="2" t="inlineStr">
@@ -14808,12 +14808,12 @@
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>A2809</t>
+          <t>A9173</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732206</t>
+          <t>00019200000012732192</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
@@ -14840,12 +14840,12 @@
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>TA0960</t>
+          <t>A2809</t>
         </is>
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732214</t>
+          <t>00019200000012732206</t>
         </is>
       </c>
       <c r="E451" s="2" t="inlineStr">
@@ -14872,12 +14872,12 @@
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>TA0960</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732222</t>
+          <t>00019200000012732214</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
@@ -14904,12 +14904,12 @@
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>A9307</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732230</t>
+          <t>00019200000012732222</t>
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr">
@@ -14936,12 +14936,12 @@
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>A7068</t>
+          <t>A9307</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732249</t>
+          <t>00019200000012732230</t>
         </is>
       </c>
       <c r="E454" s="2" t="inlineStr">
@@ -14968,12 +14968,12 @@
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>A3376</t>
+          <t>A7068</t>
         </is>
       </c>
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732257</t>
+          <t>00019200000012732249</t>
         </is>
       </c>
       <c r="E455" s="2" t="inlineStr">
@@ -15000,12 +15000,12 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>A3287</t>
+          <t>A3376</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732265</t>
+          <t>00019200000012732257</t>
         </is>
       </c>
       <c r="E456" s="2" t="inlineStr">
@@ -15032,12 +15032,12 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>A9200</t>
+          <t>A3287</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732273</t>
+          <t>00019200000012732265</t>
         </is>
       </c>
       <c r="E457" s="2" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>A5037</t>
+          <t>A9200</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732281</t>
+          <t>00019200000012732273</t>
         </is>
       </c>
       <c r="E458" s="2" t="inlineStr">
@@ -15096,12 +15096,12 @@
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>A9610</t>
+          <t>A5037</t>
         </is>
       </c>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732290</t>
+          <t>00019200000012732281</t>
         </is>
       </c>
       <c r="E459" s="2" t="inlineStr">
@@ -15128,12 +15128,12 @@
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>A1420</t>
+          <t>A9610</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>00019200000012857750</t>
+          <t>00019200000012732290</t>
         </is>
       </c>
       <c r="E460" s="2" t="inlineStr">
@@ -15150,7 +15150,7 @@
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>556224</t>
+          <t>556160</t>
         </is>
       </c>
       <c r="B461" s="2" t="inlineStr">
@@ -15160,29 +15160,29 @@
       </c>
       <c r="C461" s="2" t="inlineStr">
         <is>
-          <t>A4220</t>
+          <t>A1420</t>
         </is>
       </c>
       <c r="D461" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729043</t>
+          <t>00019200000012857750</t>
         </is>
       </c>
       <c r="E461" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 05:11</t>
+          <t>06/06/2026 11:33</t>
         </is>
       </c>
       <c r="F461" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 16:00</t>
+          <t>08/06/2026 11:46</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>556409</t>
+          <t>556224</t>
         </is>
       </c>
       <c r="B462" s="2" t="inlineStr">
@@ -15192,22 +15192,22 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>A8078</t>
+          <t>A4220</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723550</t>
+          <t>00019200000012729043</t>
         </is>
       </c>
       <c r="E462" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 06:40</t>
+          <t>11/06/2026 05:11</t>
         </is>
       </c>
       <c r="F462" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:18</t>
+          <t>12/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -15224,12 +15224,12 @@
       </c>
       <c r="C463" s="2" t="inlineStr">
         <is>
-          <t>A0401</t>
+          <t>A8078</t>
         </is>
       </c>
       <c r="D463" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723568</t>
+          <t>00019200000012723550</t>
         </is>
       </c>
       <c r="E463" s="2" t="inlineStr">
@@ -15256,12 +15256,12 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>A8580</t>
+          <t>A0401</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723592</t>
+          <t>00019200000012723568</t>
         </is>
       </c>
       <c r="E464" s="2" t="inlineStr">
@@ -15278,32 +15278,32 @@
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>555932</t>
+          <t>556409</t>
         </is>
       </c>
       <c r="B465" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>A4257</t>
+          <t>A8580</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721840</t>
+          <t>00019200000012723592</t>
         </is>
       </c>
       <c r="E465" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:18</t>
+          <t>10/06/2026 06:40</t>
         </is>
       </c>
       <c r="F465" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:33</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -15320,12 +15320,12 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>A9287</t>
+          <t>A4257</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723061</t>
+          <t>00019200000012721840</t>
         </is>
       </c>
       <c r="E466" s="2" t="inlineStr">
@@ -15342,7 +15342,7 @@
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>556161</t>
+          <t>555932</t>
         </is>
       </c>
       <c r="B467" s="2" t="inlineStr">
@@ -15352,22 +15352,22 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>A7008</t>
+          <t>A9287</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730491</t>
+          <t>00019200000012723061</t>
         </is>
       </c>
       <c r="E467" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:18</t>
         </is>
       </c>
       <c r="F467" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:51</t>
+          <t>03/06/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -15384,12 +15384,12 @@
       </c>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>A7785</t>
+          <t>A7008</t>
         </is>
       </c>
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730670</t>
+          <t>00019200000012730491</t>
         </is>
       </c>
       <c r="E468" s="2" t="inlineStr">
@@ -15416,12 +15416,12 @@
       </c>
       <c r="C469" s="2" t="inlineStr">
         <is>
-          <t>A6386</t>
+          <t>A7785</t>
         </is>
       </c>
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730688</t>
+          <t>00019200000012730670</t>
         </is>
       </c>
       <c r="E469" s="2" t="inlineStr">
@@ -15448,12 +15448,12 @@
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>A8302</t>
+          <t>A6386</t>
         </is>
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730696</t>
+          <t>00019200000012730688</t>
         </is>
       </c>
       <c r="E470" s="2" t="inlineStr">
@@ -15480,12 +15480,12 @@
       </c>
       <c r="C471" s="2" t="inlineStr">
         <is>
-          <t>A6870</t>
+          <t>A8302</t>
         </is>
       </c>
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730700</t>
+          <t>00019200000012730696</t>
         </is>
       </c>
       <c r="E471" s="2" t="inlineStr">
@@ -15512,12 +15512,12 @@
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>A8192</t>
+          <t>A6870</t>
         </is>
       </c>
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731331</t>
+          <t>00019200000012730700</t>
         </is>
       </c>
       <c r="E472" s="2" t="inlineStr">
@@ -15544,12 +15544,12 @@
       </c>
       <c r="C473" s="2" t="inlineStr">
         <is>
-          <t>A1045</t>
+          <t>A8192</t>
         </is>
       </c>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731340</t>
+          <t>00019200000012731331</t>
         </is>
       </c>
       <c r="E473" s="2" t="inlineStr">
@@ -15576,12 +15576,12 @@
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>A3603</t>
+          <t>A1045</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731358</t>
+          <t>00019200000012731340</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr">
@@ -15608,12 +15608,12 @@
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>A9427</t>
+          <t>A3603</t>
         </is>
       </c>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731366</t>
+          <t>00019200000012731358</t>
         </is>
       </c>
       <c r="E475" s="2" t="inlineStr">
@@ -15640,12 +15640,12 @@
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>A4068</t>
+          <t>A9427</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731374</t>
+          <t>00019200000012731366</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr">
@@ -15672,12 +15672,12 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>A2753</t>
+          <t>A4068</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731382</t>
+          <t>00019200000012731374</t>
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr">
@@ -15704,12 +15704,12 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>TA0353</t>
+          <t>A2753</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731390</t>
+          <t>00019200000012731382</t>
         </is>
       </c>
       <c r="E478" s="2" t="inlineStr">
@@ -15736,12 +15736,12 @@
       </c>
       <c r="C479" s="2" t="inlineStr">
         <is>
-          <t>A7155</t>
+          <t>TA0353</t>
         </is>
       </c>
       <c r="D479" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731404</t>
+          <t>00019200000012731390</t>
         </is>
       </c>
       <c r="E479" s="2" t="inlineStr">
@@ -15768,12 +15768,12 @@
       </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>A6665</t>
+          <t>A7155</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731412</t>
+          <t>00019200000012731404</t>
         </is>
       </c>
       <c r="E480" s="2" t="inlineStr">
@@ -15800,12 +15800,12 @@
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>TA0675</t>
+          <t>A6665</t>
         </is>
       </c>
       <c r="D481" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731420</t>
+          <t>00019200000012731412</t>
         </is>
       </c>
       <c r="E481" s="2" t="inlineStr">
@@ -15832,12 +15832,12 @@
       </c>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>A7142</t>
+          <t>TA0675</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731439</t>
+          <t>00019200000012731420</t>
         </is>
       </c>
       <c r="E482" s="2" t="inlineStr">
@@ -15864,12 +15864,12 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>TA0136</t>
+          <t>A7142</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731447</t>
+          <t>00019200000012731439</t>
         </is>
       </c>
       <c r="E483" s="2" t="inlineStr">
@@ -15896,12 +15896,12 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>TA0818</t>
+          <t>TA0136</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731455</t>
+          <t>00019200000012731447</t>
         </is>
       </c>
       <c r="E484" s="2" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>A6147</t>
+          <t>TA0818</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731463</t>
+          <t>00019200000012731455</t>
         </is>
       </c>
       <c r="E485" s="2" t="inlineStr">
@@ -15960,12 +15960,12 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>A4999</t>
+          <t>A6147</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731471</t>
+          <t>00019200000012731463</t>
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr">
@@ -15992,12 +15992,12 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>A5847</t>
+          <t>A4999</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731498</t>
+          <t>00019200000012731471</t>
         </is>
       </c>
       <c r="E487" s="2" t="inlineStr">
@@ -16024,12 +16024,12 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>A2981</t>
+          <t>A5847</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731501</t>
+          <t>00019200000012731498</t>
         </is>
       </c>
       <c r="E488" s="2" t="inlineStr">
@@ -16056,12 +16056,12 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>A7462</t>
+          <t>A2981</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731510</t>
+          <t>00019200000012731501</t>
         </is>
       </c>
       <c r="E489" s="2" t="inlineStr">
@@ -16088,12 +16088,12 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>A4340</t>
+          <t>A7462</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731528</t>
+          <t>00019200000012731510</t>
         </is>
       </c>
       <c r="E490" s="2" t="inlineStr">
@@ -16120,12 +16120,12 @@
       </c>
       <c r="C491" s="2" t="inlineStr">
         <is>
-          <t>A8938</t>
+          <t>A4340</t>
         </is>
       </c>
       <c r="D491" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731536</t>
+          <t>00019200000012731528</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr">
@@ -16142,7 +16142,7 @@
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>556300</t>
+          <t>556161</t>
         </is>
       </c>
       <c r="B492" s="2" t="inlineStr">
@@ -16152,54 +16152,54 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>TA0506</t>
+          <t>A8938</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728918</t>
+          <t>00019200000012731536</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 10:36</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F492" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:54</t>
+          <t>08/06/2026 14:51</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>556300</t>
         </is>
       </c>
       <c r="B493" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>TA0506</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000012728918</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>06/06/2026 10:36</t>
         </is>
       </c>
       <c r="F493" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>08/06/2026 10:54</t>
         </is>
       </c>
     </row>
@@ -16216,12 +16216,12 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr">
@@ -16248,12 +16248,12 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E495" s="2" t="inlineStr">
@@ -16270,39 +16270,39 @@
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B496" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D496" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E496" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F496" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B497" s="2" t="inlineStr">
@@ -16312,22 +16312,22 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E497" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F497" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -16344,12 +16344,12 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E498" s="2" t="inlineStr">
@@ -16376,12 +16376,12 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E499" s="2" t="inlineStr">
@@ -16408,12 +16408,12 @@
       </c>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D500" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E500" s="2" t="inlineStr">
@@ -16440,12 +16440,12 @@
       </c>
       <c r="C501" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D501" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E501" s="2" t="inlineStr">
@@ -16472,12 +16472,12 @@
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E502" s="2" t="inlineStr">
@@ -16504,12 +16504,12 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E503" s="2" t="inlineStr">
@@ -16536,12 +16536,12 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E504" s="2" t="inlineStr">
@@ -16568,12 +16568,12 @@
       </c>
       <c r="C505" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D505" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E505" s="2" t="inlineStr">
@@ -16600,12 +16600,12 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E506" s="2" t="inlineStr">
@@ -16632,12 +16632,12 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E507" s="2" t="inlineStr">
@@ -16664,12 +16664,12 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
@@ -16696,12 +16696,12 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E509" s="2" t="inlineStr">
@@ -16728,12 +16728,12 @@
       </c>
       <c r="C510" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr">
@@ -16760,12 +16760,12 @@
       </c>
       <c r="C511" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D511" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E511" s="2" t="inlineStr">
@@ -16782,7 +16782,7 @@
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B512" s="2" t="inlineStr">
@@ -16792,22 +16792,22 @@
       </c>
       <c r="C512" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D512" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E512" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F512" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -16824,12 +16824,12 @@
       </c>
       <c r="C513" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D513" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E513" s="2" t="inlineStr">
@@ -16856,12 +16856,12 @@
       </c>
       <c r="C514" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D514" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E514" s="2" t="inlineStr">
@@ -16888,12 +16888,12 @@
       </c>
       <c r="C515" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D515" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E515" s="2" t="inlineStr">
@@ -16920,27 +16920,59 @@
       </c>
       <c r="C516" s="2" t="inlineStr">
         <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B517" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
           <t>A8196</t>
         </is>
       </c>
-      <c r="D516" s="2" t="inlineStr">
+      <c r="D517" s="2" t="inlineStr">
         <is>
           <t>00019200000012728802</t>
         </is>
       </c>
-      <c r="E516" s="2" t="inlineStr">
+      <c r="E517" s="2" t="inlineStr">
         <is>
           <t>09/06/2026 02:06</t>
         </is>
       </c>
-      <c r="F516" s="2" t="inlineStr">
+      <c r="F517" s="2" t="inlineStr">
         <is>
           <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F516"/>
+  <autoFilter ref="A1:F517"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-15 07:12:33
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$553</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$554</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F553"/>
+  <dimension ref="A1:F554"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10738,39 +10738,39 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>555911</t>
+          <t>556923</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>A4881</t>
+          <t>TA0216</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715298</t>
+          <t>00019200000012656143</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:02</t>
+          <t>15/06/2026 06:58</t>
         </is>
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>556157</t>
+          <t>555911</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
@@ -10780,12 +10780,12 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>TA0188</t>
+          <t>A4881</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730203</t>
+          <t>00019200000012715298</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:00</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -10812,12 +10812,12 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>TA0670</t>
+          <t>TA0188</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730211</t>
+          <t>00019200000012730203</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
@@ -10844,12 +10844,12 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>A3810</t>
+          <t>TA0670</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730220</t>
+          <t>00019200000012730211</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
@@ -10876,12 +10876,12 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>A0800</t>
+          <t>A3810</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730238</t>
+          <t>00019200000012730220</t>
         </is>
       </c>
       <c r="E327" s="2" t="inlineStr">
@@ -10908,12 +10908,12 @@
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>A5751</t>
+          <t>A0800</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730246</t>
+          <t>00019200000012730238</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
@@ -10940,12 +10940,12 @@
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>A3830</t>
+          <t>A5751</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730254</t>
+          <t>00019200000012730246</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
@@ -10972,12 +10972,12 @@
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>A2419</t>
+          <t>A3830</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730262</t>
+          <t>00019200000012730254</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
@@ -11004,12 +11004,12 @@
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>A7535</t>
+          <t>A2419</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730270</t>
+          <t>00019200000012730262</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
@@ -11036,12 +11036,12 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>A5563</t>
+          <t>A7535</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730289</t>
+          <t>00019200000012730270</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
@@ -11068,12 +11068,12 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>A9066</t>
+          <t>A5563</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730297</t>
+          <t>00019200000012730289</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
@@ -11100,12 +11100,12 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>A5828</t>
+          <t>A9066</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730300</t>
+          <t>00019200000012730297</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
@@ -11132,12 +11132,12 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>A4055</t>
+          <t>A5828</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730319</t>
+          <t>00019200000012730300</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
@@ -11164,12 +11164,12 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>A0130</t>
+          <t>A4055</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730327</t>
+          <t>00019200000012730319</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
@@ -11196,12 +11196,12 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>A7797</t>
+          <t>A0130</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730335</t>
+          <t>00019200000012730327</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -11228,12 +11228,12 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>A9654</t>
+          <t>A7797</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730343</t>
+          <t>00019200000012730335</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
@@ -11260,12 +11260,12 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>A7482</t>
+          <t>A9654</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730351</t>
+          <t>00019200000012730343</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
@@ -11292,12 +11292,12 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>A7723</t>
+          <t>A7482</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730360</t>
+          <t>00019200000012730351</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -11324,12 +11324,12 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>A7997</t>
+          <t>A7723</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730378</t>
+          <t>00019200000012730360</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
@@ -11346,7 +11346,7 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>556258</t>
+          <t>556157</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
@@ -11356,17 +11356,17 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>A6961</t>
+          <t>A7997</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729159</t>
+          <t>00019200000012730378</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>06/06/2026 05:02</t>
         </is>
       </c>
       <c r="F342" s="2" t="inlineStr">
@@ -11378,22 +11378,22 @@
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>556158</t>
+          <t>556258</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>A8351</t>
+          <t>A6961</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715344</t>
+          <t>00019200000012729159</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F343" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:00</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -11420,12 +11420,12 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>A6522</t>
+          <t>A8351</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715352</t>
+          <t>00019200000012715344</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
@@ -11452,12 +11452,12 @@
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>A7263</t>
+          <t>A6522</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715360</t>
+          <t>00019200000012715352</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
@@ -11484,12 +11484,12 @@
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>A9019</t>
+          <t>A7263</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715379</t>
+          <t>00019200000012715360</t>
         </is>
       </c>
       <c r="E346" s="2" t="inlineStr">
@@ -11516,12 +11516,12 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>A4823</t>
+          <t>A9019</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715387</t>
+          <t>00019200000012715379</t>
         </is>
       </c>
       <c r="E347" s="2" t="inlineStr">
@@ -11548,12 +11548,12 @@
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>A5775</t>
+          <t>A4823</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715395</t>
+          <t>00019200000012715387</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
@@ -11580,12 +11580,12 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>A6931</t>
+          <t>A5775</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715409</t>
+          <t>00019200000012715395</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
@@ -11602,32 +11602,32 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>556159</t>
+          <t>556158</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>TA1119</t>
+          <t>A6931</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753440</t>
+          <t>00019200000012715409</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:08</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 13:30</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -11644,12 +11644,12 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>A6893</t>
+          <t>TA1119</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753459</t>
+          <t>00019200000012753440</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
@@ -11676,12 +11676,12 @@
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>A8127</t>
+          <t>A6893</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753467</t>
+          <t>00019200000012753459</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
@@ -11708,12 +11708,12 @@
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>A6189</t>
+          <t>A8127</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753475</t>
+          <t>00019200000012753467</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
@@ -11740,12 +11740,12 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>TA0776</t>
+          <t>A6189</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753483</t>
+          <t>00019200000012753475</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
@@ -11772,12 +11772,12 @@
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>A8534</t>
+          <t>TA0776</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753491</t>
+          <t>00019200000012753483</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
@@ -11804,12 +11804,12 @@
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>A7575</t>
+          <t>A8534</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753505</t>
+          <t>00019200000012753491</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
@@ -11836,12 +11836,12 @@
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>A0609</t>
+          <t>A7575</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753513</t>
+          <t>00019200000012753505</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
@@ -11868,12 +11868,12 @@
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>A9499</t>
+          <t>A0609</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753521</t>
+          <t>00019200000012753513</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
@@ -11900,12 +11900,12 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>A6581</t>
+          <t>A9499</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753530</t>
+          <t>00019200000012753521</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
@@ -11932,12 +11932,12 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>A8536</t>
+          <t>A6581</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753548</t>
+          <t>00019200000012753530</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
@@ -11964,12 +11964,12 @@
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>A9316</t>
+          <t>A8536</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753556</t>
+          <t>00019200000012753548</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
@@ -11996,12 +11996,12 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>TA0880</t>
+          <t>A9316</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753564</t>
+          <t>00019200000012753556</t>
         </is>
       </c>
       <c r="E362" s="2" t="inlineStr">
@@ -12028,12 +12028,12 @@
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>A1933</t>
+          <t>TA0880</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753572</t>
+          <t>00019200000012753564</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
@@ -12060,12 +12060,12 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>A0504</t>
+          <t>A1933</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753882</t>
+          <t>00019200000012753572</t>
         </is>
       </c>
       <c r="E364" s="2" t="inlineStr">
@@ -12092,12 +12092,12 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>TA0704</t>
+          <t>A0504</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753890</t>
+          <t>00019200000012753882</t>
         </is>
       </c>
       <c r="E365" s="2" t="inlineStr">
@@ -12124,12 +12124,12 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>A8967</t>
+          <t>TA0704</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753904</t>
+          <t>00019200000012753890</t>
         </is>
       </c>
       <c r="E366" s="2" t="inlineStr">
@@ -12156,12 +12156,12 @@
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>A4337</t>
+          <t>A8967</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753912</t>
+          <t>00019200000012753904</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
@@ -12188,12 +12188,12 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>A5175</t>
+          <t>A4337</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753920</t>
+          <t>00019200000012753912</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
@@ -12220,12 +12220,12 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>TA0974</t>
+          <t>A5175</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753939</t>
+          <t>00019200000012753920</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
@@ -12252,12 +12252,12 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>A6700</t>
+          <t>TA0974</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753947</t>
+          <t>00019200000012753939</t>
         </is>
       </c>
       <c r="E370" s="2" t="inlineStr">
@@ -12284,12 +12284,12 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>A8361</t>
+          <t>A6700</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753955</t>
+          <t>00019200000012753947</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
@@ -12316,12 +12316,12 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>A3121</t>
+          <t>A8361</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753963</t>
+          <t>00019200000012753955</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
@@ -12348,12 +12348,12 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>A8154</t>
+          <t>A3121</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753971</t>
+          <t>00019200000012753963</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
@@ -12380,12 +12380,12 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>TA0597</t>
+          <t>A8154</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753980</t>
+          <t>00019200000012753971</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr">
@@ -12412,12 +12412,12 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>A6883</t>
+          <t>TA0597</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753998</t>
+          <t>00019200000012753980</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
@@ -12444,12 +12444,12 @@
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>A9704</t>
+          <t>A6883</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754005</t>
+          <t>00019200000012753998</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
@@ -12476,12 +12476,12 @@
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>A9302</t>
+          <t>A9704</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754013</t>
+          <t>00019200000012754005</t>
         </is>
       </c>
       <c r="E377" s="2" t="inlineStr">
@@ -12508,12 +12508,12 @@
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>A0119</t>
+          <t>A9302</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754021</t>
+          <t>00019200000012754013</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
@@ -12540,12 +12540,12 @@
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>A9040</t>
+          <t>A0119</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754048</t>
+          <t>00019200000012754021</t>
         </is>
       </c>
       <c r="E379" s="2" t="inlineStr">
@@ -12572,12 +12572,12 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>A7876</t>
+          <t>A9040</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754056</t>
+          <t>00019200000012754048</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
@@ -12604,12 +12604,12 @@
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>A8919</t>
+          <t>A7876</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754064</t>
+          <t>00019200000012754056</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
@@ -12636,12 +12636,12 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>A6393</t>
+          <t>A8919</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754072</t>
+          <t>00019200000012754064</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
@@ -12668,12 +12668,12 @@
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>A4317</t>
+          <t>A6393</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754080</t>
+          <t>00019200000012754072</t>
         </is>
       </c>
       <c r="E383" s="2" t="inlineStr">
@@ -12700,12 +12700,12 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>A8657</t>
+          <t>A4317</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754099</t>
+          <t>00019200000012754080</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
@@ -12732,12 +12732,12 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>A8940</t>
+          <t>A8657</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754102</t>
+          <t>00019200000012754099</t>
         </is>
       </c>
       <c r="E385" s="2" t="inlineStr">
@@ -12764,12 +12764,12 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>A6261</t>
+          <t>A8940</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754110</t>
+          <t>00019200000012754102</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
@@ -12796,12 +12796,12 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>A5569</t>
+          <t>A6261</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754129</t>
+          <t>00019200000012754110</t>
         </is>
       </c>
       <c r="E387" s="2" t="inlineStr">
@@ -12828,12 +12828,12 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>A8748</t>
+          <t>A5569</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754137</t>
+          <t>00019200000012754129</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
@@ -12860,12 +12860,12 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>A9213</t>
+          <t>A8748</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754145</t>
+          <t>00019200000012754137</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr">
@@ -12892,12 +12892,12 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>TA0226</t>
+          <t>A9213</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754153</t>
+          <t>00019200000012754145</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
@@ -12924,12 +12924,12 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>A8485</t>
+          <t>TA0226</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754161</t>
+          <t>00019200000012754153</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
@@ -12956,12 +12956,12 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>A8095</t>
+          <t>A8485</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754170</t>
+          <t>00019200000012754161</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
@@ -12988,12 +12988,12 @@
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>A9152</t>
+          <t>A8095</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754188</t>
+          <t>00019200000012754170</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
@@ -13020,12 +13020,12 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>A7849</t>
+          <t>A9152</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754196</t>
+          <t>00019200000012754188</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
@@ -13052,12 +13052,12 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>A6854</t>
+          <t>A7849</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754200</t>
+          <t>00019200000012754196</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
@@ -13084,12 +13084,12 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>A8670</t>
+          <t>A6854</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754218</t>
+          <t>00019200000012754200</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
@@ -13116,12 +13116,12 @@
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>A8352</t>
+          <t>A8670</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754226</t>
+          <t>00019200000012754218</t>
         </is>
       </c>
       <c r="E397" s="2" t="inlineStr">
@@ -13148,12 +13148,12 @@
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>A6584</t>
+          <t>A8352</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754234</t>
+          <t>00019200000012754226</t>
         </is>
       </c>
       <c r="E398" s="2" t="inlineStr">
@@ -13180,12 +13180,12 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>A5394</t>
+          <t>A6584</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754242</t>
+          <t>00019200000012754234</t>
         </is>
       </c>
       <c r="E399" s="2" t="inlineStr">
@@ -13212,12 +13212,12 @@
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>A9258</t>
+          <t>A5394</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754250</t>
+          <t>00019200000012754242</t>
         </is>
       </c>
       <c r="E400" s="2" t="inlineStr">
@@ -13244,12 +13244,12 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>A2475</t>
+          <t>A9258</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754269</t>
+          <t>00019200000012754250</t>
         </is>
       </c>
       <c r="E401" s="2" t="inlineStr">
@@ -13276,12 +13276,12 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>A8952</t>
+          <t>A2475</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754277</t>
+          <t>00019200000012754269</t>
         </is>
       </c>
       <c r="E402" s="2" t="inlineStr">
@@ -13308,12 +13308,12 @@
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>A6781</t>
+          <t>A8952</t>
         </is>
       </c>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754285</t>
+          <t>00019200000012754277</t>
         </is>
       </c>
       <c r="E403" s="2" t="inlineStr">
@@ -13340,12 +13340,12 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>A8379</t>
+          <t>A6781</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754293</t>
+          <t>00019200000012754285</t>
         </is>
       </c>
       <c r="E404" s="2" t="inlineStr">
@@ -13372,12 +13372,12 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>A8243</t>
+          <t>A8379</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754307</t>
+          <t>00019200000012754293</t>
         </is>
       </c>
       <c r="E405" s="2" t="inlineStr">
@@ -13404,12 +13404,12 @@
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>A7097</t>
+          <t>A8243</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754315</t>
+          <t>00019200000012754307</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr">
@@ -13436,12 +13436,12 @@
       </c>
       <c r="C407" s="2" t="inlineStr">
         <is>
-          <t>TA0235</t>
+          <t>A7097</t>
         </is>
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754323</t>
+          <t>00019200000012754315</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr">
@@ -13468,12 +13468,12 @@
       </c>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>A8222</t>
+          <t>TA0235</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754331</t>
+          <t>00019200000012754323</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr">
@@ -13500,12 +13500,12 @@
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
-          <t>A1510</t>
+          <t>A8222</t>
         </is>
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754340</t>
+          <t>00019200000012754331</t>
         </is>
       </c>
       <c r="E409" s="2" t="inlineStr">
@@ -13532,12 +13532,12 @@
       </c>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>A0773</t>
+          <t>A1510</t>
         </is>
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754358</t>
+          <t>00019200000012754340</t>
         </is>
       </c>
       <c r="E410" s="2" t="inlineStr">
@@ -13564,12 +13564,12 @@
       </c>
       <c r="C411" s="2" t="inlineStr">
         <is>
-          <t>A8448</t>
+          <t>A0773</t>
         </is>
       </c>
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754366</t>
+          <t>00019200000012754358</t>
         </is>
       </c>
       <c r="E411" s="2" t="inlineStr">
@@ -13596,12 +13596,12 @@
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>A7767</t>
+          <t>A8448</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754374</t>
+          <t>00019200000012754366</t>
         </is>
       </c>
       <c r="E412" s="2" t="inlineStr">
@@ -13628,12 +13628,12 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>A8254</t>
+          <t>A7767</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754382</t>
+          <t>00019200000012754374</t>
         </is>
       </c>
       <c r="E413" s="2" t="inlineStr">
@@ -13660,12 +13660,12 @@
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>A9361</t>
+          <t>A8254</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754390</t>
+          <t>00019200000012754382</t>
         </is>
       </c>
       <c r="E414" s="2" t="inlineStr">
@@ -13692,12 +13692,12 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>A5087</t>
+          <t>A9361</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754404</t>
+          <t>00019200000012754390</t>
         </is>
       </c>
       <c r="E415" s="2" t="inlineStr">
@@ -13724,12 +13724,12 @@
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>A0387</t>
+          <t>A5087</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754412</t>
+          <t>00019200000012754404</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr">
@@ -13756,12 +13756,12 @@
       </c>
       <c r="C417" s="2" t="inlineStr">
         <is>
-          <t>A6996</t>
+          <t>A0387</t>
         </is>
       </c>
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754420</t>
+          <t>00019200000012754412</t>
         </is>
       </c>
       <c r="E417" s="2" t="inlineStr">
@@ -13788,12 +13788,12 @@
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>A7094</t>
+          <t>A6996</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754439</t>
+          <t>00019200000012754420</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
@@ -13820,12 +13820,12 @@
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>A7194</t>
+          <t>A7094</t>
         </is>
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754447</t>
+          <t>00019200000012754439</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
@@ -13852,12 +13852,12 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>A6941</t>
+          <t>A7194</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754455</t>
+          <t>00019200000012754447</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
@@ -13884,12 +13884,12 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>A6571</t>
+          <t>A6941</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754463</t>
+          <t>00019200000012754455</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
@@ -13916,12 +13916,12 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>A5633</t>
+          <t>A6571</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754471</t>
+          <t>00019200000012754463</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
@@ -13948,12 +13948,12 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>A9483</t>
+          <t>A5633</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754480</t>
+          <t>00019200000012754471</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
@@ -13980,12 +13980,12 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>A9277</t>
+          <t>A9483</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754498</t>
+          <t>00019200000012754480</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr">
@@ -14012,12 +14012,12 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>A6305</t>
+          <t>A9277</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754501</t>
+          <t>00019200000012754498</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
@@ -14044,12 +14044,12 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>A0745</t>
+          <t>A6305</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754510</t>
+          <t>00019200000012754501</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
@@ -14076,12 +14076,12 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>A7451</t>
+          <t>A0745</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755958</t>
+          <t>00019200000012754510</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
@@ -14108,12 +14108,12 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>A9324</t>
+          <t>A7451</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755966</t>
+          <t>00019200000012755958</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
@@ -14140,12 +14140,12 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>A8491</t>
+          <t>A9324</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755974</t>
+          <t>00019200000012755966</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
@@ -14172,12 +14172,12 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>A9490</t>
+          <t>A8491</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755982</t>
+          <t>00019200000012755974</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
@@ -14204,12 +14204,12 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>A9202</t>
+          <t>A9490</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755990</t>
+          <t>00019200000012755982</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
@@ -14236,12 +14236,12 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>A5679</t>
+          <t>A9202</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>00019200000012756008</t>
+          <t>00019200000012755990</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
@@ -14258,7 +14258,7 @@
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>556744</t>
+          <t>556159</t>
         </is>
       </c>
       <c r="B433" s="2" t="inlineStr">
@@ -14268,54 +14268,54 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>A6519</t>
+          <t>A5679</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723479</t>
+          <t>00019200000012756008</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:33</t>
+          <t>09/06/2026 09:08</t>
         </is>
       </c>
       <c r="F433" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 12:15</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>556160</t>
+          <t>556744</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>A9538</t>
+          <t>A6519</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730009</t>
+          <t>00019200000012723479</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 11:33</t>
+          <t>08/06/2026 05:33</t>
         </is>
       </c>
       <c r="F434" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 11:46</t>
+          <t>09/06/2026 12:15</t>
         </is>
       </c>
     </row>
@@ -14332,12 +14332,12 @@
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>TA0617</t>
+          <t>A9538</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730882</t>
+          <t>00019200000012730009</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
@@ -14364,12 +14364,12 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>A5841</t>
+          <t>TA0617</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730890</t>
+          <t>00019200000012730882</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -14396,12 +14396,12 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>A7704</t>
+          <t>A5841</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730904</t>
+          <t>00019200000012730890</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
@@ -14428,12 +14428,12 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>A6707</t>
+          <t>A7704</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730912</t>
+          <t>00019200000012730904</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
@@ -14458,10 +14458,14 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C439" s="2" t="inlineStr"/>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>A6707</t>
+        </is>
+      </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730920</t>
+          <t>00019200000012730912</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
@@ -14486,14 +14490,10 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C440" s="2" t="inlineStr">
-        <is>
-          <t>A5971</t>
-        </is>
-      </c>
+      <c r="C440" s="2" t="inlineStr"/>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730939</t>
+          <t>00019200000012730920</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr">
@@ -14520,12 +14520,12 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A5971</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731005</t>
+          <t>00019200000012730939</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
@@ -14552,12 +14552,12 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>A7331</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731560</t>
+          <t>00019200000012731005</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
@@ -14584,12 +14584,12 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>A2361</t>
+          <t>A7331</t>
         </is>
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731579</t>
+          <t>00019200000012731560</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr">
@@ -14616,12 +14616,12 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>A9716</t>
+          <t>A2361</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731587</t>
+          <t>00019200000012731579</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
@@ -14648,12 +14648,12 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>A9274</t>
+          <t>A9716</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731595</t>
+          <t>00019200000012731587</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
@@ -14680,12 +14680,12 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>A7020</t>
+          <t>A9274</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731609</t>
+          <t>00019200000012731595</t>
         </is>
       </c>
       <c r="E446" s="2" t="inlineStr">
@@ -14712,12 +14712,12 @@
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>A8090</t>
+          <t>A7020</t>
         </is>
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731617</t>
+          <t>00019200000012731609</t>
         </is>
       </c>
       <c r="E447" s="2" t="inlineStr">
@@ -14744,12 +14744,12 @@
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>A2173</t>
+          <t>A8090</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731625</t>
+          <t>00019200000012731617</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
@@ -14776,12 +14776,12 @@
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>A5456</t>
+          <t>A2173</t>
         </is>
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731633</t>
+          <t>00019200000012731625</t>
         </is>
       </c>
       <c r="E449" s="2" t="inlineStr">
@@ -14808,12 +14808,12 @@
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>A8993</t>
+          <t>A5456</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731641</t>
+          <t>00019200000012731633</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
@@ -14840,12 +14840,12 @@
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>A7043</t>
+          <t>A8993</t>
         </is>
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731650</t>
+          <t>00019200000012731641</t>
         </is>
       </c>
       <c r="E451" s="2" t="inlineStr">
@@ -14872,12 +14872,12 @@
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>A6600</t>
+          <t>A7043</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731668</t>
+          <t>00019200000012731650</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
@@ -14904,12 +14904,12 @@
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>A6518</t>
+          <t>A6600</t>
         </is>
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731676</t>
+          <t>00019200000012731668</t>
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr">
@@ -14936,12 +14936,12 @@
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>A6804</t>
+          <t>A6518</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731684</t>
+          <t>00019200000012731676</t>
         </is>
       </c>
       <c r="E454" s="2" t="inlineStr">
@@ -14968,12 +14968,12 @@
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>A1679</t>
+          <t>A6804</t>
         </is>
       </c>
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731692</t>
+          <t>00019200000012731684</t>
         </is>
       </c>
       <c r="E455" s="2" t="inlineStr">
@@ -15000,12 +15000,12 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>A6311</t>
+          <t>A1679</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731803</t>
+          <t>00019200000012731692</t>
         </is>
       </c>
       <c r="E456" s="2" t="inlineStr">
@@ -15032,12 +15032,12 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>TA0484</t>
+          <t>A6311</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731900</t>
+          <t>00019200000012731803</t>
         </is>
       </c>
       <c r="E457" s="2" t="inlineStr">
@@ -15064,12 +15064,12 @@
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>A9205</t>
+          <t>TA0484</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731919</t>
+          <t>00019200000012731900</t>
         </is>
       </c>
       <c r="E458" s="2" t="inlineStr">
@@ -15096,12 +15096,12 @@
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>A1019</t>
+          <t>A9205</t>
         </is>
       </c>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731927</t>
+          <t>00019200000012731919</t>
         </is>
       </c>
       <c r="E459" s="2" t="inlineStr">
@@ -15128,12 +15128,12 @@
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>A6694</t>
+          <t>A1019</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731935</t>
+          <t>00019200000012731927</t>
         </is>
       </c>
       <c r="E460" s="2" t="inlineStr">
@@ -15160,12 +15160,12 @@
       </c>
       <c r="C461" s="2" t="inlineStr">
         <is>
-          <t>A4625</t>
+          <t>A6694</t>
         </is>
       </c>
       <c r="D461" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731943</t>
+          <t>00019200000012731935</t>
         </is>
       </c>
       <c r="E461" s="2" t="inlineStr">
@@ -15192,12 +15192,12 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>A7288</t>
+          <t>A4625</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731951</t>
+          <t>00019200000012731943</t>
         </is>
       </c>
       <c r="E462" s="2" t="inlineStr">
@@ -15224,12 +15224,12 @@
       </c>
       <c r="C463" s="2" t="inlineStr">
         <is>
-          <t>A7878</t>
+          <t>A7288</t>
         </is>
       </c>
       <c r="D463" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731960</t>
+          <t>00019200000012731951</t>
         </is>
       </c>
       <c r="E463" s="2" t="inlineStr">
@@ -15256,12 +15256,12 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>A0974</t>
+          <t>A7878</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731978</t>
+          <t>00019200000012731960</t>
         </is>
       </c>
       <c r="E464" s="2" t="inlineStr">
@@ -15288,12 +15288,12 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>A8869</t>
+          <t>A0974</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731986</t>
+          <t>00019200000012731978</t>
         </is>
       </c>
       <c r="E465" s="2" t="inlineStr">
@@ -15320,12 +15320,12 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>A7491</t>
+          <t>A8869</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731994</t>
+          <t>00019200000012731986</t>
         </is>
       </c>
       <c r="E466" s="2" t="inlineStr">
@@ -15352,12 +15352,12 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>A6871</t>
+          <t>A7491</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732001</t>
+          <t>00019200000012731994</t>
         </is>
       </c>
       <c r="E467" s="2" t="inlineStr">
@@ -15384,12 +15384,12 @@
       </c>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>A1824</t>
+          <t>A6871</t>
         </is>
       </c>
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732010</t>
+          <t>00019200000012732001</t>
         </is>
       </c>
       <c r="E468" s="2" t="inlineStr">
@@ -15416,12 +15416,12 @@
       </c>
       <c r="C469" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A1824</t>
         </is>
       </c>
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732028</t>
+          <t>00019200000012732010</t>
         </is>
       </c>
       <c r="E469" s="2" t="inlineStr">
@@ -15448,12 +15448,12 @@
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>A9638</t>
+          <t>A9207</t>
         </is>
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732036</t>
+          <t>00019200000012732028</t>
         </is>
       </c>
       <c r="E470" s="2" t="inlineStr">
@@ -15480,12 +15480,12 @@
       </c>
       <c r="C471" s="2" t="inlineStr">
         <is>
-          <t>TA1173</t>
+          <t>A9638</t>
         </is>
       </c>
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732044</t>
+          <t>00019200000012732036</t>
         </is>
       </c>
       <c r="E471" s="2" t="inlineStr">
@@ -15512,12 +15512,12 @@
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>A9280</t>
+          <t>TA1173</t>
         </is>
       </c>
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732052</t>
+          <t>00019200000012732044</t>
         </is>
       </c>
       <c r="E472" s="2" t="inlineStr">
@@ -15544,12 +15544,12 @@
       </c>
       <c r="C473" s="2" t="inlineStr">
         <is>
-          <t>A6843</t>
+          <t>A9280</t>
         </is>
       </c>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732060</t>
+          <t>00019200000012732052</t>
         </is>
       </c>
       <c r="E473" s="2" t="inlineStr">
@@ -15576,12 +15576,12 @@
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>A8045</t>
+          <t>A6843</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732079</t>
+          <t>00019200000012732060</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr">
@@ -15608,12 +15608,12 @@
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A8045</t>
         </is>
       </c>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732087</t>
+          <t>00019200000012732079</t>
         </is>
       </c>
       <c r="E475" s="2" t="inlineStr">
@@ -15640,12 +15640,12 @@
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>A1989</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732095</t>
+          <t>00019200000012732087</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr">
@@ -15672,12 +15672,12 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>TA0654</t>
+          <t>A1989</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732109</t>
+          <t>00019200000012732095</t>
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr">
@@ -15704,12 +15704,12 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>A4447</t>
+          <t>TA0654</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732117</t>
+          <t>00019200000012732109</t>
         </is>
       </c>
       <c r="E478" s="2" t="inlineStr">
@@ -15736,12 +15736,12 @@
       </c>
       <c r="C479" s="2" t="inlineStr">
         <is>
-          <t>A8046</t>
+          <t>A4447</t>
         </is>
       </c>
       <c r="D479" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732125</t>
+          <t>00019200000012732117</t>
         </is>
       </c>
       <c r="E479" s="2" t="inlineStr">
@@ -15768,12 +15768,12 @@
       </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>A3920</t>
+          <t>A8046</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732133</t>
+          <t>00019200000012732125</t>
         </is>
       </c>
       <c r="E480" s="2" t="inlineStr">
@@ -15800,12 +15800,12 @@
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>A7425</t>
+          <t>A3920</t>
         </is>
       </c>
       <c r="D481" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732141</t>
+          <t>00019200000012732133</t>
         </is>
       </c>
       <c r="E481" s="2" t="inlineStr">
@@ -15832,12 +15832,12 @@
       </c>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>A3679</t>
+          <t>A7425</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732150</t>
+          <t>00019200000012732141</t>
         </is>
       </c>
       <c r="E482" s="2" t="inlineStr">
@@ -15864,12 +15864,12 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>A7985</t>
+          <t>A3679</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732168</t>
+          <t>00019200000012732150</t>
         </is>
       </c>
       <c r="E483" s="2" t="inlineStr">
@@ -15896,12 +15896,12 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>A6562</t>
+          <t>A7985</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732176</t>
+          <t>00019200000012732168</t>
         </is>
       </c>
       <c r="E484" s="2" t="inlineStr">
@@ -15928,12 +15928,12 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>A4360</t>
+          <t>A6562</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732184</t>
+          <t>00019200000012732176</t>
         </is>
       </c>
       <c r="E485" s="2" t="inlineStr">
@@ -15960,12 +15960,12 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>A9173</t>
+          <t>A4360</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732192</t>
+          <t>00019200000012732184</t>
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr">
@@ -15992,12 +15992,12 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>A2809</t>
+          <t>A9173</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732206</t>
+          <t>00019200000012732192</t>
         </is>
       </c>
       <c r="E487" s="2" t="inlineStr">
@@ -16024,12 +16024,12 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>TA0960</t>
+          <t>A2809</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732214</t>
+          <t>00019200000012732206</t>
         </is>
       </c>
       <c r="E488" s="2" t="inlineStr">
@@ -16056,12 +16056,12 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>TA0960</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732222</t>
+          <t>00019200000012732214</t>
         </is>
       </c>
       <c r="E489" s="2" t="inlineStr">
@@ -16088,12 +16088,12 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>A9307</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732230</t>
+          <t>00019200000012732222</t>
         </is>
       </c>
       <c r="E490" s="2" t="inlineStr">
@@ -16120,12 +16120,12 @@
       </c>
       <c r="C491" s="2" t="inlineStr">
         <is>
-          <t>A7068</t>
+          <t>A9307</t>
         </is>
       </c>
       <c r="D491" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732249</t>
+          <t>00019200000012732230</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr">
@@ -16152,12 +16152,12 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>A3376</t>
+          <t>A7068</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732257</t>
+          <t>00019200000012732249</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr">
@@ -16184,12 +16184,12 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>A3287</t>
+          <t>A3376</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732265</t>
+          <t>00019200000012732257</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr">
@@ -16216,12 +16216,12 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>A9200</t>
+          <t>A3287</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732273</t>
+          <t>00019200000012732265</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr">
@@ -16248,12 +16248,12 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>A5037</t>
+          <t>A9200</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732281</t>
+          <t>00019200000012732273</t>
         </is>
       </c>
       <c r="E495" s="2" t="inlineStr">
@@ -16280,12 +16280,12 @@
       </c>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>A9610</t>
+          <t>A5037</t>
         </is>
       </c>
       <c r="D496" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732290</t>
+          <t>00019200000012732281</t>
         </is>
       </c>
       <c r="E496" s="2" t="inlineStr">
@@ -16312,12 +16312,12 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>A1420</t>
+          <t>A9610</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
         <is>
-          <t>00019200000012857750</t>
+          <t>00019200000012732290</t>
         </is>
       </c>
       <c r="E497" s="2" t="inlineStr">
@@ -16334,7 +16334,7 @@
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>556224</t>
+          <t>556160</t>
         </is>
       </c>
       <c r="B498" s="2" t="inlineStr">
@@ -16344,29 +16344,29 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>A4220</t>
+          <t>A1420</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729043</t>
+          <t>00019200000012857750</t>
         </is>
       </c>
       <c r="E498" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 05:11</t>
+          <t>06/06/2026 11:33</t>
         </is>
       </c>
       <c r="F498" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 16:00</t>
+          <t>08/06/2026 11:46</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>556409</t>
+          <t>556224</t>
         </is>
       </c>
       <c r="B499" s="2" t="inlineStr">
@@ -16376,22 +16376,22 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>A8078</t>
+          <t>A4220</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723550</t>
+          <t>00019200000012729043</t>
         </is>
       </c>
       <c r="E499" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 06:40</t>
+          <t>11/06/2026 05:11</t>
         </is>
       </c>
       <c r="F499" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:18</t>
+          <t>12/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -16408,12 +16408,12 @@
       </c>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>A0401</t>
+          <t>A8078</t>
         </is>
       </c>
       <c r="D500" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723568</t>
+          <t>00019200000012723550</t>
         </is>
       </c>
       <c r="E500" s="2" t="inlineStr">
@@ -16440,12 +16440,12 @@
       </c>
       <c r="C501" s="2" t="inlineStr">
         <is>
-          <t>A8580</t>
+          <t>A0401</t>
         </is>
       </c>
       <c r="D501" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723592</t>
+          <t>00019200000012723568</t>
         </is>
       </c>
       <c r="E501" s="2" t="inlineStr">
@@ -16462,32 +16462,32 @@
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>555932</t>
+          <t>556409</t>
         </is>
       </c>
       <c r="B502" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>A4257</t>
+          <t>A8580</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721840</t>
+          <t>00019200000012723592</t>
         </is>
       </c>
       <c r="E502" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:18</t>
+          <t>10/06/2026 06:40</t>
         </is>
       </c>
       <c r="F502" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:33</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -16504,12 +16504,12 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>A9287</t>
+          <t>A4257</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723061</t>
+          <t>00019200000012721840</t>
         </is>
       </c>
       <c r="E503" s="2" t="inlineStr">
@@ -16526,7 +16526,7 @@
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>556161</t>
+          <t>555932</t>
         </is>
       </c>
       <c r="B504" s="2" t="inlineStr">
@@ -16536,22 +16536,22 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>A7008</t>
+          <t>A9287</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730491</t>
+          <t>00019200000012723061</t>
         </is>
       </c>
       <c r="E504" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:18</t>
         </is>
       </c>
       <c r="F504" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:51</t>
+          <t>03/06/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -16568,12 +16568,12 @@
       </c>
       <c r="C505" s="2" t="inlineStr">
         <is>
-          <t>A7785</t>
+          <t>A7008</t>
         </is>
       </c>
       <c r="D505" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730670</t>
+          <t>00019200000012730491</t>
         </is>
       </c>
       <c r="E505" s="2" t="inlineStr">
@@ -16600,12 +16600,12 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>A6386</t>
+          <t>A7785</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730688</t>
+          <t>00019200000012730670</t>
         </is>
       </c>
       <c r="E506" s="2" t="inlineStr">
@@ -16632,12 +16632,12 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>A8302</t>
+          <t>A6386</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730696</t>
+          <t>00019200000012730688</t>
         </is>
       </c>
       <c r="E507" s="2" t="inlineStr">
@@ -16664,12 +16664,12 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>A6870</t>
+          <t>A8302</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730700</t>
+          <t>00019200000012730696</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
@@ -16696,12 +16696,12 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>A8192</t>
+          <t>A6870</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731331</t>
+          <t>00019200000012730700</t>
         </is>
       </c>
       <c r="E509" s="2" t="inlineStr">
@@ -16728,12 +16728,12 @@
       </c>
       <c r="C510" s="2" t="inlineStr">
         <is>
-          <t>A1045</t>
+          <t>A8192</t>
         </is>
       </c>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731340</t>
+          <t>00019200000012731331</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr">
@@ -16760,12 +16760,12 @@
       </c>
       <c r="C511" s="2" t="inlineStr">
         <is>
-          <t>A3603</t>
+          <t>A1045</t>
         </is>
       </c>
       <c r="D511" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731358</t>
+          <t>00019200000012731340</t>
         </is>
       </c>
       <c r="E511" s="2" t="inlineStr">
@@ -16792,12 +16792,12 @@
       </c>
       <c r="C512" s="2" t="inlineStr">
         <is>
-          <t>A9427</t>
+          <t>A3603</t>
         </is>
       </c>
       <c r="D512" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731366</t>
+          <t>00019200000012731358</t>
         </is>
       </c>
       <c r="E512" s="2" t="inlineStr">
@@ -16824,12 +16824,12 @@
       </c>
       <c r="C513" s="2" t="inlineStr">
         <is>
-          <t>A4068</t>
+          <t>A9427</t>
         </is>
       </c>
       <c r="D513" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731374</t>
+          <t>00019200000012731366</t>
         </is>
       </c>
       <c r="E513" s="2" t="inlineStr">
@@ -16856,12 +16856,12 @@
       </c>
       <c r="C514" s="2" t="inlineStr">
         <is>
-          <t>A2753</t>
+          <t>A4068</t>
         </is>
       </c>
       <c r="D514" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731382</t>
+          <t>00019200000012731374</t>
         </is>
       </c>
       <c r="E514" s="2" t="inlineStr">
@@ -16888,12 +16888,12 @@
       </c>
       <c r="C515" s="2" t="inlineStr">
         <is>
-          <t>TA0353</t>
+          <t>A2753</t>
         </is>
       </c>
       <c r="D515" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731390</t>
+          <t>00019200000012731382</t>
         </is>
       </c>
       <c r="E515" s="2" t="inlineStr">
@@ -16920,12 +16920,12 @@
       </c>
       <c r="C516" s="2" t="inlineStr">
         <is>
-          <t>A7155</t>
+          <t>TA0353</t>
         </is>
       </c>
       <c r="D516" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731404</t>
+          <t>00019200000012731390</t>
         </is>
       </c>
       <c r="E516" s="2" t="inlineStr">
@@ -16952,12 +16952,12 @@
       </c>
       <c r="C517" s="2" t="inlineStr">
         <is>
-          <t>A6665</t>
+          <t>A7155</t>
         </is>
       </c>
       <c r="D517" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731412</t>
+          <t>00019200000012731404</t>
         </is>
       </c>
       <c r="E517" s="2" t="inlineStr">
@@ -16984,12 +16984,12 @@
       </c>
       <c r="C518" s="2" t="inlineStr">
         <is>
-          <t>TA0675</t>
+          <t>A6665</t>
         </is>
       </c>
       <c r="D518" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731420</t>
+          <t>00019200000012731412</t>
         </is>
       </c>
       <c r="E518" s="2" t="inlineStr">
@@ -17016,12 +17016,12 @@
       </c>
       <c r="C519" s="2" t="inlineStr">
         <is>
-          <t>A7142</t>
+          <t>TA0675</t>
         </is>
       </c>
       <c r="D519" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731439</t>
+          <t>00019200000012731420</t>
         </is>
       </c>
       <c r="E519" s="2" t="inlineStr">
@@ -17048,12 +17048,12 @@
       </c>
       <c r="C520" s="2" t="inlineStr">
         <is>
-          <t>TA0136</t>
+          <t>A7142</t>
         </is>
       </c>
       <c r="D520" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731447</t>
+          <t>00019200000012731439</t>
         </is>
       </c>
       <c r="E520" s="2" t="inlineStr">
@@ -17080,12 +17080,12 @@
       </c>
       <c r="C521" s="2" t="inlineStr">
         <is>
-          <t>TA0818</t>
+          <t>TA0136</t>
         </is>
       </c>
       <c r="D521" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731455</t>
+          <t>00019200000012731447</t>
         </is>
       </c>
       <c r="E521" s="2" t="inlineStr">
@@ -17112,12 +17112,12 @@
       </c>
       <c r="C522" s="2" t="inlineStr">
         <is>
-          <t>A6147</t>
+          <t>TA0818</t>
         </is>
       </c>
       <c r="D522" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731463</t>
+          <t>00019200000012731455</t>
         </is>
       </c>
       <c r="E522" s="2" t="inlineStr">
@@ -17144,12 +17144,12 @@
       </c>
       <c r="C523" s="2" t="inlineStr">
         <is>
-          <t>A4999</t>
+          <t>A6147</t>
         </is>
       </c>
       <c r="D523" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731471</t>
+          <t>00019200000012731463</t>
         </is>
       </c>
       <c r="E523" s="2" t="inlineStr">
@@ -17176,12 +17176,12 @@
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>A5847</t>
+          <t>A4999</t>
         </is>
       </c>
       <c r="D524" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731498</t>
+          <t>00019200000012731471</t>
         </is>
       </c>
       <c r="E524" s="2" t="inlineStr">
@@ -17208,12 +17208,12 @@
       </c>
       <c r="C525" s="2" t="inlineStr">
         <is>
-          <t>A2981</t>
+          <t>A5847</t>
         </is>
       </c>
       <c r="D525" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731501</t>
+          <t>00019200000012731498</t>
         </is>
       </c>
       <c r="E525" s="2" t="inlineStr">
@@ -17240,12 +17240,12 @@
       </c>
       <c r="C526" s="2" t="inlineStr">
         <is>
-          <t>A7462</t>
+          <t>A2981</t>
         </is>
       </c>
       <c r="D526" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731510</t>
+          <t>00019200000012731501</t>
         </is>
       </c>
       <c r="E526" s="2" t="inlineStr">
@@ -17272,12 +17272,12 @@
       </c>
       <c r="C527" s="2" t="inlineStr">
         <is>
-          <t>A4340</t>
+          <t>A7462</t>
         </is>
       </c>
       <c r="D527" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731528</t>
+          <t>00019200000012731510</t>
         </is>
       </c>
       <c r="E527" s="2" t="inlineStr">
@@ -17304,12 +17304,12 @@
       </c>
       <c r="C528" s="2" t="inlineStr">
         <is>
-          <t>A8938</t>
+          <t>A4340</t>
         </is>
       </c>
       <c r="D528" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731536</t>
+          <t>00019200000012731528</t>
         </is>
       </c>
       <c r="E528" s="2" t="inlineStr">
@@ -17326,7 +17326,7 @@
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>556300</t>
+          <t>556161</t>
         </is>
       </c>
       <c r="B529" s="2" t="inlineStr">
@@ -17336,54 +17336,54 @@
       </c>
       <c r="C529" s="2" t="inlineStr">
         <is>
-          <t>TA0506</t>
+          <t>A8938</t>
         </is>
       </c>
       <c r="D529" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728918</t>
+          <t>00019200000012731536</t>
         </is>
       </c>
       <c r="E529" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 10:36</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F529" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:54</t>
+          <t>08/06/2026 14:51</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>556300</t>
         </is>
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C530" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>TA0506</t>
         </is>
       </c>
       <c r="D530" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000012728918</t>
         </is>
       </c>
       <c r="E530" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>06/06/2026 10:36</t>
         </is>
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>08/06/2026 10:54</t>
         </is>
       </c>
     </row>
@@ -17400,12 +17400,12 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E531" s="2" t="inlineStr">
@@ -17432,12 +17432,12 @@
       </c>
       <c r="C532" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D532" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E532" s="2" t="inlineStr">
@@ -17454,39 +17454,39 @@
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B533" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C533" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D533" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E533" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F533" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B534" s="2" t="inlineStr">
@@ -17496,22 +17496,22 @@
       </c>
       <c r="C534" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D534" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E534" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F534" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -17528,12 +17528,12 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E535" s="2" t="inlineStr">
@@ -17560,12 +17560,12 @@
       </c>
       <c r="C536" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D536" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E536" s="2" t="inlineStr">
@@ -17592,12 +17592,12 @@
       </c>
       <c r="C537" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D537" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E537" s="2" t="inlineStr">
@@ -17624,12 +17624,12 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E538" s="2" t="inlineStr">
@@ -17656,12 +17656,12 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E539" s="2" t="inlineStr">
@@ -17688,12 +17688,12 @@
       </c>
       <c r="C540" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D540" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E540" s="2" t="inlineStr">
@@ -17720,12 +17720,12 @@
       </c>
       <c r="C541" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D541" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E541" s="2" t="inlineStr">
@@ -17752,12 +17752,12 @@
       </c>
       <c r="C542" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D542" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E542" s="2" t="inlineStr">
@@ -17784,12 +17784,12 @@
       </c>
       <c r="C543" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D543" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E543" s="2" t="inlineStr">
@@ -17816,12 +17816,12 @@
       </c>
       <c r="C544" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D544" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E544" s="2" t="inlineStr">
@@ -17848,12 +17848,12 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E545" s="2" t="inlineStr">
@@ -17880,12 +17880,12 @@
       </c>
       <c r="C546" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D546" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E546" s="2" t="inlineStr">
@@ -17912,12 +17912,12 @@
       </c>
       <c r="C547" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D547" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E547" s="2" t="inlineStr">
@@ -17944,12 +17944,12 @@
       </c>
       <c r="C548" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D548" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E548" s="2" t="inlineStr">
@@ -17966,7 +17966,7 @@
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B549" s="2" t="inlineStr">
@@ -17976,22 +17976,22 @@
       </c>
       <c r="C549" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D549" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E549" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F549" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -18008,12 +18008,12 @@
       </c>
       <c r="C550" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D550" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E550" s="2" t="inlineStr">
@@ -18040,12 +18040,12 @@
       </c>
       <c r="C551" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D551" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E551" s="2" t="inlineStr">
@@ -18072,12 +18072,12 @@
       </c>
       <c r="C552" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D552" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E552" s="2" t="inlineStr">
@@ -18104,27 +18104,59 @@
       </c>
       <c r="C553" s="2" t="inlineStr">
         <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
           <t>A8196</t>
         </is>
       </c>
-      <c r="D553" s="2" t="inlineStr">
+      <c r="D554" s="2" t="inlineStr">
         <is>
           <t>00019200000012728802</t>
         </is>
       </c>
-      <c r="E553" s="2" t="inlineStr">
+      <c r="E554" s="2" t="inlineStr">
         <is>
           <t>09/06/2026 02:06</t>
         </is>
       </c>
-      <c r="F553" s="2" t="inlineStr">
+      <c r="F554" s="2" t="inlineStr">
         <is>
           <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F553"/>
+  <autoFilter ref="A1:F554"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-15 14:35:04
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -815,7 +815,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>12/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>11/06/2026 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-16 14:53:05
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -1743,7 +1743,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>11/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>11/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:00</t>
+          <t>11/06/2026 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-16 17:23:05
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10727,7 +10727,7 @@
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:03</t>
         </is>
       </c>
     </row>
@@ -10759,7 +10759,7 @@
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:03</t>
         </is>
       </c>
     </row>
@@ -10791,7 +10791,7 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:03</t>
         </is>
       </c>
     </row>
@@ -10823,7 +10823,7 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:03</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -10951,7 +10951,7 @@
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -11015,7 +11015,7 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -11047,7 +11047,7 @@
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-16 17:53:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9575,7 +9575,7 @@
       </c>
       <c r="F286" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9607,7 +9607,7 @@
       </c>
       <c r="F287" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9639,7 +9639,7 @@
       </c>
       <c r="F288" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9671,7 +9671,7 @@
       </c>
       <c r="F289" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9703,7 +9703,7 @@
       </c>
       <c r="F290" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="F291" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
       </c>
       <c r="F292" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9799,7 +9799,7 @@
       </c>
       <c r="F293" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9831,7 +9831,7 @@
       </c>
       <c r="F294" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9863,7 +9863,7 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9895,7 +9895,7 @@
       </c>
       <c r="F296" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9927,7 +9927,7 @@
       </c>
       <c r="F297" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9959,7 +9959,7 @@
       </c>
       <c r="F298" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -9991,7 +9991,7 @@
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="F300" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10055,7 +10055,7 @@
       </c>
       <c r="F301" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10087,7 +10087,7 @@
       </c>
       <c r="F302" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10119,7 +10119,7 @@
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10183,7 +10183,7 @@
       </c>
       <c r="F305" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10215,7 +10215,7 @@
       </c>
       <c r="F306" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10247,7 +10247,7 @@
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10279,7 +10279,7 @@
       </c>
       <c r="F308" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -10343,7 +10343,7 @@
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 17:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-16 19:08:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -8551,7 +8551,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-16 19:23:07
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -2959,7 +2959,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 19:03</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 19:03</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16/06/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-18 00:09:47
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$638</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$639</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F638"/>
+  <dimension ref="A1:F639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12146,32 +12146,32 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>556173</t>
+          <t>558171</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>A5580</t>
+          <t>S0797</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714577</t>
+          <t>00019200000013210840</t>
         </is>
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 09:17</t>
+          <t>17/06/2026 23:50</t>
         </is>
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -12188,12 +12188,12 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>A4423</t>
+          <t>A5580</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714585</t>
+          <t>00019200000012714577</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
@@ -12210,39 +12210,39 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>555906</t>
+          <t>556173</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>TA1064</t>
+          <t>A4423</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>00019200000012718556</t>
+          <t>00019200000012714585</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:51</t>
+          <t>06/06/2026 09:17</t>
         </is>
       </c>
       <c r="F369" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 17:20</t>
+          <t>08/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>556105</t>
+          <t>555906</t>
         </is>
       </c>
       <c r="B370" s="2" t="inlineStr">
@@ -12252,29 +12252,29 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>A0431</t>
+          <t>TA1064</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>00019200000012717614</t>
+          <t>00019200000012718556</t>
         </is>
       </c>
       <c r="E370" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 22:37</t>
+          <t>07/06/2026 22:51</t>
         </is>
       </c>
       <c r="F370" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 10:30</t>
+          <t>09/06/2026 17:20</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>556187</t>
+          <t>556105</t>
         </is>
       </c>
       <c r="B371" s="2" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>A8822</t>
+          <t>A0431</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864242</t>
+          <t>00019200000012717614</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 21:57</t>
+          <t>08/06/2026 22:37</t>
         </is>
       </c>
       <c r="F371" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026 13:07</t>
+          <t>10/06/2026 10:30</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>556406</t>
+          <t>556187</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
@@ -12316,22 +12316,22 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>A4248</t>
+          <t>A8822</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704270</t>
+          <t>00019200000012864242</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026 04:45</t>
+          <t>02/06/2026 21:57</t>
         </is>
       </c>
       <c r="F372" s="2" t="inlineStr">
         <is>
-          <t>16/06/2026 17:03</t>
+          <t>04/06/2026 13:07</t>
         </is>
       </c>
     </row>
@@ -12348,12 +12348,12 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>TA0330</t>
+          <t>A4248</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704296</t>
+          <t>00019200000012704270</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
@@ -12380,12 +12380,12 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>A2496</t>
+          <t>TA0330</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704300</t>
+          <t>00019200000012704296</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr">
@@ -12412,12 +12412,12 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>A6046</t>
+          <t>A2496</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704326</t>
+          <t>00019200000012704300</t>
         </is>
       </c>
       <c r="E375" s="2" t="inlineStr">
@@ -12434,7 +12434,7 @@
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>556621</t>
+          <t>556406</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
@@ -12444,22 +12444,22 @@
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>A9300</t>
+          <t>A6046</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704202</t>
+          <t>00019200000012704326</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026 07:40</t>
+          <t>15/06/2026 04:45</t>
         </is>
       </c>
       <c r="F376" s="2" t="inlineStr">
         <is>
-          <t>16/06/2026 17:05</t>
+          <t>16/06/2026 17:03</t>
         </is>
       </c>
     </row>
@@ -12476,12 +12476,12 @@
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>A6669</t>
+          <t>A9300</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704210</t>
+          <t>00019200000012704202</t>
         </is>
       </c>
       <c r="E377" s="2" t="inlineStr">
@@ -12508,12 +12508,12 @@
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>A3590</t>
+          <t>A6669</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704229</t>
+          <t>00019200000012704210</t>
         </is>
       </c>
       <c r="E378" s="2" t="inlineStr">
@@ -12540,12 +12540,12 @@
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>A4299</t>
+          <t>A3590</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704245</t>
+          <t>00019200000012704229</t>
         </is>
       </c>
       <c r="E379" s="2" t="inlineStr">
@@ -12572,12 +12572,12 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>TA0874</t>
+          <t>A4299</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704350</t>
+          <t>00019200000012704245</t>
         </is>
       </c>
       <c r="E380" s="2" t="inlineStr">
@@ -12604,12 +12604,12 @@
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>A5531</t>
+          <t>TA0874</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704393</t>
+          <t>00019200000012704350</t>
         </is>
       </c>
       <c r="E381" s="2" t="inlineStr">
@@ -12636,12 +12636,12 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>A9708</t>
+          <t>A5531</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704407</t>
+          <t>00019200000012704393</t>
         </is>
       </c>
       <c r="E382" s="2" t="inlineStr">
@@ -12668,12 +12668,12 @@
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>TA0033</t>
+          <t>A9708</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>00019200000012704415</t>
+          <t>00019200000012704407</t>
         </is>
       </c>
       <c r="E383" s="2" t="inlineStr">
@@ -12690,32 +12690,32 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>556113</t>
+          <t>556621</t>
         </is>
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>A9365</t>
+          <t>TA0033</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714593</t>
+          <t>00019200000012704415</t>
         </is>
       </c>
       <c r="E384" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:53</t>
+          <t>15/06/2026 07:40</t>
         </is>
       </c>
       <c r="F384" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 19:47</t>
+          <t>16/06/2026 17:05</t>
         </is>
       </c>
     </row>
@@ -12732,12 +12732,12 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>A7132</t>
+          <t>A9365</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714607</t>
+          <t>00019200000012714593</t>
         </is>
       </c>
       <c r="E385" s="2" t="inlineStr">
@@ -12764,12 +12764,12 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>A6834</t>
+          <t>A7132</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714615</t>
+          <t>00019200000012714607</t>
         </is>
       </c>
       <c r="E386" s="2" t="inlineStr">
@@ -12796,12 +12796,12 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>A8249</t>
+          <t>A6834</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714623</t>
+          <t>00019200000012714615</t>
         </is>
       </c>
       <c r="E387" s="2" t="inlineStr">
@@ -12828,12 +12828,12 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>A8816</t>
+          <t>A8249</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714640</t>
+          <t>00019200000012714623</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
@@ -12850,7 +12850,7 @@
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>556339</t>
+          <t>556113</t>
         </is>
       </c>
       <c r="B389" s="2" t="inlineStr">
@@ -12860,29 +12860,29 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>A7748</t>
+          <t>A8816</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729124</t>
+          <t>00019200000012714640</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 03:51</t>
+          <t>08/06/2026 10:53</t>
         </is>
       </c>
       <c r="F389" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 17:19</t>
+          <t>11/06/2026 19:47</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>556549</t>
+          <t>556339</t>
         </is>
       </c>
       <c r="B390" s="2" t="inlineStr">
@@ -12892,61 +12892,61 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>A7654</t>
+          <t>A7748</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730505</t>
+          <t>00019200000012729124</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:31</t>
+          <t>09/06/2026 03:51</t>
         </is>
       </c>
       <c r="F390" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 17:00</t>
+          <t>10/06/2026 17:19</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>20260717</t>
+          <t>556549</t>
         </is>
       </c>
       <c r="B391" s="2" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>A5970</t>
+          <t>A7654</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721034</t>
+          <t>00019200000012730505</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 01:14</t>
+          <t>08/06/2026 05:31</t>
         </is>
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 13:12</t>
+          <t>09/06/2026 17:00</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>556743</t>
+          <t>20260717</t>
         </is>
       </c>
       <c r="B392" s="2" t="inlineStr">
@@ -12956,54 +12956,54 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>A7321</t>
+          <t>A5970</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723487</t>
+          <t>00019200000012721034</t>
         </is>
       </c>
       <c r="E392" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026 22:50</t>
+          <t>02/06/2026 01:14</t>
         </is>
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:50</t>
+          <t>03/06/2026 13:12</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>556083</t>
+          <t>556743</t>
         </is>
       </c>
       <c r="B393" s="2" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>A5844</t>
+          <t>A7321</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721867</t>
+          <t>00019200000012723487</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:05</t>
+          <t>07/06/2026 22:50</t>
         </is>
       </c>
       <c r="F393" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 17:29</t>
+          <t>09/06/2026 10:50</t>
         </is>
       </c>
     </row>
@@ -13020,12 +13020,12 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>A4723</t>
+          <t>A5844</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721891</t>
+          <t>00019200000012721867</t>
         </is>
       </c>
       <c r="E394" s="2" t="inlineStr">
@@ -13042,7 +13042,7 @@
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>556294</t>
+          <t>556083</t>
         </is>
       </c>
       <c r="B395" s="2" t="inlineStr">
@@ -13052,22 +13052,22 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>A3519</t>
+          <t>A4723</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714704</t>
+          <t>00019200000012721891</t>
         </is>
       </c>
       <c r="E395" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026 13:37</t>
+          <t>01/06/2026 22:05</t>
         </is>
       </c>
       <c r="F395" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 16:38</t>
+          <t>03/06/2026 17:29</t>
         </is>
       </c>
     </row>
@@ -13084,12 +13084,12 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>A9135</t>
+          <t>A3519</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714712</t>
+          <t>00019200000012714704</t>
         </is>
       </c>
       <c r="E396" s="2" t="inlineStr">
@@ -13116,12 +13116,12 @@
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>TA0487</t>
+          <t>A9135</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714720</t>
+          <t>00019200000012714712</t>
         </is>
       </c>
       <c r="E397" s="2" t="inlineStr">
@@ -13148,12 +13148,12 @@
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>TA1114</t>
+          <t>TA0487</t>
         </is>
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714739</t>
+          <t>00019200000012714720</t>
         </is>
       </c>
       <c r="E398" s="2" t="inlineStr">
@@ -13180,12 +13180,12 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>A8445</t>
+          <t>TA1114</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714747</t>
+          <t>00019200000012714739</t>
         </is>
       </c>
       <c r="E399" s="2" t="inlineStr">
@@ -13212,12 +13212,12 @@
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>A6194</t>
+          <t>A8445</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714763</t>
+          <t>00019200000012714747</t>
         </is>
       </c>
       <c r="E400" s="2" t="inlineStr">
@@ -13244,12 +13244,12 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>A9186</t>
+          <t>A6194</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714771</t>
+          <t>00019200000012714763</t>
         </is>
       </c>
       <c r="E401" s="2" t="inlineStr">
@@ -13276,12 +13276,12 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>A8034</t>
+          <t>A9186</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714780</t>
+          <t>00019200000012714771</t>
         </is>
       </c>
       <c r="E402" s="2" t="inlineStr">
@@ -13308,12 +13308,12 @@
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>A0774</t>
+          <t>A8034</t>
         </is>
       </c>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714798</t>
+          <t>00019200000012714780</t>
         </is>
       </c>
       <c r="E403" s="2" t="inlineStr">
@@ -13340,12 +13340,12 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>A8373</t>
+          <t>A0774</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714801</t>
+          <t>00019200000012714798</t>
         </is>
       </c>
       <c r="E404" s="2" t="inlineStr">
@@ -13372,12 +13372,12 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>A8792</t>
+          <t>A8373</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714810</t>
+          <t>00019200000012714801</t>
         </is>
       </c>
       <c r="E405" s="2" t="inlineStr">
@@ -13404,12 +13404,12 @@
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>A0162</t>
+          <t>A8792</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>00019200000012714828</t>
+          <t>00019200000012714810</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr">
@@ -13426,7 +13426,7 @@
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>556923</t>
+          <t>556294</t>
         </is>
       </c>
       <c r="B407" s="2" t="inlineStr">
@@ -13436,61 +13436,61 @@
       </c>
       <c r="C407" s="2" t="inlineStr">
         <is>
-          <t>TA0216</t>
+          <t>A0162</t>
         </is>
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>00019200000012656143</t>
+          <t>00019200000012714828</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026 06:58</t>
+          <t>02/06/2026 13:37</t>
         </is>
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>16/06/2026 14:00</t>
+          <t>03/06/2026 16:38</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>555911</t>
+          <t>556923</t>
         </is>
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>A4881</t>
+          <t>TA0216</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715298</t>
+          <t>00019200000012656143</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:02</t>
+          <t>15/06/2026 06:58</t>
         </is>
       </c>
       <c r="F408" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>16/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>556157</t>
+          <t>555911</t>
         </is>
       </c>
       <c r="B409" s="2" t="inlineStr">
@@ -13500,12 +13500,12 @@
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
-          <t>TA0188</t>
+          <t>A4881</t>
         </is>
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730203</t>
+          <t>00019200000012715298</t>
         </is>
       </c>
       <c r="E409" s="2" t="inlineStr">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="F409" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:00</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -13532,12 +13532,12 @@
       </c>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>TA0670</t>
+          <t>TA0188</t>
         </is>
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730211</t>
+          <t>00019200000012730203</t>
         </is>
       </c>
       <c r="E410" s="2" t="inlineStr">
@@ -13564,12 +13564,12 @@
       </c>
       <c r="C411" s="2" t="inlineStr">
         <is>
-          <t>A3810</t>
+          <t>TA0670</t>
         </is>
       </c>
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730220</t>
+          <t>00019200000012730211</t>
         </is>
       </c>
       <c r="E411" s="2" t="inlineStr">
@@ -13596,12 +13596,12 @@
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>A0800</t>
+          <t>A3810</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730238</t>
+          <t>00019200000012730220</t>
         </is>
       </c>
       <c r="E412" s="2" t="inlineStr">
@@ -13628,12 +13628,12 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>A5751</t>
+          <t>A0800</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730246</t>
+          <t>00019200000012730238</t>
         </is>
       </c>
       <c r="E413" s="2" t="inlineStr">
@@ -13660,12 +13660,12 @@
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>A3830</t>
+          <t>A5751</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730254</t>
+          <t>00019200000012730246</t>
         </is>
       </c>
       <c r="E414" s="2" t="inlineStr">
@@ -13692,12 +13692,12 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>A2419</t>
+          <t>A3830</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730262</t>
+          <t>00019200000012730254</t>
         </is>
       </c>
       <c r="E415" s="2" t="inlineStr">
@@ -13724,12 +13724,12 @@
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>A7535</t>
+          <t>A2419</t>
         </is>
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730270</t>
+          <t>00019200000012730262</t>
         </is>
       </c>
       <c r="E416" s="2" t="inlineStr">
@@ -13756,12 +13756,12 @@
       </c>
       <c r="C417" s="2" t="inlineStr">
         <is>
-          <t>A5563</t>
+          <t>A7535</t>
         </is>
       </c>
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730289</t>
+          <t>00019200000012730270</t>
         </is>
       </c>
       <c r="E417" s="2" t="inlineStr">
@@ -13788,12 +13788,12 @@
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>A9066</t>
+          <t>A5563</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730297</t>
+          <t>00019200000012730289</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
@@ -13820,12 +13820,12 @@
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>A5828</t>
+          <t>A9066</t>
         </is>
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730300</t>
+          <t>00019200000012730297</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
@@ -13852,12 +13852,12 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>A4055</t>
+          <t>A5828</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730319</t>
+          <t>00019200000012730300</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
@@ -13884,12 +13884,12 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>A0130</t>
+          <t>A4055</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730327</t>
+          <t>00019200000012730319</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
@@ -13916,12 +13916,12 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>A7797</t>
+          <t>A0130</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730335</t>
+          <t>00019200000012730327</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
@@ -13948,12 +13948,12 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>A9654</t>
+          <t>A7797</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730343</t>
+          <t>00019200000012730335</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
@@ -13980,12 +13980,12 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>A7482</t>
+          <t>A9654</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730351</t>
+          <t>00019200000012730343</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr">
@@ -14012,12 +14012,12 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>A7723</t>
+          <t>A7482</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730360</t>
+          <t>00019200000012730351</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
@@ -14044,12 +14044,12 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>A7997</t>
+          <t>A7723</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730378</t>
+          <t>00019200000012730360</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
@@ -14066,7 +14066,7 @@
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>556258</t>
+          <t>556157</t>
         </is>
       </c>
       <c r="B427" s="2" t="inlineStr">
@@ -14076,17 +14076,17 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>A6961</t>
+          <t>A7997</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729159</t>
+          <t>00019200000012730378</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>06/06/2026 05:02</t>
         </is>
       </c>
       <c r="F427" s="2" t="inlineStr">
@@ -14098,22 +14098,22 @@
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>556158</t>
+          <t>556258</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>A8351</t>
+          <t>A6961</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715344</t>
+          <t>00019200000012729159</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="F428" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 10:00</t>
+          <t>09/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -14140,12 +14140,12 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>A6522</t>
+          <t>A8351</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715352</t>
+          <t>00019200000012715344</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
@@ -14172,12 +14172,12 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>A7263</t>
+          <t>A6522</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715360</t>
+          <t>00019200000012715352</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
@@ -14204,12 +14204,12 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>A9019</t>
+          <t>A7263</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715379</t>
+          <t>00019200000012715360</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
@@ -14236,12 +14236,12 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>A4823</t>
+          <t>A9019</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715387</t>
+          <t>00019200000012715379</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
@@ -14268,12 +14268,12 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>A5775</t>
+          <t>A4823</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715395</t>
+          <t>00019200000012715387</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
@@ -14300,12 +14300,12 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>A6931</t>
+          <t>A5775</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>00019200000012715409</t>
+          <t>00019200000012715395</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
@@ -14322,32 +14322,32 @@
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>556159</t>
+          <t>556158</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>TA1119</t>
+          <t>A6931</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753440</t>
+          <t>00019200000012715409</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 09:08</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F435" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 13:30</t>
+          <t>09/06/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -14364,12 +14364,12 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>A6893</t>
+          <t>TA1119</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753459</t>
+          <t>00019200000012753440</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
@@ -14396,12 +14396,12 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>A8127</t>
+          <t>A6893</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753467</t>
+          <t>00019200000012753459</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
@@ -14428,12 +14428,12 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>A6189</t>
+          <t>A8127</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753475</t>
+          <t>00019200000012753467</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
@@ -14460,12 +14460,12 @@
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>TA0776</t>
+          <t>A6189</t>
         </is>
       </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753483</t>
+          <t>00019200000012753475</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
@@ -14492,12 +14492,12 @@
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>A8534</t>
+          <t>TA0776</t>
         </is>
       </c>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753491</t>
+          <t>00019200000012753483</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr">
@@ -14524,12 +14524,12 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>A7575</t>
+          <t>A8534</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753505</t>
+          <t>00019200000012753491</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
@@ -14556,12 +14556,12 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>A0609</t>
+          <t>A7575</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753513</t>
+          <t>00019200000012753505</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
@@ -14588,12 +14588,12 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>A9499</t>
+          <t>A0609</t>
         </is>
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753521</t>
+          <t>00019200000012753513</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr">
@@ -14620,12 +14620,12 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>A6581</t>
+          <t>A9499</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753530</t>
+          <t>00019200000012753521</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
@@ -14652,12 +14652,12 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>A8536</t>
+          <t>A6581</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753548</t>
+          <t>00019200000012753530</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
@@ -14684,12 +14684,12 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>A9316</t>
+          <t>A8536</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753556</t>
+          <t>00019200000012753548</t>
         </is>
       </c>
       <c r="E446" s="2" t="inlineStr">
@@ -14716,12 +14716,12 @@
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>TA0880</t>
+          <t>A9316</t>
         </is>
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753564</t>
+          <t>00019200000012753556</t>
         </is>
       </c>
       <c r="E447" s="2" t="inlineStr">
@@ -14748,12 +14748,12 @@
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>A1933</t>
+          <t>TA0880</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753572</t>
+          <t>00019200000012753564</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
@@ -14780,12 +14780,12 @@
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>A0504</t>
+          <t>A1933</t>
         </is>
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753882</t>
+          <t>00019200000012753572</t>
         </is>
       </c>
       <c r="E449" s="2" t="inlineStr">
@@ -14812,12 +14812,12 @@
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>TA0704</t>
+          <t>A0504</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753890</t>
+          <t>00019200000012753882</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
@@ -14844,12 +14844,12 @@
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>A8967</t>
+          <t>TA0704</t>
         </is>
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753904</t>
+          <t>00019200000012753890</t>
         </is>
       </c>
       <c r="E451" s="2" t="inlineStr">
@@ -14876,12 +14876,12 @@
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>A4337</t>
+          <t>A8967</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753912</t>
+          <t>00019200000012753904</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
@@ -14908,12 +14908,12 @@
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>A5175</t>
+          <t>A4337</t>
         </is>
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753920</t>
+          <t>00019200000012753912</t>
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr">
@@ -14940,12 +14940,12 @@
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>TA0974</t>
+          <t>A5175</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753939</t>
+          <t>00019200000012753920</t>
         </is>
       </c>
       <c r="E454" s="2" t="inlineStr">
@@ -14972,12 +14972,12 @@
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>A6700</t>
+          <t>TA0974</t>
         </is>
       </c>
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753947</t>
+          <t>00019200000012753939</t>
         </is>
       </c>
       <c r="E455" s="2" t="inlineStr">
@@ -15004,12 +15004,12 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>A8361</t>
+          <t>A6700</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753955</t>
+          <t>00019200000012753947</t>
         </is>
       </c>
       <c r="E456" s="2" t="inlineStr">
@@ -15036,12 +15036,12 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>A3121</t>
+          <t>A8361</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753963</t>
+          <t>00019200000012753955</t>
         </is>
       </c>
       <c r="E457" s="2" t="inlineStr">
@@ -15068,12 +15068,12 @@
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>A8154</t>
+          <t>A3121</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753971</t>
+          <t>00019200000012753963</t>
         </is>
       </c>
       <c r="E458" s="2" t="inlineStr">
@@ -15100,12 +15100,12 @@
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>TA0597</t>
+          <t>A8154</t>
         </is>
       </c>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753980</t>
+          <t>00019200000012753971</t>
         </is>
       </c>
       <c r="E459" s="2" t="inlineStr">
@@ -15132,12 +15132,12 @@
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>A6883</t>
+          <t>TA0597</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>00019200000012753998</t>
+          <t>00019200000012753980</t>
         </is>
       </c>
       <c r="E460" s="2" t="inlineStr">
@@ -15164,12 +15164,12 @@
       </c>
       <c r="C461" s="2" t="inlineStr">
         <is>
-          <t>A9704</t>
+          <t>A6883</t>
         </is>
       </c>
       <c r="D461" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754005</t>
+          <t>00019200000012753998</t>
         </is>
       </c>
       <c r="E461" s="2" t="inlineStr">
@@ -15196,12 +15196,12 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>A9302</t>
+          <t>A9704</t>
         </is>
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754013</t>
+          <t>00019200000012754005</t>
         </is>
       </c>
       <c r="E462" s="2" t="inlineStr">
@@ -15228,12 +15228,12 @@
       </c>
       <c r="C463" s="2" t="inlineStr">
         <is>
-          <t>A0119</t>
+          <t>A9302</t>
         </is>
       </c>
       <c r="D463" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754021</t>
+          <t>00019200000012754013</t>
         </is>
       </c>
       <c r="E463" s="2" t="inlineStr">
@@ -15260,12 +15260,12 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>A9040</t>
+          <t>A0119</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754048</t>
+          <t>00019200000012754021</t>
         </is>
       </c>
       <c r="E464" s="2" t="inlineStr">
@@ -15292,12 +15292,12 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>A7876</t>
+          <t>A9040</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754056</t>
+          <t>00019200000012754048</t>
         </is>
       </c>
       <c r="E465" s="2" t="inlineStr">
@@ -15324,12 +15324,12 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>A8919</t>
+          <t>A7876</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754064</t>
+          <t>00019200000012754056</t>
         </is>
       </c>
       <c r="E466" s="2" t="inlineStr">
@@ -15356,12 +15356,12 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>A6393</t>
+          <t>A8919</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754072</t>
+          <t>00019200000012754064</t>
         </is>
       </c>
       <c r="E467" s="2" t="inlineStr">
@@ -15388,12 +15388,12 @@
       </c>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>A4317</t>
+          <t>A6393</t>
         </is>
       </c>
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754080</t>
+          <t>00019200000012754072</t>
         </is>
       </c>
       <c r="E468" s="2" t="inlineStr">
@@ -15420,12 +15420,12 @@
       </c>
       <c r="C469" s="2" t="inlineStr">
         <is>
-          <t>A8657</t>
+          <t>A4317</t>
         </is>
       </c>
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754099</t>
+          <t>00019200000012754080</t>
         </is>
       </c>
       <c r="E469" s="2" t="inlineStr">
@@ -15452,12 +15452,12 @@
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>A8940</t>
+          <t>A8657</t>
         </is>
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754102</t>
+          <t>00019200000012754099</t>
         </is>
       </c>
       <c r="E470" s="2" t="inlineStr">
@@ -15484,12 +15484,12 @@
       </c>
       <c r="C471" s="2" t="inlineStr">
         <is>
-          <t>A6261</t>
+          <t>A8940</t>
         </is>
       </c>
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754110</t>
+          <t>00019200000012754102</t>
         </is>
       </c>
       <c r="E471" s="2" t="inlineStr">
@@ -15516,12 +15516,12 @@
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>A5569</t>
+          <t>A6261</t>
         </is>
       </c>
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754129</t>
+          <t>00019200000012754110</t>
         </is>
       </c>
       <c r="E472" s="2" t="inlineStr">
@@ -15548,12 +15548,12 @@
       </c>
       <c r="C473" s="2" t="inlineStr">
         <is>
-          <t>A8748</t>
+          <t>A5569</t>
         </is>
       </c>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754137</t>
+          <t>00019200000012754129</t>
         </is>
       </c>
       <c r="E473" s="2" t="inlineStr">
@@ -15580,12 +15580,12 @@
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>A9213</t>
+          <t>A8748</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754145</t>
+          <t>00019200000012754137</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr">
@@ -15612,12 +15612,12 @@
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>TA0226</t>
+          <t>A9213</t>
         </is>
       </c>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754153</t>
+          <t>00019200000012754145</t>
         </is>
       </c>
       <c r="E475" s="2" t="inlineStr">
@@ -15644,12 +15644,12 @@
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>A8485</t>
+          <t>TA0226</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754161</t>
+          <t>00019200000012754153</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr">
@@ -15676,12 +15676,12 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>A8095</t>
+          <t>A8485</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754170</t>
+          <t>00019200000012754161</t>
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr">
@@ -15708,12 +15708,12 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>A9152</t>
+          <t>A8095</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754188</t>
+          <t>00019200000012754170</t>
         </is>
       </c>
       <c r="E478" s="2" t="inlineStr">
@@ -15740,12 +15740,12 @@
       </c>
       <c r="C479" s="2" t="inlineStr">
         <is>
-          <t>A7849</t>
+          <t>A9152</t>
         </is>
       </c>
       <c r="D479" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754196</t>
+          <t>00019200000012754188</t>
         </is>
       </c>
       <c r="E479" s="2" t="inlineStr">
@@ -15772,12 +15772,12 @@
       </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>A6854</t>
+          <t>A7849</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754200</t>
+          <t>00019200000012754196</t>
         </is>
       </c>
       <c r="E480" s="2" t="inlineStr">
@@ -15804,12 +15804,12 @@
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>A8670</t>
+          <t>A6854</t>
         </is>
       </c>
       <c r="D481" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754218</t>
+          <t>00019200000012754200</t>
         </is>
       </c>
       <c r="E481" s="2" t="inlineStr">
@@ -15836,12 +15836,12 @@
       </c>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>A8352</t>
+          <t>A8670</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754226</t>
+          <t>00019200000012754218</t>
         </is>
       </c>
       <c r="E482" s="2" t="inlineStr">
@@ -15868,12 +15868,12 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>A6584</t>
+          <t>A8352</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754234</t>
+          <t>00019200000012754226</t>
         </is>
       </c>
       <c r="E483" s="2" t="inlineStr">
@@ -15900,12 +15900,12 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>A5394</t>
+          <t>A6584</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754242</t>
+          <t>00019200000012754234</t>
         </is>
       </c>
       <c r="E484" s="2" t="inlineStr">
@@ -15932,12 +15932,12 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>A9258</t>
+          <t>A5394</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754250</t>
+          <t>00019200000012754242</t>
         </is>
       </c>
       <c r="E485" s="2" t="inlineStr">
@@ -15964,12 +15964,12 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>A2475</t>
+          <t>A9258</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754269</t>
+          <t>00019200000012754250</t>
         </is>
       </c>
       <c r="E486" s="2" t="inlineStr">
@@ -15996,12 +15996,12 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>A8952</t>
+          <t>A2475</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754277</t>
+          <t>00019200000012754269</t>
         </is>
       </c>
       <c r="E487" s="2" t="inlineStr">
@@ -16028,12 +16028,12 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>A6781</t>
+          <t>A8952</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754285</t>
+          <t>00019200000012754277</t>
         </is>
       </c>
       <c r="E488" s="2" t="inlineStr">
@@ -16060,12 +16060,12 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>A8379</t>
+          <t>A6781</t>
         </is>
       </c>
       <c r="D489" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754293</t>
+          <t>00019200000012754285</t>
         </is>
       </c>
       <c r="E489" s="2" t="inlineStr">
@@ -16092,12 +16092,12 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>A8243</t>
+          <t>A8379</t>
         </is>
       </c>
       <c r="D490" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754307</t>
+          <t>00019200000012754293</t>
         </is>
       </c>
       <c r="E490" s="2" t="inlineStr">
@@ -16124,12 +16124,12 @@
       </c>
       <c r="C491" s="2" t="inlineStr">
         <is>
-          <t>A7097</t>
+          <t>A8243</t>
         </is>
       </c>
       <c r="D491" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754315</t>
+          <t>00019200000012754307</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr">
@@ -16156,12 +16156,12 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>TA0235</t>
+          <t>A7097</t>
         </is>
       </c>
       <c r="D492" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754323</t>
+          <t>00019200000012754315</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr">
@@ -16188,12 +16188,12 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>A8222</t>
+          <t>TA0235</t>
         </is>
       </c>
       <c r="D493" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754331</t>
+          <t>00019200000012754323</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr">
@@ -16220,12 +16220,12 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>A1510</t>
+          <t>A8222</t>
         </is>
       </c>
       <c r="D494" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754340</t>
+          <t>00019200000012754331</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>A0773</t>
+          <t>A1510</t>
         </is>
       </c>
       <c r="D495" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754358</t>
+          <t>00019200000012754340</t>
         </is>
       </c>
       <c r="E495" s="2" t="inlineStr">
@@ -16284,12 +16284,12 @@
       </c>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>A8448</t>
+          <t>A0773</t>
         </is>
       </c>
       <c r="D496" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754366</t>
+          <t>00019200000012754358</t>
         </is>
       </c>
       <c r="E496" s="2" t="inlineStr">
@@ -16316,12 +16316,12 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>A7767</t>
+          <t>A8448</t>
         </is>
       </c>
       <c r="D497" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754374</t>
+          <t>00019200000012754366</t>
         </is>
       </c>
       <c r="E497" s="2" t="inlineStr">
@@ -16348,12 +16348,12 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>A8254</t>
+          <t>A7767</t>
         </is>
       </c>
       <c r="D498" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754382</t>
+          <t>00019200000012754374</t>
         </is>
       </c>
       <c r="E498" s="2" t="inlineStr">
@@ -16380,12 +16380,12 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>A9361</t>
+          <t>A8254</t>
         </is>
       </c>
       <c r="D499" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754390</t>
+          <t>00019200000012754382</t>
         </is>
       </c>
       <c r="E499" s="2" t="inlineStr">
@@ -16412,12 +16412,12 @@
       </c>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>A5087</t>
+          <t>A9361</t>
         </is>
       </c>
       <c r="D500" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754404</t>
+          <t>00019200000012754390</t>
         </is>
       </c>
       <c r="E500" s="2" t="inlineStr">
@@ -16444,12 +16444,12 @@
       </c>
       <c r="C501" s="2" t="inlineStr">
         <is>
-          <t>A0387</t>
+          <t>A5087</t>
         </is>
       </c>
       <c r="D501" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754412</t>
+          <t>00019200000012754404</t>
         </is>
       </c>
       <c r="E501" s="2" t="inlineStr">
@@ -16476,12 +16476,12 @@
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>A6996</t>
+          <t>A0387</t>
         </is>
       </c>
       <c r="D502" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754420</t>
+          <t>00019200000012754412</t>
         </is>
       </c>
       <c r="E502" s="2" t="inlineStr">
@@ -16508,12 +16508,12 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>A7094</t>
+          <t>A6996</t>
         </is>
       </c>
       <c r="D503" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754439</t>
+          <t>00019200000012754420</t>
         </is>
       </c>
       <c r="E503" s="2" t="inlineStr">
@@ -16540,12 +16540,12 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>A7194</t>
+          <t>A7094</t>
         </is>
       </c>
       <c r="D504" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754447</t>
+          <t>00019200000012754439</t>
         </is>
       </c>
       <c r="E504" s="2" t="inlineStr">
@@ -16572,12 +16572,12 @@
       </c>
       <c r="C505" s="2" t="inlineStr">
         <is>
-          <t>A6941</t>
+          <t>A7194</t>
         </is>
       </c>
       <c r="D505" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754455</t>
+          <t>00019200000012754447</t>
         </is>
       </c>
       <c r="E505" s="2" t="inlineStr">
@@ -16604,12 +16604,12 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>A6571</t>
+          <t>A6941</t>
         </is>
       </c>
       <c r="D506" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754463</t>
+          <t>00019200000012754455</t>
         </is>
       </c>
       <c r="E506" s="2" t="inlineStr">
@@ -16636,12 +16636,12 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>A5633</t>
+          <t>A6571</t>
         </is>
       </c>
       <c r="D507" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754471</t>
+          <t>00019200000012754463</t>
         </is>
       </c>
       <c r="E507" s="2" t="inlineStr">
@@ -16668,12 +16668,12 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>A9483</t>
+          <t>A5633</t>
         </is>
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754480</t>
+          <t>00019200000012754471</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
@@ -16700,12 +16700,12 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>A9277</t>
+          <t>A9483</t>
         </is>
       </c>
       <c r="D509" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754498</t>
+          <t>00019200000012754480</t>
         </is>
       </c>
       <c r="E509" s="2" t="inlineStr">
@@ -16732,12 +16732,12 @@
       </c>
       <c r="C510" s="2" t="inlineStr">
         <is>
-          <t>A6305</t>
+          <t>A9277</t>
         </is>
       </c>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754501</t>
+          <t>00019200000012754498</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr">
@@ -16764,12 +16764,12 @@
       </c>
       <c r="C511" s="2" t="inlineStr">
         <is>
-          <t>A0745</t>
+          <t>A6305</t>
         </is>
       </c>
       <c r="D511" s="2" t="inlineStr">
         <is>
-          <t>00019200000012754510</t>
+          <t>00019200000012754501</t>
         </is>
       </c>
       <c r="E511" s="2" t="inlineStr">
@@ -16796,12 +16796,12 @@
       </c>
       <c r="C512" s="2" t="inlineStr">
         <is>
-          <t>A7451</t>
+          <t>A0745</t>
         </is>
       </c>
       <c r="D512" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755958</t>
+          <t>00019200000012754510</t>
         </is>
       </c>
       <c r="E512" s="2" t="inlineStr">
@@ -16828,12 +16828,12 @@
       </c>
       <c r="C513" s="2" t="inlineStr">
         <is>
-          <t>A9324</t>
+          <t>A7451</t>
         </is>
       </c>
       <c r="D513" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755966</t>
+          <t>00019200000012755958</t>
         </is>
       </c>
       <c r="E513" s="2" t="inlineStr">
@@ -16860,12 +16860,12 @@
       </c>
       <c r="C514" s="2" t="inlineStr">
         <is>
-          <t>A8491</t>
+          <t>A9324</t>
         </is>
       </c>
       <c r="D514" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755974</t>
+          <t>00019200000012755966</t>
         </is>
       </c>
       <c r="E514" s="2" t="inlineStr">
@@ -16892,12 +16892,12 @@
       </c>
       <c r="C515" s="2" t="inlineStr">
         <is>
-          <t>A9490</t>
+          <t>A8491</t>
         </is>
       </c>
       <c r="D515" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755982</t>
+          <t>00019200000012755974</t>
         </is>
       </c>
       <c r="E515" s="2" t="inlineStr">
@@ -16924,12 +16924,12 @@
       </c>
       <c r="C516" s="2" t="inlineStr">
         <is>
-          <t>A9202</t>
+          <t>A9490</t>
         </is>
       </c>
       <c r="D516" s="2" t="inlineStr">
         <is>
-          <t>00019200000012755990</t>
+          <t>00019200000012755982</t>
         </is>
       </c>
       <c r="E516" s="2" t="inlineStr">
@@ -16956,12 +16956,12 @@
       </c>
       <c r="C517" s="2" t="inlineStr">
         <is>
-          <t>A5679</t>
+          <t>A9202</t>
         </is>
       </c>
       <c r="D517" s="2" t="inlineStr">
         <is>
-          <t>00019200000012756008</t>
+          <t>00019200000012755990</t>
         </is>
       </c>
       <c r="E517" s="2" t="inlineStr">
@@ -16978,7 +16978,7 @@
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>556744</t>
+          <t>556159</t>
         </is>
       </c>
       <c r="B518" s="2" t="inlineStr">
@@ -16988,54 +16988,54 @@
       </c>
       <c r="C518" s="2" t="inlineStr">
         <is>
-          <t>A6519</t>
+          <t>A5679</t>
         </is>
       </c>
       <c r="D518" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723479</t>
+          <t>00019200000012756008</t>
         </is>
       </c>
       <c r="E518" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 05:33</t>
+          <t>09/06/2026 09:08</t>
         </is>
       </c>
       <c r="F518" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 12:15</t>
+          <t>11/06/2026 13:30</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>556160</t>
+          <t>556744</t>
         </is>
       </c>
       <c r="B519" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C519" s="2" t="inlineStr">
         <is>
-          <t>A9538</t>
+          <t>A6519</t>
         </is>
       </c>
       <c r="D519" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730009</t>
+          <t>00019200000012723479</t>
         </is>
       </c>
       <c r="E519" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 11:33</t>
+          <t>08/06/2026 05:33</t>
         </is>
       </c>
       <c r="F519" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 11:46</t>
+          <t>09/06/2026 12:15</t>
         </is>
       </c>
     </row>
@@ -17052,12 +17052,12 @@
       </c>
       <c r="C520" s="2" t="inlineStr">
         <is>
-          <t>TA0617</t>
+          <t>A9538</t>
         </is>
       </c>
       <c r="D520" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730882</t>
+          <t>00019200000012730009</t>
         </is>
       </c>
       <c r="E520" s="2" t="inlineStr">
@@ -17084,12 +17084,12 @@
       </c>
       <c r="C521" s="2" t="inlineStr">
         <is>
-          <t>A5841</t>
+          <t>TA0617</t>
         </is>
       </c>
       <c r="D521" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730890</t>
+          <t>00019200000012730882</t>
         </is>
       </c>
       <c r="E521" s="2" t="inlineStr">
@@ -17116,12 +17116,12 @@
       </c>
       <c r="C522" s="2" t="inlineStr">
         <is>
-          <t>A7704</t>
+          <t>A5841</t>
         </is>
       </c>
       <c r="D522" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730904</t>
+          <t>00019200000012730890</t>
         </is>
       </c>
       <c r="E522" s="2" t="inlineStr">
@@ -17148,12 +17148,12 @@
       </c>
       <c r="C523" s="2" t="inlineStr">
         <is>
-          <t>A6707</t>
+          <t>A7704</t>
         </is>
       </c>
       <c r="D523" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730912</t>
+          <t>00019200000012730904</t>
         </is>
       </c>
       <c r="E523" s="2" t="inlineStr">
@@ -17178,10 +17178,14 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C524" s="2" t="inlineStr"/>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>A6707</t>
+        </is>
+      </c>
       <c r="D524" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730920</t>
+          <t>00019200000012730912</t>
         </is>
       </c>
       <c r="E524" s="2" t="inlineStr">
@@ -17206,14 +17210,10 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="C525" s="2" t="inlineStr">
-        <is>
-          <t>A5971</t>
-        </is>
-      </c>
+      <c r="C525" s="2" t="inlineStr"/>
       <c r="D525" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730939</t>
+          <t>00019200000012730920</t>
         </is>
       </c>
       <c r="E525" s="2" t="inlineStr">
@@ -17240,12 +17240,12 @@
       </c>
       <c r="C526" s="2" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A5971</t>
         </is>
       </c>
       <c r="D526" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731005</t>
+          <t>00019200000012730939</t>
         </is>
       </c>
       <c r="E526" s="2" t="inlineStr">
@@ -17272,12 +17272,12 @@
       </c>
       <c r="C527" s="2" t="inlineStr">
         <is>
-          <t>A7331</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D527" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731560</t>
+          <t>00019200000012731005</t>
         </is>
       </c>
       <c r="E527" s="2" t="inlineStr">
@@ -17304,12 +17304,12 @@
       </c>
       <c r="C528" s="2" t="inlineStr">
         <is>
-          <t>A2361</t>
+          <t>A7331</t>
         </is>
       </c>
       <c r="D528" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731579</t>
+          <t>00019200000012731560</t>
         </is>
       </c>
       <c r="E528" s="2" t="inlineStr">
@@ -17336,12 +17336,12 @@
       </c>
       <c r="C529" s="2" t="inlineStr">
         <is>
-          <t>A9716</t>
+          <t>A2361</t>
         </is>
       </c>
       <c r="D529" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731587</t>
+          <t>00019200000012731579</t>
         </is>
       </c>
       <c r="E529" s="2" t="inlineStr">
@@ -17368,12 +17368,12 @@
       </c>
       <c r="C530" s="2" t="inlineStr">
         <is>
-          <t>A9274</t>
+          <t>A9716</t>
         </is>
       </c>
       <c r="D530" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731595</t>
+          <t>00019200000012731587</t>
         </is>
       </c>
       <c r="E530" s="2" t="inlineStr">
@@ -17400,12 +17400,12 @@
       </c>
       <c r="C531" s="2" t="inlineStr">
         <is>
-          <t>A7020</t>
+          <t>A9274</t>
         </is>
       </c>
       <c r="D531" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731609</t>
+          <t>00019200000012731595</t>
         </is>
       </c>
       <c r="E531" s="2" t="inlineStr">
@@ -17432,12 +17432,12 @@
       </c>
       <c r="C532" s="2" t="inlineStr">
         <is>
-          <t>A8090</t>
+          <t>A7020</t>
         </is>
       </c>
       <c r="D532" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731617</t>
+          <t>00019200000012731609</t>
         </is>
       </c>
       <c r="E532" s="2" t="inlineStr">
@@ -17464,12 +17464,12 @@
       </c>
       <c r="C533" s="2" t="inlineStr">
         <is>
-          <t>A2173</t>
+          <t>A8090</t>
         </is>
       </c>
       <c r="D533" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731625</t>
+          <t>00019200000012731617</t>
         </is>
       </c>
       <c r="E533" s="2" t="inlineStr">
@@ -17496,12 +17496,12 @@
       </c>
       <c r="C534" s="2" t="inlineStr">
         <is>
-          <t>A5456</t>
+          <t>A2173</t>
         </is>
       </c>
       <c r="D534" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731633</t>
+          <t>00019200000012731625</t>
         </is>
       </c>
       <c r="E534" s="2" t="inlineStr">
@@ -17528,12 +17528,12 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>A8993</t>
+          <t>A5456</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731641</t>
+          <t>00019200000012731633</t>
         </is>
       </c>
       <c r="E535" s="2" t="inlineStr">
@@ -17560,12 +17560,12 @@
       </c>
       <c r="C536" s="2" t="inlineStr">
         <is>
-          <t>A7043</t>
+          <t>A8993</t>
         </is>
       </c>
       <c r="D536" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731650</t>
+          <t>00019200000012731641</t>
         </is>
       </c>
       <c r="E536" s="2" t="inlineStr">
@@ -17592,12 +17592,12 @@
       </c>
       <c r="C537" s="2" t="inlineStr">
         <is>
-          <t>A6600</t>
+          <t>A7043</t>
         </is>
       </c>
       <c r="D537" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731668</t>
+          <t>00019200000012731650</t>
         </is>
       </c>
       <c r="E537" s="2" t="inlineStr">
@@ -17624,12 +17624,12 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>A6518</t>
+          <t>A6600</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731676</t>
+          <t>00019200000012731668</t>
         </is>
       </c>
       <c r="E538" s="2" t="inlineStr">
@@ -17656,12 +17656,12 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>A6804</t>
+          <t>A6518</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731684</t>
+          <t>00019200000012731676</t>
         </is>
       </c>
       <c r="E539" s="2" t="inlineStr">
@@ -17688,12 +17688,12 @@
       </c>
       <c r="C540" s="2" t="inlineStr">
         <is>
-          <t>A1679</t>
+          <t>A6804</t>
         </is>
       </c>
       <c r="D540" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731692</t>
+          <t>00019200000012731684</t>
         </is>
       </c>
       <c r="E540" s="2" t="inlineStr">
@@ -17720,12 +17720,12 @@
       </c>
       <c r="C541" s="2" t="inlineStr">
         <is>
-          <t>A6311</t>
+          <t>A1679</t>
         </is>
       </c>
       <c r="D541" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731803</t>
+          <t>00019200000012731692</t>
         </is>
       </c>
       <c r="E541" s="2" t="inlineStr">
@@ -17752,12 +17752,12 @@
       </c>
       <c r="C542" s="2" t="inlineStr">
         <is>
-          <t>TA0484</t>
+          <t>A6311</t>
         </is>
       </c>
       <c r="D542" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731900</t>
+          <t>00019200000012731803</t>
         </is>
       </c>
       <c r="E542" s="2" t="inlineStr">
@@ -17784,12 +17784,12 @@
       </c>
       <c r="C543" s="2" t="inlineStr">
         <is>
-          <t>A9205</t>
+          <t>TA0484</t>
         </is>
       </c>
       <c r="D543" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731919</t>
+          <t>00019200000012731900</t>
         </is>
       </c>
       <c r="E543" s="2" t="inlineStr">
@@ -17816,12 +17816,12 @@
       </c>
       <c r="C544" s="2" t="inlineStr">
         <is>
-          <t>A1019</t>
+          <t>A9205</t>
         </is>
       </c>
       <c r="D544" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731927</t>
+          <t>00019200000012731919</t>
         </is>
       </c>
       <c r="E544" s="2" t="inlineStr">
@@ -17848,12 +17848,12 @@
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>A6694</t>
+          <t>A1019</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731935</t>
+          <t>00019200000012731927</t>
         </is>
       </c>
       <c r="E545" s="2" t="inlineStr">
@@ -17880,12 +17880,12 @@
       </c>
       <c r="C546" s="2" t="inlineStr">
         <is>
-          <t>A4625</t>
+          <t>A6694</t>
         </is>
       </c>
       <c r="D546" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731943</t>
+          <t>00019200000012731935</t>
         </is>
       </c>
       <c r="E546" s="2" t="inlineStr">
@@ -17912,12 +17912,12 @@
       </c>
       <c r="C547" s="2" t="inlineStr">
         <is>
-          <t>A7288</t>
+          <t>A4625</t>
         </is>
       </c>
       <c r="D547" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731951</t>
+          <t>00019200000012731943</t>
         </is>
       </c>
       <c r="E547" s="2" t="inlineStr">
@@ -17944,12 +17944,12 @@
       </c>
       <c r="C548" s="2" t="inlineStr">
         <is>
-          <t>A7878</t>
+          <t>A7288</t>
         </is>
       </c>
       <c r="D548" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731960</t>
+          <t>00019200000012731951</t>
         </is>
       </c>
       <c r="E548" s="2" t="inlineStr">
@@ -17976,12 +17976,12 @@
       </c>
       <c r="C549" s="2" t="inlineStr">
         <is>
-          <t>A0974</t>
+          <t>A7878</t>
         </is>
       </c>
       <c r="D549" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731978</t>
+          <t>00019200000012731960</t>
         </is>
       </c>
       <c r="E549" s="2" t="inlineStr">
@@ -18008,12 +18008,12 @@
       </c>
       <c r="C550" s="2" t="inlineStr">
         <is>
-          <t>A8869</t>
+          <t>A0974</t>
         </is>
       </c>
       <c r="D550" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731986</t>
+          <t>00019200000012731978</t>
         </is>
       </c>
       <c r="E550" s="2" t="inlineStr">
@@ -18040,12 +18040,12 @@
       </c>
       <c r="C551" s="2" t="inlineStr">
         <is>
-          <t>A7491</t>
+          <t>A8869</t>
         </is>
       </c>
       <c r="D551" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731994</t>
+          <t>00019200000012731986</t>
         </is>
       </c>
       <c r="E551" s="2" t="inlineStr">
@@ -18072,12 +18072,12 @@
       </c>
       <c r="C552" s="2" t="inlineStr">
         <is>
-          <t>A6871</t>
+          <t>A7491</t>
         </is>
       </c>
       <c r="D552" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732001</t>
+          <t>00019200000012731994</t>
         </is>
       </c>
       <c r="E552" s="2" t="inlineStr">
@@ -18104,12 +18104,12 @@
       </c>
       <c r="C553" s="2" t="inlineStr">
         <is>
-          <t>A1824</t>
+          <t>A6871</t>
         </is>
       </c>
       <c r="D553" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732010</t>
+          <t>00019200000012732001</t>
         </is>
       </c>
       <c r="E553" s="2" t="inlineStr">
@@ -18136,12 +18136,12 @@
       </c>
       <c r="C554" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A1824</t>
         </is>
       </c>
       <c r="D554" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732028</t>
+          <t>00019200000012732010</t>
         </is>
       </c>
       <c r="E554" s="2" t="inlineStr">
@@ -18168,12 +18168,12 @@
       </c>
       <c r="C555" s="2" t="inlineStr">
         <is>
-          <t>A9638</t>
+          <t>A9207</t>
         </is>
       </c>
       <c r="D555" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732036</t>
+          <t>00019200000012732028</t>
         </is>
       </c>
       <c r="E555" s="2" t="inlineStr">
@@ -18200,12 +18200,12 @@
       </c>
       <c r="C556" s="2" t="inlineStr">
         <is>
-          <t>TA1173</t>
+          <t>A9638</t>
         </is>
       </c>
       <c r="D556" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732044</t>
+          <t>00019200000012732036</t>
         </is>
       </c>
       <c r="E556" s="2" t="inlineStr">
@@ -18232,12 +18232,12 @@
       </c>
       <c r="C557" s="2" t="inlineStr">
         <is>
-          <t>A9280</t>
+          <t>TA1173</t>
         </is>
       </c>
       <c r="D557" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732052</t>
+          <t>00019200000012732044</t>
         </is>
       </c>
       <c r="E557" s="2" t="inlineStr">
@@ -18264,12 +18264,12 @@
       </c>
       <c r="C558" s="2" t="inlineStr">
         <is>
-          <t>A6843</t>
+          <t>A9280</t>
         </is>
       </c>
       <c r="D558" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732060</t>
+          <t>00019200000012732052</t>
         </is>
       </c>
       <c r="E558" s="2" t="inlineStr">
@@ -18296,12 +18296,12 @@
       </c>
       <c r="C559" s="2" t="inlineStr">
         <is>
-          <t>A8045</t>
+          <t>A6843</t>
         </is>
       </c>
       <c r="D559" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732079</t>
+          <t>00019200000012732060</t>
         </is>
       </c>
       <c r="E559" s="2" t="inlineStr">
@@ -18328,12 +18328,12 @@
       </c>
       <c r="C560" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A8045</t>
         </is>
       </c>
       <c r="D560" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732087</t>
+          <t>00019200000012732079</t>
         </is>
       </c>
       <c r="E560" s="2" t="inlineStr">
@@ -18360,12 +18360,12 @@
       </c>
       <c r="C561" s="2" t="inlineStr">
         <is>
-          <t>A1989</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D561" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732095</t>
+          <t>00019200000012732087</t>
         </is>
       </c>
       <c r="E561" s="2" t="inlineStr">
@@ -18392,12 +18392,12 @@
       </c>
       <c r="C562" s="2" t="inlineStr">
         <is>
-          <t>TA0654</t>
+          <t>A1989</t>
         </is>
       </c>
       <c r="D562" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732109</t>
+          <t>00019200000012732095</t>
         </is>
       </c>
       <c r="E562" s="2" t="inlineStr">
@@ -18424,12 +18424,12 @@
       </c>
       <c r="C563" s="2" t="inlineStr">
         <is>
-          <t>A4447</t>
+          <t>TA0654</t>
         </is>
       </c>
       <c r="D563" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732117</t>
+          <t>00019200000012732109</t>
         </is>
       </c>
       <c r="E563" s="2" t="inlineStr">
@@ -18456,12 +18456,12 @@
       </c>
       <c r="C564" s="2" t="inlineStr">
         <is>
-          <t>A8046</t>
+          <t>A4447</t>
         </is>
       </c>
       <c r="D564" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732125</t>
+          <t>00019200000012732117</t>
         </is>
       </c>
       <c r="E564" s="2" t="inlineStr">
@@ -18488,12 +18488,12 @@
       </c>
       <c r="C565" s="2" t="inlineStr">
         <is>
-          <t>A3920</t>
+          <t>A8046</t>
         </is>
       </c>
       <c r="D565" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732133</t>
+          <t>00019200000012732125</t>
         </is>
       </c>
       <c r="E565" s="2" t="inlineStr">
@@ -18520,12 +18520,12 @@
       </c>
       <c r="C566" s="2" t="inlineStr">
         <is>
-          <t>A7425</t>
+          <t>A3920</t>
         </is>
       </c>
       <c r="D566" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732141</t>
+          <t>00019200000012732133</t>
         </is>
       </c>
       <c r="E566" s="2" t="inlineStr">
@@ -18552,12 +18552,12 @@
       </c>
       <c r="C567" s="2" t="inlineStr">
         <is>
-          <t>A3679</t>
+          <t>A7425</t>
         </is>
       </c>
       <c r="D567" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732150</t>
+          <t>00019200000012732141</t>
         </is>
       </c>
       <c r="E567" s="2" t="inlineStr">
@@ -18584,12 +18584,12 @@
       </c>
       <c r="C568" s="2" t="inlineStr">
         <is>
-          <t>A7985</t>
+          <t>A3679</t>
         </is>
       </c>
       <c r="D568" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732168</t>
+          <t>00019200000012732150</t>
         </is>
       </c>
       <c r="E568" s="2" t="inlineStr">
@@ -18616,12 +18616,12 @@
       </c>
       <c r="C569" s="2" t="inlineStr">
         <is>
-          <t>A6562</t>
+          <t>A7985</t>
         </is>
       </c>
       <c r="D569" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732176</t>
+          <t>00019200000012732168</t>
         </is>
       </c>
       <c r="E569" s="2" t="inlineStr">
@@ -18648,12 +18648,12 @@
       </c>
       <c r="C570" s="2" t="inlineStr">
         <is>
-          <t>A4360</t>
+          <t>A6562</t>
         </is>
       </c>
       <c r="D570" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732184</t>
+          <t>00019200000012732176</t>
         </is>
       </c>
       <c r="E570" s="2" t="inlineStr">
@@ -18680,12 +18680,12 @@
       </c>
       <c r="C571" s="2" t="inlineStr">
         <is>
-          <t>A9173</t>
+          <t>A4360</t>
         </is>
       </c>
       <c r="D571" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732192</t>
+          <t>00019200000012732184</t>
         </is>
       </c>
       <c r="E571" s="2" t="inlineStr">
@@ -18712,12 +18712,12 @@
       </c>
       <c r="C572" s="2" t="inlineStr">
         <is>
-          <t>A2809</t>
+          <t>A9173</t>
         </is>
       </c>
       <c r="D572" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732206</t>
+          <t>00019200000012732192</t>
         </is>
       </c>
       <c r="E572" s="2" t="inlineStr">
@@ -18744,12 +18744,12 @@
       </c>
       <c r="C573" s="2" t="inlineStr">
         <is>
-          <t>TA0960</t>
+          <t>A2809</t>
         </is>
       </c>
       <c r="D573" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732214</t>
+          <t>00019200000012732206</t>
         </is>
       </c>
       <c r="E573" s="2" t="inlineStr">
@@ -18776,12 +18776,12 @@
       </c>
       <c r="C574" s="2" t="inlineStr">
         <is>
-          <t>A8179</t>
+          <t>TA0960</t>
         </is>
       </c>
       <c r="D574" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732222</t>
+          <t>00019200000012732214</t>
         </is>
       </c>
       <c r="E574" s="2" t="inlineStr">
@@ -18808,12 +18808,12 @@
       </c>
       <c r="C575" s="2" t="inlineStr">
         <is>
-          <t>A9307</t>
+          <t>A8179</t>
         </is>
       </c>
       <c r="D575" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732230</t>
+          <t>00019200000012732222</t>
         </is>
       </c>
       <c r="E575" s="2" t="inlineStr">
@@ -18840,12 +18840,12 @@
       </c>
       <c r="C576" s="2" t="inlineStr">
         <is>
-          <t>A7068</t>
+          <t>A9307</t>
         </is>
       </c>
       <c r="D576" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732249</t>
+          <t>00019200000012732230</t>
         </is>
       </c>
       <c r="E576" s="2" t="inlineStr">
@@ -18872,12 +18872,12 @@
       </c>
       <c r="C577" s="2" t="inlineStr">
         <is>
-          <t>A3376</t>
+          <t>A7068</t>
         </is>
       </c>
       <c r="D577" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732257</t>
+          <t>00019200000012732249</t>
         </is>
       </c>
       <c r="E577" s="2" t="inlineStr">
@@ -18904,12 +18904,12 @@
       </c>
       <c r="C578" s="2" t="inlineStr">
         <is>
-          <t>A3287</t>
+          <t>A3376</t>
         </is>
       </c>
       <c r="D578" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732265</t>
+          <t>00019200000012732257</t>
         </is>
       </c>
       <c r="E578" s="2" t="inlineStr">
@@ -18936,12 +18936,12 @@
       </c>
       <c r="C579" s="2" t="inlineStr">
         <is>
-          <t>A9200</t>
+          <t>A3287</t>
         </is>
       </c>
       <c r="D579" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732273</t>
+          <t>00019200000012732265</t>
         </is>
       </c>
       <c r="E579" s="2" t="inlineStr">
@@ -18968,12 +18968,12 @@
       </c>
       <c r="C580" s="2" t="inlineStr">
         <is>
-          <t>A5037</t>
+          <t>A9200</t>
         </is>
       </c>
       <c r="D580" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732281</t>
+          <t>00019200000012732273</t>
         </is>
       </c>
       <c r="E580" s="2" t="inlineStr">
@@ -19000,12 +19000,12 @@
       </c>
       <c r="C581" s="2" t="inlineStr">
         <is>
-          <t>A9610</t>
+          <t>A5037</t>
         </is>
       </c>
       <c r="D581" s="2" t="inlineStr">
         <is>
-          <t>00019200000012732290</t>
+          <t>00019200000012732281</t>
         </is>
       </c>
       <c r="E581" s="2" t="inlineStr">
@@ -19032,12 +19032,12 @@
       </c>
       <c r="C582" s="2" t="inlineStr">
         <is>
-          <t>A1420</t>
+          <t>A9610</t>
         </is>
       </c>
       <c r="D582" s="2" t="inlineStr">
         <is>
-          <t>00019200000012857750</t>
+          <t>00019200000012732290</t>
         </is>
       </c>
       <c r="E582" s="2" t="inlineStr">
@@ -19054,7 +19054,7 @@
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>556224</t>
+          <t>556160</t>
         </is>
       </c>
       <c r="B583" s="2" t="inlineStr">
@@ -19064,29 +19064,29 @@
       </c>
       <c r="C583" s="2" t="inlineStr">
         <is>
-          <t>A4220</t>
+          <t>A1420</t>
         </is>
       </c>
       <c r="D583" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729043</t>
+          <t>00019200000012857750</t>
         </is>
       </c>
       <c r="E583" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 05:11</t>
+          <t>06/06/2026 11:33</t>
         </is>
       </c>
       <c r="F583" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 16:00</t>
+          <t>08/06/2026 11:46</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>556409</t>
+          <t>556224</t>
         </is>
       </c>
       <c r="B584" s="2" t="inlineStr">
@@ -19096,22 +19096,22 @@
       </c>
       <c r="C584" s="2" t="inlineStr">
         <is>
-          <t>A8078</t>
+          <t>A4220</t>
         </is>
       </c>
       <c r="D584" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723550</t>
+          <t>00019200000012729043</t>
         </is>
       </c>
       <c r="E584" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 06:40</t>
+          <t>11/06/2026 05:11</t>
         </is>
       </c>
       <c r="F584" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026 17:18</t>
+          <t>12/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -19128,12 +19128,12 @@
       </c>
       <c r="C585" s="2" t="inlineStr">
         <is>
-          <t>A0401</t>
+          <t>A8078</t>
         </is>
       </c>
       <c r="D585" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723568</t>
+          <t>00019200000012723550</t>
         </is>
       </c>
       <c r="E585" s="2" t="inlineStr">
@@ -19160,12 +19160,12 @@
       </c>
       <c r="C586" s="2" t="inlineStr">
         <is>
-          <t>A8580</t>
+          <t>A0401</t>
         </is>
       </c>
       <c r="D586" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723592</t>
+          <t>00019200000012723568</t>
         </is>
       </c>
       <c r="E586" s="2" t="inlineStr">
@@ -19182,32 +19182,32 @@
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>555932</t>
+          <t>556409</t>
         </is>
       </c>
       <c r="B587" s="2" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C587" s="2" t="inlineStr">
         <is>
-          <t>A4257</t>
+          <t>A8580</t>
         </is>
       </c>
       <c r="D587" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721840</t>
+          <t>00019200000012723592</t>
         </is>
       </c>
       <c r="E587" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:18</t>
+          <t>10/06/2026 06:40</t>
         </is>
       </c>
       <c r="F587" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 09:33</t>
+          <t>11/06/2026 17:18</t>
         </is>
       </c>
     </row>
@@ -19224,12 +19224,12 @@
       </c>
       <c r="C588" s="2" t="inlineStr">
         <is>
-          <t>A9287</t>
+          <t>A4257</t>
         </is>
       </c>
       <c r="D588" s="2" t="inlineStr">
         <is>
-          <t>00019200000012723061</t>
+          <t>00019200000012721840</t>
         </is>
       </c>
       <c r="E588" s="2" t="inlineStr">
@@ -19246,7 +19246,7 @@
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>556161</t>
+          <t>555932</t>
         </is>
       </c>
       <c r="B589" s="2" t="inlineStr">
@@ -19256,22 +19256,22 @@
       </c>
       <c r="C589" s="2" t="inlineStr">
         <is>
-          <t>A7008</t>
+          <t>A9287</t>
         </is>
       </c>
       <c r="D589" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730491</t>
+          <t>00019200000012723061</t>
         </is>
       </c>
       <c r="E589" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:18</t>
         </is>
       </c>
       <c r="F589" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 14:51</t>
+          <t>03/06/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -19288,12 +19288,12 @@
       </c>
       <c r="C590" s="2" t="inlineStr">
         <is>
-          <t>A7785</t>
+          <t>A7008</t>
         </is>
       </c>
       <c r="D590" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730670</t>
+          <t>00019200000012730491</t>
         </is>
       </c>
       <c r="E590" s="2" t="inlineStr">
@@ -19320,12 +19320,12 @@
       </c>
       <c r="C591" s="2" t="inlineStr">
         <is>
-          <t>A6386</t>
+          <t>A7785</t>
         </is>
       </c>
       <c r="D591" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730688</t>
+          <t>00019200000012730670</t>
         </is>
       </c>
       <c r="E591" s="2" t="inlineStr">
@@ -19352,12 +19352,12 @@
       </c>
       <c r="C592" s="2" t="inlineStr">
         <is>
-          <t>A8302</t>
+          <t>A6386</t>
         </is>
       </c>
       <c r="D592" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730696</t>
+          <t>00019200000012730688</t>
         </is>
       </c>
       <c r="E592" s="2" t="inlineStr">
@@ -19384,12 +19384,12 @@
       </c>
       <c r="C593" s="2" t="inlineStr">
         <is>
-          <t>A6870</t>
+          <t>A8302</t>
         </is>
       </c>
       <c r="D593" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730700</t>
+          <t>00019200000012730696</t>
         </is>
       </c>
       <c r="E593" s="2" t="inlineStr">
@@ -19416,12 +19416,12 @@
       </c>
       <c r="C594" s="2" t="inlineStr">
         <is>
-          <t>A8192</t>
+          <t>A6870</t>
         </is>
       </c>
       <c r="D594" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731331</t>
+          <t>00019200000012730700</t>
         </is>
       </c>
       <c r="E594" s="2" t="inlineStr">
@@ -19448,12 +19448,12 @@
       </c>
       <c r="C595" s="2" t="inlineStr">
         <is>
-          <t>A1045</t>
+          <t>A8192</t>
         </is>
       </c>
       <c r="D595" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731340</t>
+          <t>00019200000012731331</t>
         </is>
       </c>
       <c r="E595" s="2" t="inlineStr">
@@ -19480,12 +19480,12 @@
       </c>
       <c r="C596" s="2" t="inlineStr">
         <is>
-          <t>A3603</t>
+          <t>A1045</t>
         </is>
       </c>
       <c r="D596" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731358</t>
+          <t>00019200000012731340</t>
         </is>
       </c>
       <c r="E596" s="2" t="inlineStr">
@@ -19512,12 +19512,12 @@
       </c>
       <c r="C597" s="2" t="inlineStr">
         <is>
-          <t>A9427</t>
+          <t>A3603</t>
         </is>
       </c>
       <c r="D597" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731366</t>
+          <t>00019200000012731358</t>
         </is>
       </c>
       <c r="E597" s="2" t="inlineStr">
@@ -19544,12 +19544,12 @@
       </c>
       <c r="C598" s="2" t="inlineStr">
         <is>
-          <t>A4068</t>
+          <t>A9427</t>
         </is>
       </c>
       <c r="D598" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731374</t>
+          <t>00019200000012731366</t>
         </is>
       </c>
       <c r="E598" s="2" t="inlineStr">
@@ -19576,12 +19576,12 @@
       </c>
       <c r="C599" s="2" t="inlineStr">
         <is>
-          <t>A2753</t>
+          <t>A4068</t>
         </is>
       </c>
       <c r="D599" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731382</t>
+          <t>00019200000012731374</t>
         </is>
       </c>
       <c r="E599" s="2" t="inlineStr">
@@ -19608,12 +19608,12 @@
       </c>
       <c r="C600" s="2" t="inlineStr">
         <is>
-          <t>TA0353</t>
+          <t>A2753</t>
         </is>
       </c>
       <c r="D600" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731390</t>
+          <t>00019200000012731382</t>
         </is>
       </c>
       <c r="E600" s="2" t="inlineStr">
@@ -19640,12 +19640,12 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>A7155</t>
+          <t>TA0353</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731404</t>
+          <t>00019200000012731390</t>
         </is>
       </c>
       <c r="E601" s="2" t="inlineStr">
@@ -19672,12 +19672,12 @@
       </c>
       <c r="C602" s="2" t="inlineStr">
         <is>
-          <t>A6665</t>
+          <t>A7155</t>
         </is>
       </c>
       <c r="D602" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731412</t>
+          <t>00019200000012731404</t>
         </is>
       </c>
       <c r="E602" s="2" t="inlineStr">
@@ -19704,12 +19704,12 @@
       </c>
       <c r="C603" s="2" t="inlineStr">
         <is>
-          <t>TA0675</t>
+          <t>A6665</t>
         </is>
       </c>
       <c r="D603" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731420</t>
+          <t>00019200000012731412</t>
         </is>
       </c>
       <c r="E603" s="2" t="inlineStr">
@@ -19736,12 +19736,12 @@
       </c>
       <c r="C604" s="2" t="inlineStr">
         <is>
-          <t>A7142</t>
+          <t>TA0675</t>
         </is>
       </c>
       <c r="D604" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731439</t>
+          <t>00019200000012731420</t>
         </is>
       </c>
       <c r="E604" s="2" t="inlineStr">
@@ -19768,12 +19768,12 @@
       </c>
       <c r="C605" s="2" t="inlineStr">
         <is>
-          <t>TA0136</t>
+          <t>A7142</t>
         </is>
       </c>
       <c r="D605" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731447</t>
+          <t>00019200000012731439</t>
         </is>
       </c>
       <c r="E605" s="2" t="inlineStr">
@@ -19800,12 +19800,12 @@
       </c>
       <c r="C606" s="2" t="inlineStr">
         <is>
-          <t>TA0818</t>
+          <t>TA0136</t>
         </is>
       </c>
       <c r="D606" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731455</t>
+          <t>00019200000012731447</t>
         </is>
       </c>
       <c r="E606" s="2" t="inlineStr">
@@ -19832,12 +19832,12 @@
       </c>
       <c r="C607" s="2" t="inlineStr">
         <is>
-          <t>A6147</t>
+          <t>TA0818</t>
         </is>
       </c>
       <c r="D607" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731463</t>
+          <t>00019200000012731455</t>
         </is>
       </c>
       <c r="E607" s="2" t="inlineStr">
@@ -19864,12 +19864,12 @@
       </c>
       <c r="C608" s="2" t="inlineStr">
         <is>
-          <t>A4999</t>
+          <t>A6147</t>
         </is>
       </c>
       <c r="D608" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731471</t>
+          <t>00019200000012731463</t>
         </is>
       </c>
       <c r="E608" s="2" t="inlineStr">
@@ -19896,12 +19896,12 @@
       </c>
       <c r="C609" s="2" t="inlineStr">
         <is>
-          <t>A5847</t>
+          <t>A4999</t>
         </is>
       </c>
       <c r="D609" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731498</t>
+          <t>00019200000012731471</t>
         </is>
       </c>
       <c r="E609" s="2" t="inlineStr">
@@ -19928,12 +19928,12 @@
       </c>
       <c r="C610" s="2" t="inlineStr">
         <is>
-          <t>A2981</t>
+          <t>A5847</t>
         </is>
       </c>
       <c r="D610" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731501</t>
+          <t>00019200000012731498</t>
         </is>
       </c>
       <c r="E610" s="2" t="inlineStr">
@@ -19960,12 +19960,12 @@
       </c>
       <c r="C611" s="2" t="inlineStr">
         <is>
-          <t>A7462</t>
+          <t>A2981</t>
         </is>
       </c>
       <c r="D611" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731510</t>
+          <t>00019200000012731501</t>
         </is>
       </c>
       <c r="E611" s="2" t="inlineStr">
@@ -19992,12 +19992,12 @@
       </c>
       <c r="C612" s="2" t="inlineStr">
         <is>
-          <t>A4340</t>
+          <t>A7462</t>
         </is>
       </c>
       <c r="D612" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731528</t>
+          <t>00019200000012731510</t>
         </is>
       </c>
       <c r="E612" s="2" t="inlineStr">
@@ -20024,12 +20024,12 @@
       </c>
       <c r="C613" s="2" t="inlineStr">
         <is>
-          <t>A8938</t>
+          <t>A4340</t>
         </is>
       </c>
       <c r="D613" s="2" t="inlineStr">
         <is>
-          <t>00019200000012731536</t>
+          <t>00019200000012731528</t>
         </is>
       </c>
       <c r="E613" s="2" t="inlineStr">
@@ -20046,7 +20046,7 @@
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>556300</t>
+          <t>556161</t>
         </is>
       </c>
       <c r="B614" s="2" t="inlineStr">
@@ -20056,54 +20056,54 @@
       </c>
       <c r="C614" s="2" t="inlineStr">
         <is>
-          <t>TA0506</t>
+          <t>A8938</t>
         </is>
       </c>
       <c r="D614" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728918</t>
+          <t>00019200000012731536</t>
         </is>
       </c>
       <c r="E614" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 10:36</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F614" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026 10:54</t>
+          <t>08/06/2026 14:51</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>556300</t>
         </is>
       </c>
       <c r="B615" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C615" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>TA0506</t>
         </is>
       </c>
       <c r="D615" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000012728918</t>
         </is>
       </c>
       <c r="E615" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>06/06/2026 10:36</t>
         </is>
       </c>
       <c r="F615" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>08/06/2026 10:54</t>
         </is>
       </c>
     </row>
@@ -20120,12 +20120,12 @@
       </c>
       <c r="C616" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D616" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E616" s="2" t="inlineStr">
@@ -20152,12 +20152,12 @@
       </c>
       <c r="C617" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D617" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E617" s="2" t="inlineStr">
@@ -20174,39 +20174,39 @@
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B618" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C618" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D618" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E618" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F618" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B619" s="2" t="inlineStr">
@@ -20216,22 +20216,22 @@
       </c>
       <c r="C619" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D619" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E619" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F619" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -20248,12 +20248,12 @@
       </c>
       <c r="C620" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D620" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E620" s="2" t="inlineStr">
@@ -20280,12 +20280,12 @@
       </c>
       <c r="C621" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D621" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E621" s="2" t="inlineStr">
@@ -20312,12 +20312,12 @@
       </c>
       <c r="C622" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D622" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E622" s="2" t="inlineStr">
@@ -20344,12 +20344,12 @@
       </c>
       <c r="C623" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D623" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E623" s="2" t="inlineStr">
@@ -20376,12 +20376,12 @@
       </c>
       <c r="C624" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D624" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E624" s="2" t="inlineStr">
@@ -20408,12 +20408,12 @@
       </c>
       <c r="C625" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D625" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E625" s="2" t="inlineStr">
@@ -20440,12 +20440,12 @@
       </c>
       <c r="C626" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D626" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E626" s="2" t="inlineStr">
@@ -20472,12 +20472,12 @@
       </c>
       <c r="C627" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D627" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E627" s="2" t="inlineStr">
@@ -20504,12 +20504,12 @@
       </c>
       <c r="C628" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D628" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E628" s="2" t="inlineStr">
@@ -20536,12 +20536,12 @@
       </c>
       <c r="C629" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D629" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E629" s="2" t="inlineStr">
@@ -20568,12 +20568,12 @@
       </c>
       <c r="C630" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D630" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E630" s="2" t="inlineStr">
@@ -20600,12 +20600,12 @@
       </c>
       <c r="C631" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D631" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E631" s="2" t="inlineStr">
@@ -20632,12 +20632,12 @@
       </c>
       <c r="C632" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D632" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E632" s="2" t="inlineStr">
@@ -20664,12 +20664,12 @@
       </c>
       <c r="C633" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D633" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E633" s="2" t="inlineStr">
@@ -20686,7 +20686,7 @@
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B634" s="2" t="inlineStr">
@@ -20696,22 +20696,22 @@
       </c>
       <c r="C634" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D634" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E634" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F634" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -20728,12 +20728,12 @@
       </c>
       <c r="C635" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D635" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E635" s="2" t="inlineStr">
@@ -20760,12 +20760,12 @@
       </c>
       <c r="C636" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D636" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E636" s="2" t="inlineStr">
@@ -20792,12 +20792,12 @@
       </c>
       <c r="C637" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D637" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E637" s="2" t="inlineStr">
@@ -20824,27 +20824,59 @@
       </c>
       <c r="C638" s="2" t="inlineStr">
         <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E638" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F638" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
           <t>A8196</t>
         </is>
       </c>
-      <c r="D638" s="2" t="inlineStr">
+      <c r="D639" s="2" t="inlineStr">
         <is>
           <t>00019200000012728802</t>
         </is>
       </c>
-      <c r="E638" s="2" t="inlineStr">
+      <c r="E639" s="2" t="inlineStr">
         <is>
           <t>09/06/2026 02:06</t>
         </is>
       </c>
-      <c r="F638" s="2" t="inlineStr">
+      <c r="F639" s="2" t="inlineStr">
         <is>
           <t>10/06/2026 11:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F638"/>
+  <autoFilter ref="A1:F639"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-18 12:20:31
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -6059,7 +6059,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6187,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6315,7 +6315,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6507,7 +6507,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6667,7 +6667,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6763,7 +6763,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6795,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6827,7 +6827,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6891,7 +6891,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6955,7 +6955,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -6987,7 +6987,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7019,7 +7019,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7051,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7147,7 +7147,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7211,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7275,7 +7275,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7307,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7339,7 +7339,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7371,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7403,7 +7403,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7435,7 +7435,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7467,7 +7467,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7499,7 +7499,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7563,7 +7563,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7595,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7723,7 +7723,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7947,7 +7947,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -8011,7 +8011,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18/06/2026 12:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-18 14:53:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10823,7 +10823,7 @@
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17/06/2026 08:00</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17/06/2026 08:00</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17/06/2026 08:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-19 11:50:57
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3403,7 +3403,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 10:46</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 10:46</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 10:46</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 10:46</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 10:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-19 18:13:17
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3051,7 +3051,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19/06/2026 18:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-22 13:48:55
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3646,7 +3646,11 @@
           <t>AM</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr"/>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>A6993</t>
+        </is>
+      </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
           <t>00019200000013211293</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-23 11:49:15
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$857</definedName>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-25 11:51:49
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -31271,7 +31271,7 @@
       </c>
       <c r="F964" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:49</t>
         </is>
       </c>
     </row>
@@ -31303,7 +31303,7 @@
       </c>
       <c r="F965" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:49</t>
         </is>
       </c>
     </row>
@@ -31335,7 +31335,7 @@
       </c>
       <c r="F966" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:49</t>
         </is>
       </c>
     </row>
@@ -31367,7 +31367,7 @@
       </c>
       <c r="F967" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-25 17:53:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -18891,7 +18891,7 @@
       </c>
       <c r="F577" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -18923,7 +18923,7 @@
       </c>
       <c r="F578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -18955,7 +18955,7 @@
       </c>
       <c r="F579" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -18987,7 +18987,7 @@
       </c>
       <c r="F580" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19019,7 +19019,7 @@
       </c>
       <c r="F581" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19051,7 +19051,7 @@
       </c>
       <c r="F582" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19083,7 +19083,7 @@
       </c>
       <c r="F583" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19115,7 +19115,7 @@
       </c>
       <c r="F584" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19147,7 +19147,7 @@
       </c>
       <c r="F585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19179,7 +19179,7 @@
       </c>
       <c r="F586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19211,7 +19211,7 @@
       </c>
       <c r="F587" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>
@@ -19243,7 +19243,7 @@
       </c>
       <c r="F588" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 08:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-26 10:18:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -14763,7 +14763,7 @@
       </c>
       <c r="F448" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14795,7 +14795,7 @@
       </c>
       <c r="F449" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14827,7 +14827,7 @@
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14859,7 +14859,7 @@
       </c>
       <c r="F451" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14891,7 +14891,7 @@
       </c>
       <c r="F452" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14923,7 +14923,7 @@
       </c>
       <c r="F453" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14955,7 +14955,7 @@
       </c>
       <c r="F454" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -14987,7 +14987,7 @@
       </c>
       <c r="F455" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15019,7 +15019,7 @@
       </c>
       <c r="F456" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15051,7 +15051,7 @@
       </c>
       <c r="F457" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15083,7 +15083,7 @@
       </c>
       <c r="F458" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15115,7 +15115,7 @@
       </c>
       <c r="F459" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15147,7 +15147,7 @@
       </c>
       <c r="F460" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>
@@ -15179,7 +15179,7 @@
       </c>
       <c r="F461" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 14:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-26 12:18:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -23371,7 +23371,7 @@
       </c>
       <c r="F717" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23403,7 +23403,7 @@
       </c>
       <c r="F718" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23435,7 +23435,7 @@
       </c>
       <c r="F719" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23467,7 +23467,7 @@
       </c>
       <c r="F720" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23499,7 +23499,7 @@
       </c>
       <c r="F721" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23531,7 +23531,7 @@
       </c>
       <c r="F722" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23563,7 +23563,7 @@
       </c>
       <c r="F723" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23595,7 +23595,7 @@
       </c>
       <c r="F724" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23627,7 +23627,7 @@
       </c>
       <c r="F725" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23659,7 +23659,7 @@
       </c>
       <c r="F726" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23691,7 +23691,7 @@
       </c>
       <c r="F727" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23723,7 +23723,7 @@
       </c>
       <c r="F728" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23755,7 +23755,7 @@
       </c>
       <c r="F729" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23787,7 +23787,7 @@
       </c>
       <c r="F730" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23819,7 +23819,7 @@
       </c>
       <c r="F731" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23851,7 +23851,7 @@
       </c>
       <c r="F732" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23883,7 +23883,7 @@
       </c>
       <c r="F733" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23915,7 +23915,7 @@
       </c>
       <c r="F734" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23947,7 +23947,7 @@
       </c>
       <c r="F735" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -23979,7 +23979,7 @@
       </c>
       <c r="F736" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24011,7 +24011,7 @@
       </c>
       <c r="F737" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24043,7 +24043,7 @@
       </c>
       <c r="F738" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24075,7 +24075,7 @@
       </c>
       <c r="F739" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24107,7 +24107,7 @@
       </c>
       <c r="F740" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24139,7 +24139,7 @@
       </c>
       <c r="F741" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24171,7 +24171,7 @@
       </c>
       <c r="F742" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24203,7 +24203,7 @@
       </c>
       <c r="F743" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24235,7 +24235,7 @@
       </c>
       <c r="F744" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24267,7 +24267,7 @@
       </c>
       <c r="F745" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -24299,7 +24299,7 @@
       </c>
       <c r="F746" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>25/06/2026 11:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-26 14:56:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -19644,7 +19644,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>A9183</t>
+          <t>A8841</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -23644,7 +23644,7 @@
       </c>
       <c r="C726" s="2" t="inlineStr">
         <is>
-          <t>A5656</t>
+          <t>A6993</t>
         </is>
       </c>
       <c r="D726" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-26 15:23:11
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -16299,7 +16299,7 @@
       </c>
       <c r="F496" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -16331,7 +16331,7 @@
       </c>
       <c r="F497" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 10:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-26 17:35:36
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -19644,7 +19644,7 @@
       </c>
       <c r="C601" s="2" t="inlineStr">
         <is>
-          <t>A8841</t>
+          <t>A3013</t>
         </is>
       </c>
       <c r="D601" s="2" t="inlineStr">
@@ -23644,7 +23644,7 @@
       </c>
       <c r="C726" s="2" t="inlineStr">
         <is>
-          <t>A6993</t>
+          <t>A5656</t>
         </is>
       </c>
       <c r="D726" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-27 09:26:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -31143,7 +31143,7 @@
       </c>
       <c r="F960" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -31175,7 +31175,7 @@
       </c>
       <c r="F961" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -31207,7 +31207,7 @@
       </c>
       <c r="F962" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 16:00</t>
         </is>
       </c>
     </row>
@@ -31239,7 +31239,7 @@
       </c>
       <c r="F963" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 16:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-29 16:47:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -17835,7 +17835,7 @@
       </c>
       <c r="F544" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17867,7 @@
       </c>
       <c r="F545" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -17899,7 +17899,7 @@
       </c>
       <c r="F546" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -17931,7 +17931,7 @@
       </c>
       <c r="F547" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -17963,7 +17963,7 @@
       </c>
       <c r="F548" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -17995,7 +17995,7 @@
       </c>
       <c r="F549" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18027,7 +18027,7 @@
       </c>
       <c r="F550" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18059,7 +18059,7 @@
       </c>
       <c r="F551" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18091,7 +18091,7 @@
       </c>
       <c r="F552" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18123,7 @@
       </c>
       <c r="F553" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18155,7 +18155,7 @@
       </c>
       <c r="F554" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18187,7 @@
       </c>
       <c r="F555" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18219,7 @@
       </c>
       <c r="F556" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18251,7 +18251,7 @@
       </c>
       <c r="F557" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18283,7 +18283,7 @@
       </c>
       <c r="F558" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18315,7 +18315,7 @@
       </c>
       <c r="F559" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18347,7 +18347,7 @@
       </c>
       <c r="F560" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18379,7 +18379,7 @@
       </c>
       <c r="F561" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18411,7 +18411,7 @@
       </c>
       <c r="F562" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18443,7 +18443,7 @@
       </c>
       <c r="F563" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18475,7 +18475,7 @@
       </c>
       <c r="F564" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18507,7 +18507,7 @@
       </c>
       <c r="F565" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18539,7 +18539,7 @@
       </c>
       <c r="F566" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18571,7 +18571,7 @@
       </c>
       <c r="F567" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18603,7 +18603,7 @@
       </c>
       <c r="F568" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18635,7 +18635,7 @@
       </c>
       <c r="F569" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18667,7 +18667,7 @@
       </c>
       <c r="F570" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18699,7 +18699,7 @@
       </c>
       <c r="F571" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18731,7 +18731,7 @@
       </c>
       <c r="F572" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18763,7 +18763,7 @@
       </c>
       <c r="F573" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18795,7 +18795,7 @@
       </c>
       <c r="F574" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18827,7 +18827,7 @@
       </c>
       <c r="F575" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -18859,7 +18859,7 @@
       </c>
       <c r="F576" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-06-30 12:38:55
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4719,7 +4719,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26/06/2026 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-01 17:55:27
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026 17:00</t>
+          <t>11/06/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -22603,7 +22603,7 @@
       </c>
       <c r="F693" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01/07/2026 15:21</t>
         </is>
       </c>
     </row>
@@ -22635,7 +22635,7 @@
       </c>
       <c r="F694" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01/07/2026 15:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-06 17:16:54
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -847,7 +847,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>06/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>06/07/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-07 21:50:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -17314,7 +17314,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C529" s="2" t="inlineStr"/>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>A0981</t>
+        </is>
+      </c>
       <c r="D529" s="2" t="inlineStr">
         <is>
           <t>00019200000012920711</t>
@@ -17342,7 +17346,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C530" s="2" t="inlineStr"/>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>A8237</t>
+        </is>
+      </c>
       <c r="D530" s="2" t="inlineStr">
         <is>
           <t>00019200000012920720</t>
@@ -17370,7 +17378,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C531" s="2" t="inlineStr"/>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>A8781</t>
+        </is>
+      </c>
       <c r="D531" s="2" t="inlineStr">
         <is>
           <t>00019200000012920738</t>
@@ -17398,7 +17410,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C532" s="2" t="inlineStr"/>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>A9569</t>
+        </is>
+      </c>
       <c r="D532" s="2" t="inlineStr">
         <is>
           <t>00019200000012920746</t>
@@ -18290,7 +18306,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C563" s="2" t="inlineStr"/>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>A8318</t>
+        </is>
+      </c>
       <c r="D563" s="2" t="inlineStr">
         <is>
           <t>00019200000013225715</t>
@@ -18318,7 +18338,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C564" s="2" t="inlineStr"/>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>A0854</t>
+        </is>
+      </c>
       <c r="D564" s="2" t="inlineStr">
         <is>
           <t>00019200000013225723</t>
@@ -18378,7 +18402,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C566" s="2" t="inlineStr"/>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>TA1072</t>
+        </is>
+      </c>
       <c r="D566" s="2" t="inlineStr">
         <is>
           <t>00019200000013225740</t>
@@ -18406,7 +18434,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C567" s="2" t="inlineStr"/>
+      <c r="C567" s="2" t="inlineStr">
+        <is>
+          <t>A3519</t>
+        </is>
+      </c>
       <c r="D567" s="2" t="inlineStr">
         <is>
           <t>00019200000013225758</t>
@@ -18434,7 +18466,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C568" s="2" t="inlineStr"/>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>A4443</t>
+        </is>
+      </c>
       <c r="D568" s="2" t="inlineStr">
         <is>
           <t>00019200000013225766</t>
@@ -18462,7 +18498,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C569" s="2" t="inlineStr"/>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>A6621</t>
+        </is>
+      </c>
       <c r="D569" s="2" t="inlineStr">
         <is>
           <t>00019200000013225774</t>
@@ -18490,7 +18530,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C570" s="2" t="inlineStr"/>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>A1201</t>
+        </is>
+      </c>
       <c r="D570" s="2" t="inlineStr">
         <is>
           <t>00019200000013225782</t>
@@ -18518,7 +18562,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C571" s="2" t="inlineStr"/>
+      <c r="C571" s="2" t="inlineStr">
+        <is>
+          <t>TA1084</t>
+        </is>
+      </c>
       <c r="D571" s="2" t="inlineStr">
         <is>
           <t>00019200000013225790</t>
@@ -18546,7 +18594,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C572" s="2" t="inlineStr"/>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>A7813</t>
+        </is>
+      </c>
       <c r="D572" s="2" t="inlineStr">
         <is>
           <t>00019200000013225804</t>
@@ -18574,7 +18626,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C573" s="2" t="inlineStr"/>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>A5803</t>
+        </is>
+      </c>
       <c r="D573" s="2" t="inlineStr">
         <is>
           <t>00019200000013225812</t>
@@ -18602,7 +18658,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C574" s="2" t="inlineStr"/>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>A4009</t>
+        </is>
+      </c>
       <c r="D574" s="2" t="inlineStr">
         <is>
           <t>00019200000013225820</t>
@@ -18630,7 +18690,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C575" s="2" t="inlineStr"/>
+      <c r="C575" s="2" t="inlineStr">
+        <is>
+          <t>A3330</t>
+        </is>
+      </c>
       <c r="D575" s="2" t="inlineStr">
         <is>
           <t>00019200000013225839</t>
@@ -18658,7 +18722,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C576" s="2" t="inlineStr"/>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>A9205</t>
+        </is>
+      </c>
       <c r="D576" s="2" t="inlineStr">
         <is>
           <t>00019200000013225847</t>
@@ -18686,7 +18754,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C577" s="2" t="inlineStr"/>
+      <c r="C577" s="2" t="inlineStr">
+        <is>
+          <t>A4620</t>
+        </is>
+      </c>
       <c r="D577" s="2" t="inlineStr">
         <is>
           <t>00019200000013225855</t>
@@ -18714,7 +18786,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C578" s="2" t="inlineStr"/>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>A9630</t>
+        </is>
+      </c>
       <c r="D578" s="2" t="inlineStr">
         <is>
           <t>00019200000013225863</t>
@@ -18742,7 +18818,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C579" s="2" t="inlineStr"/>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>A5327</t>
+        </is>
+      </c>
       <c r="D579" s="2" t="inlineStr">
         <is>
           <t>00019200000013225871</t>
@@ -18882,7 +18962,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C584" s="2" t="inlineStr"/>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>A6915</t>
+        </is>
+      </c>
       <c r="D584" s="2" t="inlineStr">
         <is>
           <t>00019200000013226282</t>
@@ -23183,7 +23267,7 @@
       </c>
       <c r="F719" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>07/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -23215,7 +23299,7 @@
       </c>
       <c r="F720" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>07/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -23247,7 +23331,7 @@
       </c>
       <c r="F721" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>07/07/2026 19:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 00:40:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$1151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$1167</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1151"/>
+  <dimension ref="A1:F1167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35974,711 +35974,711 @@
     <row r="1117">
       <c r="A1117" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1117" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1117" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>A7202</t>
         </is>
       </c>
       <c r="D1117" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000013417380</t>
         </is>
       </c>
       <c r="E1117" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1117" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1118">
       <c r="A1118" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1118" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1118" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>A8913</t>
         </is>
       </c>
       <c r="D1118" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000013417398</t>
         </is>
       </c>
       <c r="E1118" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1118" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1119">
       <c r="A1119" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1119" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1119" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A4339</t>
         </is>
       </c>
       <c r="D1119" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000013417606</t>
         </is>
       </c>
       <c r="E1119" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1119" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1120">
       <c r="A1120" s="2" t="inlineStr">
         <is>
-          <t>558604</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1120" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1120" s="2" t="inlineStr">
         <is>
-          <t>TA0996</t>
+          <t>A6547</t>
         </is>
       </c>
       <c r="D1120" s="2" t="inlineStr">
         <is>
-          <t>00019200000013336460</t>
+          <t>00019200000013417614</t>
         </is>
       </c>
       <c r="E1120" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1120" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:35</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1121">
       <c r="A1121" s="2" t="inlineStr">
         <is>
-          <t>558604</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1121" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1121" s="2" t="inlineStr">
         <is>
-          <t>A2883</t>
+          <t>A3702</t>
         </is>
       </c>
       <c r="D1121" s="2" t="inlineStr">
         <is>
-          <t>00019200000013336479</t>
+          <t>00019200000013417649</t>
         </is>
       </c>
       <c r="E1121" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1121" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:35</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1122">
       <c r="A1122" s="2" t="inlineStr">
         <is>
-          <t>558714</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1122" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1122" s="2" t="inlineStr">
         <is>
-          <t>A5902</t>
+          <t>A6309</t>
         </is>
       </c>
       <c r="D1122" s="2" t="inlineStr">
         <is>
-          <t>00019200000013234994</t>
+          <t>00019200000013417657</t>
         </is>
       </c>
       <c r="E1122" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1122" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:39</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1123">
       <c r="A1123" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1123" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1123" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A0745</t>
         </is>
       </c>
       <c r="D1123" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000013417665</t>
         </is>
       </c>
       <c r="E1123" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1123" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1124">
       <c r="A1124" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1124" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1124" s="2" t="inlineStr">
         <is>
-          <t>A0830</t>
+          <t>TA0005</t>
         </is>
       </c>
       <c r="D1124" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211269</t>
+          <t>00019200000013417673</t>
         </is>
       </c>
       <c r="E1124" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1124" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1125">
       <c r="A1125" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1125" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1125" s="2" t="inlineStr">
         <is>
-          <t>A0222</t>
+          <t>A8203</t>
         </is>
       </c>
       <c r="D1125" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211277</t>
+          <t>00019200000013417681</t>
         </is>
       </c>
       <c r="E1125" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1125" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1126">
       <c r="A1126" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
         <is>
-          <t>A8417</t>
+          <t>TA0512</t>
         </is>
       </c>
       <c r="D1126" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211285</t>
+          <t>00019200000013417690</t>
         </is>
       </c>
       <c r="E1126" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1126" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1127">
       <c r="A1127" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1127" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1127" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A3675</t>
         </is>
       </c>
       <c r="D1127" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000013417703</t>
         </is>
       </c>
       <c r="E1127" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1127" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1128">
       <c r="A1128" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1128" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1128" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A7527</t>
         </is>
       </c>
       <c r="D1128" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000013417711</t>
         </is>
       </c>
       <c r="E1128" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1128" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1129">
       <c r="A1129" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1129" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1129" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A3674</t>
         </is>
       </c>
       <c r="D1129" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000013417720</t>
         </is>
       </c>
       <c r="E1129" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1129" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1130">
       <c r="A1130" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1130" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1130" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>A5377</t>
         </is>
       </c>
       <c r="D1130" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000013417738</t>
         </is>
       </c>
       <c r="E1130" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1130" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1131">
       <c r="A1131" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1131" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1131" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>TA0205</t>
         </is>
       </c>
       <c r="D1131" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000013417746</t>
         </is>
       </c>
       <c r="E1131" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1131" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1132">
       <c r="A1132" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557870</t>
         </is>
       </c>
       <c r="B1132" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1132" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>A1051</t>
         </is>
       </c>
       <c r="D1132" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000013417754</t>
         </is>
       </c>
       <c r="E1132" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:19</t>
         </is>
       </c>
       <c r="F1132" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1133">
       <c r="A1133" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1133" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1133" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D1133" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E1133" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1133" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1134" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1134" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D1134" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E1134" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1134" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1135" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1135" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D1135" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E1135" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1135" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>558604</t>
         </is>
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>TA0996</t>
         </is>
       </c>
       <c r="D1136" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000013336460</t>
         </is>
       </c>
       <c r="E1136" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1136" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 21:35</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>558604</t>
         </is>
       </c>
       <c r="B1137" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1137" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A2883</t>
         </is>
       </c>
       <c r="D1137" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000013336479</t>
         </is>
       </c>
       <c r="E1137" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1137" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 21:35</t>
         </is>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>558714</t>
         </is>
       </c>
       <c r="B1138" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1138" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A5902</t>
         </is>
       </c>
       <c r="D1138" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000013234994</t>
         </is>
       </c>
       <c r="E1138" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1138" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 21:39</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B1139" s="2" t="inlineStr">
@@ -36688,29 +36688,29 @@
       </c>
       <c r="C1139" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D1139" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E1139" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F1139" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1140" s="2" t="inlineStr">
@@ -36720,29 +36720,29 @@
       </c>
       <c r="C1140" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A0830</t>
         </is>
       </c>
       <c r="D1140" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000013211269</t>
         </is>
       </c>
       <c r="E1140" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1140" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1141" s="2" t="inlineStr">
@@ -36752,29 +36752,29 @@
       </c>
       <c r="C1141" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A0222</t>
         </is>
       </c>
       <c r="D1141" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000013211277</t>
         </is>
       </c>
       <c r="E1141" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1141" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1142" s="2" t="inlineStr">
@@ -36784,29 +36784,29 @@
       </c>
       <c r="C1142" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A8417</t>
         </is>
       </c>
       <c r="D1142" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000013211285</t>
         </is>
       </c>
       <c r="E1142" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1142" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1143" s="2" t="inlineStr">
@@ -36816,29 +36816,29 @@
       </c>
       <c r="C1143" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D1143" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E1143" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1143" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1144" s="2" t="inlineStr">
@@ -36848,29 +36848,29 @@
       </c>
       <c r="C1144" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D1144" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E1144" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1144" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1145" s="2" t="inlineStr">
@@ -36880,29 +36880,29 @@
       </c>
       <c r="C1145" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D1145" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E1145" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1145" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1146" s="2" t="inlineStr">
@@ -36912,29 +36912,29 @@
       </c>
       <c r="C1146" s="2" t="inlineStr">
         <is>
-          <t>A8196</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D1146" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728802</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E1146" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1146" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1147" s="2" t="inlineStr">
@@ -36944,29 +36944,29 @@
       </c>
       <c r="C1147" s="2" t="inlineStr">
         <is>
-          <t>A6374</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D1147" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419200</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E1147" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1147" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1148">
       <c r="A1148" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1148" s="2" t="inlineStr">
@@ -36976,29 +36976,29 @@
       </c>
       <c r="C1148" s="2" t="inlineStr">
         <is>
-          <t>A4452</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D1148" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419218</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E1148" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1148" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1149">
       <c r="A1149" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1149" s="2" t="inlineStr">
@@ -37008,29 +37008,29 @@
       </c>
       <c r="C1149" s="2" t="inlineStr">
         <is>
-          <t>A2241</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D1149" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419340</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E1149" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1149" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1150">
       <c r="A1150" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1150" s="2" t="inlineStr">
@@ -37040,59 +37040,571 @@
       </c>
       <c r="C1150" s="2" t="inlineStr">
         <is>
-          <t>A9562</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D1150" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419358</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E1150" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="F1150" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
     </row>
     <row r="1151">
       <c r="A1151" s="2" t="inlineStr">
         <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1151" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1151" s="2" t="inlineStr">
+        <is>
+          <t>A6758</t>
+        </is>
+      </c>
+      <c r="D1151" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730084</t>
+        </is>
+      </c>
+      <c r="E1151" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1151" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1152" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1152" s="2" t="inlineStr">
+        <is>
+          <t>A9095</t>
+        </is>
+      </c>
+      <c r="D1152" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730092</t>
+        </is>
+      </c>
+      <c r="E1152" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1152" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1153" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1153" s="2" t="inlineStr">
+        <is>
+          <t>A7630</t>
+        </is>
+      </c>
+      <c r="D1153" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730106</t>
+        </is>
+      </c>
+      <c r="E1153" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1153" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1154" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1154" s="2" t="inlineStr">
+        <is>
+          <t>A2166</t>
+        </is>
+      </c>
+      <c r="D1154" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730114</t>
+        </is>
+      </c>
+      <c r="E1154" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1154" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1155" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1155" s="2" t="inlineStr">
+        <is>
+          <t>A7031</t>
+        </is>
+      </c>
+      <c r="D1155" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730122</t>
+        </is>
+      </c>
+      <c r="E1155" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1155" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1156" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1156" s="2" t="inlineStr">
+        <is>
+          <t>A8477</t>
+        </is>
+      </c>
+      <c r="D1156" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730769</t>
+        </is>
+      </c>
+      <c r="E1156" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1156" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1157" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1157" s="2" t="inlineStr">
+        <is>
+          <t>A3086</t>
+        </is>
+      </c>
+      <c r="D1157" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730980</t>
+        </is>
+      </c>
+      <c r="E1157" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1157" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1158" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1158" s="2" t="inlineStr">
+        <is>
+          <t>A6151</t>
+        </is>
+      </c>
+      <c r="D1158" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728721</t>
+        </is>
+      </c>
+      <c r="E1158" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1158" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1159" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1159" s="2" t="inlineStr">
+        <is>
+          <t>A9532</t>
+        </is>
+      </c>
+      <c r="D1159" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728730</t>
+        </is>
+      </c>
+      <c r="E1159" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1159" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1160" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1160" s="2" t="inlineStr">
+        <is>
+          <t>A5035</t>
+        </is>
+      </c>
+      <c r="D1160" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728748</t>
+        </is>
+      </c>
+      <c r="E1160" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1160" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1161" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1161" s="2" t="inlineStr">
+        <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D1161" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E1161" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1161" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1162" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1162" s="2" t="inlineStr">
+        <is>
+          <t>A8196</t>
+        </is>
+      </c>
+      <c r="D1162" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728802</t>
+        </is>
+      </c>
+      <c r="E1162" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1162" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1163" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1163" s="2" t="inlineStr">
+        <is>
+          <t>A6374</t>
+        </is>
+      </c>
+      <c r="D1163" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419200</t>
+        </is>
+      </c>
+      <c r="E1163" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1163" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1164" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1164" s="2" t="inlineStr">
+        <is>
+          <t>A4452</t>
+        </is>
+      </c>
+      <c r="D1164" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419218</t>
+        </is>
+      </c>
+      <c r="E1164" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1164" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1165" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1165" s="2" t="inlineStr">
+        <is>
+          <t>A2241</t>
+        </is>
+      </c>
+      <c r="D1165" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419340</t>
+        </is>
+      </c>
+      <c r="E1165" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1165" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1166" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1166" s="2" t="inlineStr">
+        <is>
+          <t>A9562</t>
+        </is>
+      </c>
+      <c r="D1166" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419358</t>
+        </is>
+      </c>
+      <c r="E1166" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1166" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="2" t="inlineStr">
+        <is>
           <t>559975</t>
         </is>
       </c>
-      <c r="B1151" s="2" t="inlineStr">
+      <c r="B1167" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="C1151" s="2" t="inlineStr">
+      <c r="C1167" s="2" t="inlineStr">
         <is>
           <t>TA0880</t>
         </is>
       </c>
-      <c r="D1151" s="2" t="inlineStr">
+      <c r="D1167" s="2" t="inlineStr">
         <is>
           <t>00019200000013419242</t>
         </is>
       </c>
-      <c r="E1151" s="2" t="inlineStr">
+      <c r="E1167" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="F1151" s="2" t="inlineStr">
+      <c r="F1167" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1151"/>
+  <autoFilter ref="A1:F1167"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 01:00:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$1167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$F$1191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1167"/>
+  <dimension ref="A1:F1191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36486,967 +36486,967 @@
     <row r="1133">
       <c r="A1133" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1133" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1133" s="2" t="inlineStr">
         <is>
-          <t>TA0739</t>
+          <t>A4627</t>
         </is>
       </c>
       <c r="D1133" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721247</t>
+          <t>00019200000013207857</t>
         </is>
       </c>
       <c r="E1133" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1133" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1134" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1134" s="2" t="inlineStr">
         <is>
-          <t>A9099</t>
+          <t>A4476</t>
         </is>
       </c>
       <c r="D1134" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864250</t>
+          <t>00019200000013207865</t>
         </is>
       </c>
       <c r="E1134" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1134" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" s="2" t="inlineStr">
         <is>
-          <t>556176</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1135" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1135" s="2" t="inlineStr">
         <is>
-          <t>A8780</t>
+          <t>A5005</t>
         </is>
       </c>
       <c r="D1135" s="2" t="inlineStr">
         <is>
-          <t>00019200000012864269</t>
+          <t>00019200000013207873</t>
         </is>
       </c>
       <c r="E1135" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 01:17</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1135" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" s="2" t="inlineStr">
         <is>
-          <t>558604</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1136" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1136" s="2" t="inlineStr">
         <is>
-          <t>TA0996</t>
+          <t>A8822</t>
         </is>
       </c>
       <c r="D1136" s="2" t="inlineStr">
         <is>
-          <t>00019200000013336460</t>
+          <t>00019200000013418785</t>
         </is>
       </c>
       <c r="E1136" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1136" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:35</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" s="2" t="inlineStr">
         <is>
-          <t>558604</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1137" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1137" s="2" t="inlineStr">
         <is>
-          <t>A2883</t>
+          <t>A8991</t>
         </is>
       </c>
       <c r="D1137" s="2" t="inlineStr">
         <is>
-          <t>00019200000013336479</t>
+          <t>00019200000013418793</t>
         </is>
       </c>
       <c r="E1137" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1137" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:35</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" s="2" t="inlineStr">
         <is>
-          <t>558714</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1138" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1138" s="2" t="inlineStr">
         <is>
-          <t>A5902</t>
+          <t>A6628</t>
         </is>
       </c>
       <c r="D1138" s="2" t="inlineStr">
         <is>
-          <t>00019200000013234994</t>
+          <t>00019200000013418807</t>
         </is>
       </c>
       <c r="E1138" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 03:54</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1138" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 21:39</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1139" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1139" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A3065</t>
         </is>
       </c>
       <c r="D1139" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000013418815</t>
         </is>
       </c>
       <c r="E1139" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1139" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1140" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1140" s="2" t="inlineStr">
         <is>
-          <t>A0830</t>
+          <t>A6327</t>
         </is>
       </c>
       <c r="D1140" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211269</t>
+          <t>00019200000013418823</t>
         </is>
       </c>
       <c r="E1140" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1140" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1141" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1141" s="2" t="inlineStr">
         <is>
-          <t>A0222</t>
+          <t>TA1079</t>
         </is>
       </c>
       <c r="D1141" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211277</t>
+          <t>00019200000013418831</t>
         </is>
       </c>
       <c r="E1141" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1141" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1142" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1142" s="2" t="inlineStr">
         <is>
-          <t>A8417</t>
+          <t>A3193</t>
         </is>
       </c>
       <c r="D1142" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211285</t>
+          <t>00019200000013418840</t>
         </is>
       </c>
       <c r="E1142" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1142" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1143" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1143" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A2988</t>
         </is>
       </c>
       <c r="D1143" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000013418858</t>
         </is>
       </c>
       <c r="E1143" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1143" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1144" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1144" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A3580</t>
         </is>
       </c>
       <c r="D1144" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000013418866</t>
         </is>
       </c>
       <c r="E1144" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1144" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1145" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1145" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A4751</t>
         </is>
       </c>
       <c r="D1145" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000013418874</t>
         </is>
       </c>
       <c r="E1145" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1145" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1146" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1146" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>A9364</t>
         </is>
       </c>
       <c r="D1146" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000013418882</t>
         </is>
       </c>
       <c r="E1146" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1146" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1147" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1147" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A7329</t>
         </is>
       </c>
       <c r="D1147" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000013418890</t>
         </is>
       </c>
       <c r="E1147" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1147" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1148">
       <c r="A1148" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1148" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1148" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D1148" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000013418904</t>
         </is>
       </c>
       <c r="E1148" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1148" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1149">
       <c r="A1149" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1149" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1149" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A8335</t>
         </is>
       </c>
       <c r="D1149" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000013418912</t>
         </is>
       </c>
       <c r="E1149" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1149" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1150">
       <c r="A1150" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1150" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1150" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A8963</t>
         </is>
       </c>
       <c r="D1150" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000013418920</t>
         </is>
       </c>
       <c r="E1150" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1150" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1151">
       <c r="A1151" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1151" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1151" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A4520</t>
         </is>
       </c>
       <c r="D1151" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000013418939</t>
         </is>
       </c>
       <c r="E1151" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1151" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1152">
       <c r="A1152" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1152" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1152" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A1144</t>
         </is>
       </c>
       <c r="D1152" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000013418947</t>
         </is>
       </c>
       <c r="E1152" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1152" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1153">
       <c r="A1153" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1153" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1153" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A2621</t>
         </is>
       </c>
       <c r="D1153" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000013418955</t>
         </is>
       </c>
       <c r="E1153" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1153" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1154">
       <c r="A1154" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1154" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1154" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A8260</t>
         </is>
       </c>
       <c r="D1154" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000013418963</t>
         </is>
       </c>
       <c r="E1154" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1154" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1155">
       <c r="A1155" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1155" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1155" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A0322</t>
         </is>
       </c>
       <c r="D1155" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000013418971</t>
         </is>
       </c>
       <c r="E1155" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1155" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1156">
       <c r="A1156" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>557875</t>
         </is>
       </c>
       <c r="B1156" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C1156" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A8880</t>
         </is>
       </c>
       <c r="D1156" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000013418980</t>
         </is>
       </c>
       <c r="E1156" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>08/07/2026 00:40</t>
         </is>
       </c>
       <c r="F1156" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="1157">
       <c r="A1157" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1157" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1157" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>TA0739</t>
         </is>
       </c>
       <c r="D1157" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012721247</t>
         </is>
       </c>
       <c r="E1157" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1157" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1158">
       <c r="A1158" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1158" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1158" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A9099</t>
         </is>
       </c>
       <c r="D1158" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012864250</t>
         </is>
       </c>
       <c r="E1158" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1158" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1159">
       <c r="A1159" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556176</t>
         </is>
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A8780</t>
         </is>
       </c>
       <c r="D1159" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012864269</t>
         </is>
       </c>
       <c r="E1159" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>03/06/2026 01:17</t>
         </is>
       </c>
       <c r="F1159" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>03/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1160">
       <c r="A1160" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>558604</t>
         </is>
       </c>
       <c r="B1160" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1160" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>TA0996</t>
         </is>
       </c>
       <c r="D1160" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000013336460</t>
         </is>
       </c>
       <c r="E1160" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1160" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>23/06/2026 21:35</t>
         </is>
       </c>
     </row>
     <row r="1161">
       <c r="A1161" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>558604</t>
         </is>
       </c>
       <c r="B1161" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1161" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A2883</t>
         </is>
       </c>
       <c r="D1161" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000013336479</t>
         </is>
       </c>
       <c r="E1161" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1161" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>23/06/2026 21:35</t>
         </is>
       </c>
     </row>
     <row r="1162">
       <c r="A1162" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>558714</t>
         </is>
       </c>
       <c r="B1162" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1162" s="2" t="inlineStr">
         <is>
-          <t>A8196</t>
+          <t>A5902</t>
         </is>
       </c>
       <c r="D1162" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728802</t>
+          <t>00019200000013234994</t>
         </is>
       </c>
       <c r="E1162" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>23/06/2026 03:54</t>
         </is>
       </c>
       <c r="F1162" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>23/06/2026 21:39</t>
         </is>
       </c>
     </row>
     <row r="1163">
       <c r="A1163" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B1163" s="2" t="inlineStr">
@@ -37456,29 +37456,29 @@
       </c>
       <c r="C1163" s="2" t="inlineStr">
         <is>
-          <t>A6374</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D1163" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419200</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E1163" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="F1163" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
     </row>
     <row r="1164">
       <c r="A1164" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1164" s="2" t="inlineStr">
@@ -37488,29 +37488,29 @@
       </c>
       <c r="C1164" s="2" t="inlineStr">
         <is>
-          <t>A4452</t>
+          <t>A0830</t>
         </is>
       </c>
       <c r="D1164" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419218</t>
+          <t>00019200000013211269</t>
         </is>
       </c>
       <c r="E1164" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1164" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1165">
       <c r="A1165" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1165" s="2" t="inlineStr">
@@ -37520,29 +37520,29 @@
       </c>
       <c r="C1165" s="2" t="inlineStr">
         <is>
-          <t>A2241</t>
+          <t>A0222</t>
         </is>
       </c>
       <c r="D1165" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419340</t>
+          <t>00019200000013211277</t>
         </is>
       </c>
       <c r="E1165" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1165" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1166">
       <c r="A1166" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1166" s="2" t="inlineStr">
@@ -37552,59 +37552,827 @@
       </c>
       <c r="C1166" s="2" t="inlineStr">
         <is>
-          <t>A9562</t>
+          <t>A8417</t>
         </is>
       </c>
       <c r="D1166" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419358</t>
+          <t>00019200000013211285</t>
         </is>
       </c>
       <c r="E1166" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="F1166" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
     <row r="1167">
       <c r="A1167" s="2" t="inlineStr">
         <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1167" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1167" s="2" t="inlineStr">
+        <is>
+          <t>A6892</t>
+        </is>
+      </c>
+      <c r="D1167" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012729990</t>
+        </is>
+      </c>
+      <c r="E1167" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1167" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1168" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1168" s="2" t="inlineStr">
+        <is>
+          <t>A9466</t>
+        </is>
+      </c>
+      <c r="D1168" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730017</t>
+        </is>
+      </c>
+      <c r="E1168" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1168" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1169" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1169" s="2" t="inlineStr">
+        <is>
+          <t>TA0682</t>
+        </is>
+      </c>
+      <c r="D1169" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730025</t>
+        </is>
+      </c>
+      <c r="E1169" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1169" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1170" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1170" s="2" t="inlineStr">
+        <is>
+          <t>A1433</t>
+        </is>
+      </c>
+      <c r="D1170" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730033</t>
+        </is>
+      </c>
+      <c r="E1170" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1170" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1171" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1171" s="2" t="inlineStr">
+        <is>
+          <t>TA0977</t>
+        </is>
+      </c>
+      <c r="D1171" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730041</t>
+        </is>
+      </c>
+      <c r="E1171" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1171" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1172" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1172" s="2" t="inlineStr">
+        <is>
+          <t>A6225</t>
+        </is>
+      </c>
+      <c r="D1172" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730050</t>
+        </is>
+      </c>
+      <c r="E1172" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1172" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1173" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1173" s="2" t="inlineStr">
+        <is>
+          <t>A3875</t>
+        </is>
+      </c>
+      <c r="D1173" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730068</t>
+        </is>
+      </c>
+      <c r="E1173" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1173" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1174" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1174" s="2" t="inlineStr">
+        <is>
+          <t>A9643</t>
+        </is>
+      </c>
+      <c r="D1174" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730076</t>
+        </is>
+      </c>
+      <c r="E1174" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1174" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1175" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1175" s="2" t="inlineStr">
+        <is>
+          <t>A6758</t>
+        </is>
+      </c>
+      <c r="D1175" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730084</t>
+        </is>
+      </c>
+      <c r="E1175" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1175" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1176" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1176" s="2" t="inlineStr">
+        <is>
+          <t>A9095</t>
+        </is>
+      </c>
+      <c r="D1176" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730092</t>
+        </is>
+      </c>
+      <c r="E1176" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1176" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1177" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1177" s="2" t="inlineStr">
+        <is>
+          <t>A7630</t>
+        </is>
+      </c>
+      <c r="D1177" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730106</t>
+        </is>
+      </c>
+      <c r="E1177" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1177" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1178" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1178" s="2" t="inlineStr">
+        <is>
+          <t>A2166</t>
+        </is>
+      </c>
+      <c r="D1178" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730114</t>
+        </is>
+      </c>
+      <c r="E1178" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1178" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1179" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1179" s="2" t="inlineStr">
+        <is>
+          <t>A7031</t>
+        </is>
+      </c>
+      <c r="D1179" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730122</t>
+        </is>
+      </c>
+      <c r="E1179" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1179" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1180" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1180" s="2" t="inlineStr">
+        <is>
+          <t>A8477</t>
+        </is>
+      </c>
+      <c r="D1180" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730769</t>
+        </is>
+      </c>
+      <c r="E1180" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1180" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="2" t="inlineStr">
+        <is>
+          <t>556163</t>
+        </is>
+      </c>
+      <c r="B1181" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1181" s="2" t="inlineStr">
+        <is>
+          <t>A3086</t>
+        </is>
+      </c>
+      <c r="D1181" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012730980</t>
+        </is>
+      </c>
+      <c r="E1181" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026 05:01</t>
+        </is>
+      </c>
+      <c r="F1181" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1182" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1182" s="2" t="inlineStr">
+        <is>
+          <t>A6151</t>
+        </is>
+      </c>
+      <c r="D1182" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728721</t>
+        </is>
+      </c>
+      <c r="E1182" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1182" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1183" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1183" s="2" t="inlineStr">
+        <is>
+          <t>A9532</t>
+        </is>
+      </c>
+      <c r="D1183" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728730</t>
+        </is>
+      </c>
+      <c r="E1183" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1183" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1184" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1184" s="2" t="inlineStr">
+        <is>
+          <t>A5035</t>
+        </is>
+      </c>
+      <c r="D1184" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728748</t>
+        </is>
+      </c>
+      <c r="E1184" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1184" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1185" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1185" s="2" t="inlineStr">
+        <is>
+          <t>A6598</t>
+        </is>
+      </c>
+      <c r="D1185" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728756</t>
+        </is>
+      </c>
+      <c r="E1185" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1185" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="2" t="inlineStr">
+        <is>
+          <t>556236</t>
+        </is>
+      </c>
+      <c r="B1186" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1186" s="2" t="inlineStr">
+        <is>
+          <t>A8196</t>
+        </is>
+      </c>
+      <c r="D1186" s="2" t="inlineStr">
+        <is>
+          <t>00019200000012728802</t>
+        </is>
+      </c>
+      <c r="E1186" s="2" t="inlineStr">
+        <is>
+          <t>09/06/2026 02:06</t>
+        </is>
+      </c>
+      <c r="F1186" s="2" t="inlineStr">
+        <is>
+          <t>10/06/2026 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1187" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1187" s="2" t="inlineStr">
+        <is>
+          <t>A6374</t>
+        </is>
+      </c>
+      <c r="D1187" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419200</t>
+        </is>
+      </c>
+      <c r="E1187" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1187" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1188" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1188" s="2" t="inlineStr">
+        <is>
+          <t>A4452</t>
+        </is>
+      </c>
+      <c r="D1188" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419218</t>
+        </is>
+      </c>
+      <c r="E1188" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1188" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1189" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1189" s="2" t="inlineStr">
+        <is>
+          <t>A2241</t>
+        </is>
+      </c>
+      <c r="D1189" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419340</t>
+        </is>
+      </c>
+      <c r="E1189" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1189" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="2" t="inlineStr">
+        <is>
+          <t>559781</t>
+        </is>
+      </c>
+      <c r="B1190" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1190" s="2" t="inlineStr">
+        <is>
+          <t>A9562</t>
+        </is>
+      </c>
+      <c r="D1190" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013419358</t>
+        </is>
+      </c>
+      <c r="E1190" s="2" t="inlineStr">
+        <is>
+          <t>07/07/2026 01:13</t>
+        </is>
+      </c>
+      <c r="F1190" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="2" t="inlineStr">
+        <is>
           <t>559975</t>
         </is>
       </c>
-      <c r="B1167" s="2" t="inlineStr">
+      <c r="B1191" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="C1167" s="2" t="inlineStr">
+      <c r="C1191" s="2" t="inlineStr">
         <is>
           <t>TA0880</t>
         </is>
       </c>
-      <c r="D1167" s="2" t="inlineStr">
+      <c r="D1191" s="2" t="inlineStr">
         <is>
           <t>00019200000013419242</t>
         </is>
       </c>
-      <c r="E1167" s="2" t="inlineStr">
+      <c r="E1191" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="F1167" s="2" t="inlineStr">
+      <c r="F1191" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1167"/>
+  <autoFilter ref="A1:F1191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 10:31:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -43531,7 +43531,7 @@
       </c>
       <c r="F1355" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 10:23</t>
         </is>
       </c>
     </row>
@@ -43659,7 +43659,7 @@
       </c>
       <c r="F1359" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 10:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 16:21:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -29775,7 +29775,7 @@
       </c>
       <c r="F927" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 16:12</t>
         </is>
       </c>
     </row>
@@ -30063,7 +30063,7 @@
       </c>
       <c r="F936" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 10:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 16:51:22
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -44811,7 +44811,7 @@
       </c>
       <c r="F1397" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 16:40</t>
         </is>
       </c>
     </row>
@@ -44843,7 +44843,7 @@
       </c>
       <c r="F1398" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 16:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 17:31:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -29999,7 +29999,7 @@
       </c>
       <c r="F934" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 12:02</t>
         </is>
       </c>
     </row>
@@ -30031,7 +30031,7 @@
       </c>
       <c r="F935" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 12:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 17:41:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -33711,7 +33711,7 @@
       </c>
       <c r="F1050" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33743,7 +33743,7 @@
       </c>
       <c r="F1051" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33775,7 +33775,7 @@
       </c>
       <c r="F1052" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33807,7 +33807,7 @@
       </c>
       <c r="F1053" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33839,7 +33839,7 @@
       </c>
       <c r="F1054" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33871,7 +33871,7 @@
       </c>
       <c r="F1055" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33903,7 +33903,7 @@
       </c>
       <c r="F1056" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33935,7 +33935,7 @@
       </c>
       <c r="F1057" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33967,7 +33967,7 @@
       </c>
       <c r="F1058" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -33999,7 +33999,7 @@
       </c>
       <c r="F1059" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34031,7 +34031,7 @@
       </c>
       <c r="F1060" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34063,7 +34063,7 @@
       </c>
       <c r="F1061" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34095,7 +34095,7 @@
       </c>
       <c r="F1062" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34127,7 +34127,7 @@
       </c>
       <c r="F1063" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34159,7 +34159,7 @@
       </c>
       <c r="F1064" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>
@@ -34191,7 +34191,7 @@
       </c>
       <c r="F1065" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 17:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 18:21:12
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -26622,7 +26622,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C827" s="2" t="inlineStr"/>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>A6348</t>
+        </is>
+      </c>
       <c r="D827" s="2" t="inlineStr">
         <is>
           <t>00019200000013414070</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 19:11:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -23666,7 +23666,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C732" s="2" t="inlineStr"/>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>A0444</t>
+        </is>
+      </c>
       <c r="D732" s="2" t="inlineStr">
         <is>
           <t>00019200000013415484</t>
@@ -23694,7 +23698,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C733" s="2" t="inlineStr"/>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>A5955</t>
+        </is>
+      </c>
       <c r="D733" s="2" t="inlineStr">
         <is>
           <t>00019200000013415492</t>
@@ -23722,7 +23730,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C734" s="2" t="inlineStr"/>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>A6542</t>
+        </is>
+      </c>
       <c r="D734" s="2" t="inlineStr">
         <is>
           <t>00019200000013415506</t>
@@ -23750,7 +23762,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C735" s="2" t="inlineStr"/>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>A5877</t>
+        </is>
+      </c>
       <c r="D735" s="2" t="inlineStr">
         <is>
           <t>00019200000013415514</t>
@@ -23810,7 +23826,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C737" s="2" t="inlineStr"/>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>A7281</t>
+        </is>
+      </c>
       <c r="D737" s="2" t="inlineStr">
         <is>
           <t>00019200000013415549</t>
@@ -23838,7 +23858,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C738" s="2" t="inlineStr"/>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>A6492</t>
+        </is>
+      </c>
       <c r="D738" s="2" t="inlineStr">
         <is>
           <t>00019200000013415557</t>
@@ -23866,7 +23890,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C739" s="2" t="inlineStr"/>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>A8849</t>
+        </is>
+      </c>
       <c r="D739" s="2" t="inlineStr">
         <is>
           <t>00019200000013415565</t>
@@ -23894,7 +23922,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C740" s="2" t="inlineStr"/>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>A7760</t>
+        </is>
+      </c>
       <c r="D740" s="2" t="inlineStr">
         <is>
           <t>00019200000013415573</t>
@@ -23950,7 +23982,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C742" s="2" t="inlineStr"/>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>A9608</t>
+        </is>
+      </c>
       <c r="D742" s="2" t="inlineStr">
         <is>
           <t>00019200000013415590</t>
@@ -23978,7 +24014,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C743" s="2" t="inlineStr"/>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>A1458</t>
+        </is>
+      </c>
       <c r="D743" s="2" t="inlineStr">
         <is>
           <t>00019200000013415603</t>
@@ -24006,7 +24046,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C744" s="2" t="inlineStr"/>
+      <c r="C744" s="2" t="inlineStr">
+        <is>
+          <t>A6499</t>
+        </is>
+      </c>
       <c r="D744" s="2" t="inlineStr">
         <is>
           <t>00019200000013415611</t>
@@ -24062,7 +24106,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C746" s="2" t="inlineStr"/>
+      <c r="C746" s="2" t="inlineStr">
+        <is>
+          <t>TA0349</t>
+        </is>
+      </c>
       <c r="D746" s="2" t="inlineStr">
         <is>
           <t>00019200000013415638</t>
@@ -24118,7 +24166,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C748" s="2" t="inlineStr"/>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>A5677</t>
+        </is>
+      </c>
       <c r="D748" s="2" t="inlineStr">
         <is>
           <t>00019200000013415654</t>
@@ -24146,7 +24198,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C749" s="2" t="inlineStr"/>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>A4231</t>
+        </is>
+      </c>
       <c r="D749" s="2" t="inlineStr">
         <is>
           <t>00019200000013415662</t>
@@ -24358,7 +24414,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C756" s="2" t="inlineStr"/>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>A9267</t>
+        </is>
+      </c>
       <c r="D756" s="2" t="inlineStr">
         <is>
           <t>00019200000013415735</t>
@@ -24866,7 +24926,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C772" s="2" t="inlineStr"/>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>A1049</t>
+        </is>
+      </c>
       <c r="D772" s="2" t="inlineStr">
         <is>
           <t>00019200000013417320</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 19:21:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -23954,7 +23954,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C741" s="2" t="inlineStr"/>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>A8355</t>
+        </is>
+      </c>
       <c r="D741" s="2" t="inlineStr">
         <is>
           <t>00019200000013415581</t>
@@ -24078,7 +24082,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C745" s="2" t="inlineStr"/>
+      <c r="C745" s="2" t="inlineStr">
+        <is>
+          <t>A5992</t>
+        </is>
+      </c>
       <c r="D745" s="2" t="inlineStr">
         <is>
           <t>00019200000013415620</t>
@@ -24138,7 +24146,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C747" s="2" t="inlineStr"/>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>A5456</t>
+        </is>
+      </c>
       <c r="D747" s="2" t="inlineStr">
         <is>
           <t>00019200000013415646</t>
@@ -24230,7 +24242,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C750" s="2" t="inlineStr"/>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>A3633</t>
+        </is>
+      </c>
       <c r="D750" s="2" t="inlineStr">
         <is>
           <t>00019200000013415670</t>
@@ -24258,7 +24274,11 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="C751" s="2" t="inlineStr"/>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>A5271</t>
+        </is>
+      </c>
       <c r="D751" s="2" t="inlineStr">
         <is>
           <t>00019200000013415689</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 21:21:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -21526,7 +21526,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C662" s="2" t="inlineStr"/>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>A5686</t>
+        </is>
+      </c>
       <c r="D662" s="2" t="inlineStr">
         <is>
           <t>00019200000012925985</t>
@@ -22766,7 +22770,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C703" s="2" t="inlineStr"/>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>A9232</t>
+        </is>
+      </c>
       <c r="D703" s="2" t="inlineStr">
         <is>
           <t>00019200000013226320</t>
@@ -22850,7 +22858,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C706" s="2" t="inlineStr"/>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>A6035</t>
+        </is>
+      </c>
       <c r="D706" s="2" t="inlineStr">
         <is>
           <t>00019200000013226355</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 21:31:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -21122,7 +21122,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C648" s="2" t="inlineStr"/>
+      <c r="C648" s="2" t="inlineStr">
+        <is>
+          <t>A8569</t>
+        </is>
+      </c>
       <c r="D648" s="2" t="inlineStr">
         <is>
           <t>00019200000012923702</t>
@@ -21470,7 +21474,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C660" s="2" t="inlineStr"/>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>A0185</t>
+        </is>
+      </c>
       <c r="D660" s="2" t="inlineStr">
         <is>
           <t>00019200000012925969</t>
@@ -21526,11 +21534,7 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C662" s="2" t="inlineStr">
-        <is>
-          <t>A5686</t>
-        </is>
-      </c>
+      <c r="C662" s="2" t="inlineStr"/>
       <c r="D662" s="2" t="inlineStr">
         <is>
           <t>00019200000012925985</t>
@@ -21698,7 +21702,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C668" s="2" t="inlineStr"/>
+      <c r="C668" s="2" t="inlineStr">
+        <is>
+          <t>TA0971</t>
+        </is>
+      </c>
       <c r="D668" s="2" t="inlineStr">
         <is>
           <t>00019200000012926159</t>
@@ -21754,7 +21762,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C670" s="2" t="inlineStr"/>
+      <c r="C670" s="2" t="inlineStr">
+        <is>
+          <t>A0135</t>
+        </is>
+      </c>
       <c r="D670" s="2" t="inlineStr">
         <is>
           <t>00019200000012926175</t>
@@ -22742,7 +22754,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C702" s="2" t="inlineStr"/>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>A8185</t>
+        </is>
+      </c>
       <c r="D702" s="2" t="inlineStr">
         <is>
           <t>00019200000013226312</t>
@@ -22802,7 +22818,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C704" s="2" t="inlineStr"/>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>A9299</t>
+        </is>
+      </c>
       <c r="D704" s="2" t="inlineStr">
         <is>
           <t>00019200000013226339</t>
@@ -22830,7 +22850,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C705" s="2" t="inlineStr"/>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>A1768</t>
+        </is>
+      </c>
       <c r="D705" s="2" t="inlineStr">
         <is>
           <t>00019200000013226347</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 21:41:33
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -21326,7 +21326,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C655" s="2" t="inlineStr"/>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>A9577</t>
+        </is>
+      </c>
       <c r="D655" s="2" t="inlineStr">
         <is>
           <t>00019200000012925918</t>
@@ -21354,7 +21358,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C656" s="2" t="inlineStr"/>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t>A5524</t>
+        </is>
+      </c>
       <c r="D656" s="2" t="inlineStr">
         <is>
           <t>00019200000012925926</t>
@@ -21382,7 +21390,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C657" s="2" t="inlineStr"/>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>TA0409</t>
+        </is>
+      </c>
       <c r="D657" s="2" t="inlineStr">
         <is>
           <t>00019200000012925934</t>
@@ -21850,7 +21862,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C673" s="2" t="inlineStr"/>
+      <c r="C673" s="2" t="inlineStr">
+        <is>
+          <t>TA0598</t>
+        </is>
+      </c>
       <c r="D673" s="2" t="inlineStr">
         <is>
           <t>00019200000013210629</t>
@@ -22546,7 +22562,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C695" s="2" t="inlineStr"/>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>A6704</t>
+        </is>
+      </c>
       <c r="D695" s="2" t="inlineStr">
         <is>
           <t>00019200000013225880</t>
@@ -22574,7 +22594,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C696" s="2" t="inlineStr"/>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>A8921</t>
+        </is>
+      </c>
       <c r="D696" s="2" t="inlineStr">
         <is>
           <t>00019200000013225898</t>
@@ -22602,7 +22626,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C697" s="2" t="inlineStr"/>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>TA0509</t>
+        </is>
+      </c>
       <c r="D697" s="2" t="inlineStr">
         <is>
           <t>00019200000013225901</t>
@@ -22630,7 +22658,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C698" s="2" t="inlineStr"/>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>A1220</t>
+        </is>
+      </c>
       <c r="D698" s="2" t="inlineStr">
         <is>
           <t>00019200000013225910</t>
@@ -23330,7 +23362,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C720" s="2" t="inlineStr"/>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>A1969</t>
+        </is>
+      </c>
       <c r="D720" s="2" t="inlineStr">
         <is>
           <t>00019200000013243195</t>
@@ -23358,7 +23394,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C721" s="2" t="inlineStr"/>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>A9121</t>
+        </is>
+      </c>
       <c r="D721" s="2" t="inlineStr">
         <is>
           <t>00019200000013243209</t>
@@ -23386,7 +23426,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C722" s="2" t="inlineStr"/>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>A8466</t>
+        </is>
+      </c>
       <c r="D722" s="2" t="inlineStr">
         <is>
           <t>00019200000013243217</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 21:51:22
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -20826,7 +20826,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C638" s="2" t="inlineStr"/>
+      <c r="C638" s="2" t="inlineStr">
+        <is>
+          <t>A6161</t>
+        </is>
+      </c>
       <c r="D638" s="2" t="inlineStr">
         <is>
           <t>00019200000012696455</t>
@@ -20854,7 +20858,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C639" s="2" t="inlineStr"/>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
+          <t>A9234</t>
+        </is>
+      </c>
       <c r="D639" s="2" t="inlineStr">
         <is>
           <t>00019200000012696463</t>
@@ -20882,7 +20890,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C640" s="2" t="inlineStr"/>
+      <c r="C640" s="2" t="inlineStr">
+        <is>
+          <t>A6335</t>
+        </is>
+      </c>
       <c r="D640" s="2" t="inlineStr">
         <is>
           <t>00019200000012696471</t>
@@ -20910,7 +20922,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C641" s="2" t="inlineStr"/>
+      <c r="C641" s="2" t="inlineStr">
+        <is>
+          <t>A4784</t>
+        </is>
+      </c>
       <c r="D641" s="2" t="inlineStr">
         <is>
           <t>00019200000012920681</t>
@@ -20938,7 +20954,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C642" s="2" t="inlineStr"/>
+      <c r="C642" s="2" t="inlineStr">
+        <is>
+          <t>A2026</t>
+        </is>
+      </c>
       <c r="D642" s="2" t="inlineStr">
         <is>
           <t>00019200000012920690</t>
@@ -20966,7 +20986,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C643" s="2" t="inlineStr"/>
+      <c r="C643" s="2" t="inlineStr">
+        <is>
+          <t>A2158</t>
+        </is>
+      </c>
       <c r="D643" s="2" t="inlineStr">
         <is>
           <t>00019200000012920703</t>
@@ -21154,7 +21178,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C649" s="2" t="inlineStr"/>
+      <c r="C649" s="2" t="inlineStr">
+        <is>
+          <t>A8796</t>
+        </is>
+      </c>
       <c r="D649" s="2" t="inlineStr">
         <is>
           <t>00019200000012923710</t>
@@ -21182,7 +21210,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C650" s="2" t="inlineStr"/>
+      <c r="C650" s="2" t="inlineStr">
+        <is>
+          <t>A8042</t>
+        </is>
+      </c>
       <c r="D650" s="2" t="inlineStr">
         <is>
           <t>00019200000012923729</t>
@@ -21210,7 +21242,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C651" s="2" t="inlineStr"/>
+      <c r="C651" s="2" t="inlineStr">
+        <is>
+          <t>A4694</t>
+        </is>
+      </c>
       <c r="D651" s="2" t="inlineStr">
         <is>
           <t>00019200000012923737</t>
@@ -21238,7 +21274,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C652" s="2" t="inlineStr"/>
+      <c r="C652" s="2" t="inlineStr">
+        <is>
+          <t>A6775</t>
+        </is>
+      </c>
       <c r="D652" s="2" t="inlineStr">
         <is>
           <t>00019200000012923745</t>
@@ -21266,7 +21306,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C653" s="2" t="inlineStr"/>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>A7008</t>
+        </is>
+      </c>
       <c r="D653" s="2" t="inlineStr">
         <is>
           <t>00019200000012923753</t>
@@ -21518,7 +21562,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C661" s="2" t="inlineStr"/>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>TA0711</t>
+        </is>
+      </c>
       <c r="D661" s="2" t="inlineStr">
         <is>
           <t>00019200000012925977</t>
@@ -21574,7 +21622,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C663" s="2" t="inlineStr"/>
+      <c r="C663" s="2" t="inlineStr">
+        <is>
+          <t>A1510</t>
+        </is>
+      </c>
       <c r="D663" s="2" t="inlineStr">
         <is>
           <t>00019200000012925993</t>
@@ -21602,7 +21654,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C664" s="2" t="inlineStr"/>
+      <c r="C664" s="2" t="inlineStr">
+        <is>
+          <t>A3028</t>
+        </is>
+      </c>
       <c r="D664" s="2" t="inlineStr">
         <is>
           <t>00019200000012926116</t>
@@ -21630,7 +21686,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C665" s="2" t="inlineStr"/>
+      <c r="C665" s="2" t="inlineStr">
+        <is>
+          <t>A3302</t>
+        </is>
+      </c>
       <c r="D665" s="2" t="inlineStr">
         <is>
           <t>00019200000012926124</t>
@@ -21658,7 +21718,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C666" s="2" t="inlineStr"/>
+      <c r="C666" s="2" t="inlineStr">
+        <is>
+          <t>A2883</t>
+        </is>
+      </c>
       <c r="D666" s="2" t="inlineStr">
         <is>
           <t>00019200000012926132</t>
@@ -21686,7 +21750,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C667" s="2" t="inlineStr"/>
+      <c r="C667" s="2" t="inlineStr">
+        <is>
+          <t>A1275</t>
+        </is>
+      </c>
       <c r="D667" s="2" t="inlineStr">
         <is>
           <t>00019200000012926140</t>
@@ -21806,7 +21874,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C671" s="2" t="inlineStr"/>
+      <c r="C671" s="2" t="inlineStr">
+        <is>
+          <t>A9413</t>
+        </is>
+      </c>
       <c r="D671" s="2" t="inlineStr">
         <is>
           <t>00019200000013210602</t>
@@ -21834,7 +21906,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C672" s="2" t="inlineStr"/>
+      <c r="C672" s="2" t="inlineStr">
+        <is>
+          <t>A9032</t>
+        </is>
+      </c>
       <c r="D672" s="2" t="inlineStr">
         <is>
           <t>00019200000013210610</t>
@@ -27070,7 +27146,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C837" s="2" t="inlineStr"/>
+      <c r="C837" s="2" t="inlineStr">
+        <is>
+          <t>A4809</t>
+        </is>
+      </c>
       <c r="D837" s="2" t="inlineStr">
         <is>
           <t>00019200000013414178</t>
@@ -27098,7 +27178,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C838" s="2" t="inlineStr"/>
+      <c r="C838" s="2" t="inlineStr">
+        <is>
+          <t>TA0429</t>
+        </is>
+      </c>
       <c r="D838" s="2" t="inlineStr">
         <is>
           <t>00019200000013414186</t>
@@ -27126,7 +27210,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C839" s="2" t="inlineStr"/>
+      <c r="C839" s="2" t="inlineStr">
+        <is>
+          <t>A9603</t>
+        </is>
+      </c>
       <c r="D839" s="2" t="inlineStr">
         <is>
           <t>00019200000013414194</t>
@@ -27154,7 +27242,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C840" s="2" t="inlineStr"/>
+      <c r="C840" s="2" t="inlineStr">
+        <is>
+          <t>A7379</t>
+        </is>
+      </c>
       <c r="D840" s="2" t="inlineStr">
         <is>
           <t>00019200000013414208</t>
@@ -27182,7 +27274,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C841" s="2" t="inlineStr"/>
+      <c r="C841" s="2" t="inlineStr">
+        <is>
+          <t>A9080</t>
+        </is>
+      </c>
       <c r="D841" s="2" t="inlineStr">
         <is>
           <t>00019200000013414216</t>
@@ -27210,7 +27306,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C842" s="2" t="inlineStr"/>
+      <c r="C842" s="2" t="inlineStr">
+        <is>
+          <t>A7835</t>
+        </is>
+      </c>
       <c r="D842" s="2" t="inlineStr">
         <is>
           <t>00019200000013414224</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-08 22:01:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -21814,7 +21814,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C669" s="2" t="inlineStr"/>
+      <c r="C669" s="2" t="inlineStr">
+        <is>
+          <t>A6302</t>
+        </is>
+      </c>
       <c r="D669" s="2" t="inlineStr">
         <is>
           <t>00019200000012926167</t>
@@ -21970,7 +21974,11 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="C674" s="2" t="inlineStr"/>
+      <c r="C674" s="2" t="inlineStr">
+        <is>
+          <t>A8782</t>
+        </is>
+      </c>
       <c r="D674" s="2" t="inlineStr">
         <is>
           <t>00019200000013210637</t>
@@ -26894,7 +26902,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C828" s="2" t="inlineStr"/>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>A6433</t>
+        </is>
+      </c>
       <c r="D828" s="2" t="inlineStr">
         <is>
           <t>00019200000013414089</t>
@@ -26922,7 +26934,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C829" s="2" t="inlineStr"/>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>A8506</t>
+        </is>
+      </c>
       <c r="D829" s="2" t="inlineStr">
         <is>
           <t>00019200000013414097</t>
@@ -26950,7 +26966,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C830" s="2" t="inlineStr"/>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>A8122</t>
+        </is>
+      </c>
       <c r="D830" s="2" t="inlineStr">
         <is>
           <t>00019200000013414100</t>
@@ -26978,7 +26998,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C831" s="2" t="inlineStr"/>
+      <c r="C831" s="2" t="inlineStr">
+        <is>
+          <t>A3012</t>
+        </is>
+      </c>
       <c r="D831" s="2" t="inlineStr">
         <is>
           <t>00019200000013414119</t>
@@ -27006,7 +27030,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C832" s="2" t="inlineStr"/>
+      <c r="C832" s="2" t="inlineStr">
+        <is>
+          <t>TA1167</t>
+        </is>
+      </c>
       <c r="D832" s="2" t="inlineStr">
         <is>
           <t>00019200000013414127</t>
@@ -27034,7 +27062,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C833" s="2" t="inlineStr"/>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>A8631</t>
+        </is>
+      </c>
       <c r="D833" s="2" t="inlineStr">
         <is>
           <t>00019200000013414135</t>
@@ -27062,7 +27094,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C834" s="2" t="inlineStr"/>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>A9580</t>
+        </is>
+      </c>
       <c r="D834" s="2" t="inlineStr">
         <is>
           <t>00019200000013414143</t>
@@ -27090,7 +27126,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C835" s="2" t="inlineStr"/>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>A2643</t>
+        </is>
+      </c>
       <c r="D835" s="2" t="inlineStr">
         <is>
           <t>00019200000013414151</t>
@@ -27118,7 +27158,11 @@
           <t>PB</t>
         </is>
       </c>
-      <c r="C836" s="2" t="inlineStr"/>
+      <c r="C836" s="2" t="inlineStr">
+        <is>
+          <t>A4914</t>
+        </is>
+      </c>
       <c r="D836" s="2" t="inlineStr">
         <is>
           <t>00019200000013414160</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 09:53:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -52323,7 +52323,7 @@
       </c>
       <c r="F1629" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -52355,7 +52355,7 @@
       </c>
       <c r="F1630" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -52387,7 +52387,7 @@
       </c>
       <c r="F1631" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -52419,7 +52419,7 @@
       </c>
       <c r="F1632" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -52515,7 +52515,7 @@
       </c>
       <c r="F1635" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 11:03:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -7751,7 +7751,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -19843,7 +19843,7 @@
       </c>
       <c r="F611" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -19875,7 +19875,7 @@
       </c>
       <c r="F612" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -19907,7 +19907,7 @@
       </c>
       <c r="F613" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -22275,7 +22275,7 @@
       </c>
       <c r="F687" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 11:33:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -21347,7 +21347,7 @@
       </c>
       <c r="F658" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21379,7 +21379,7 @@
       </c>
       <c r="F659" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21411,7 +21411,7 @@
       </c>
       <c r="F660" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21443,7 +21443,7 @@
       </c>
       <c r="F661" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21475,7 +21475,7 @@
       </c>
       <c r="F662" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21507,7 +21507,7 @@
       </c>
       <c r="F663" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21539,7 +21539,7 @@
       </c>
       <c r="F664" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21571,7 +21571,7 @@
       </c>
       <c r="F665" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21603,7 +21603,7 @@
       </c>
       <c r="F666" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21635,7 +21635,7 @@
       </c>
       <c r="F667" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21667,7 +21667,7 @@
       </c>
       <c r="F668" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="F669" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21731,7 +21731,7 @@
       </c>
       <c r="F670" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21763,7 +21763,7 @@
       </c>
       <c r="F671" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21795,7 +21795,7 @@
       </c>
       <c r="F672" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21827,7 +21827,7 @@
       </c>
       <c r="F673" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21859,7 +21859,7 @@
       </c>
       <c r="F674" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21891,7 +21891,7 @@
       </c>
       <c r="F675" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21923,7 +21923,7 @@
       </c>
       <c r="F676" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21955,7 +21955,7 @@
       </c>
       <c r="F677" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -21987,7 +21987,7 @@
       </c>
       <c r="F678" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22019,7 +22019,7 @@
       </c>
       <c r="F679" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22051,7 +22051,7 @@
       </c>
       <c r="F680" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22083,7 +22083,7 @@
       </c>
       <c r="F681" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22115,7 +22115,7 @@
       </c>
       <c r="F682" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22147,7 +22147,7 @@
       </c>
       <c r="F683" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22179,7 +22179,7 @@
       </c>
       <c r="F684" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -22211,7 +22211,7 @@
       </c>
       <c r="F685" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -31331,7 +31331,7 @@
       </c>
       <c r="F970" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 11:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 13:22:52
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -45767,7 +45767,7 @@
       </c>
       <c r="F1424" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
     </row>
@@ -45799,7 +45799,7 @@
       </c>
       <c r="F1425" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 13:42:42
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -7783,7 +7783,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 12:00</t>
         </is>
       </c>
     </row>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 12:00</t>
         </is>
       </c>
     </row>
@@ -7847,7 +7847,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 12:00</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7879,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 12:00</t>
         </is>
       </c>
     </row>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 12:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 14:02:41
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -19043,7 +19043,7 @@
       </c>
       <c r="F586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -19075,7 +19075,7 @@
       </c>
       <c r="F587" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 17:12:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -14915,7 +14915,7 @@
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -53547,7 +53547,7 @@
       </c>
       <c r="I1135" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 17:52:51
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -32526,7 +32526,7 @@
       </c>
       <c r="G686" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 09:33</t>
         </is>
       </c>
       <c r="H686" s="2" t="inlineStr">
@@ -32536,7 +32536,7 @@
       </c>
       <c r="I686" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 09:33</t>
         </is>
       </c>
     </row>
@@ -39247,7 +39247,7 @@
       </c>
       <c r="G829" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H829" s="2" t="inlineStr">
@@ -39294,7 +39294,7 @@
       </c>
       <c r="G830" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H830" s="2" t="inlineStr">
@@ -39341,7 +39341,7 @@
       </c>
       <c r="G831" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H831" s="2" t="inlineStr">
@@ -39388,7 +39388,7 @@
       </c>
       <c r="G832" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H832" s="2" t="inlineStr">
@@ -39435,7 +39435,7 @@
       </c>
       <c r="G833" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H833" s="2" t="inlineStr">
@@ -39445,7 +39445,7 @@
       </c>
       <c r="I833" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -39482,7 +39482,7 @@
       </c>
       <c r="G834" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H834" s="2" t="inlineStr">
@@ -39529,7 +39529,7 @@
       </c>
       <c r="G835" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H835" s="2" t="inlineStr">
@@ -39576,7 +39576,7 @@
       </c>
       <c r="G836" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H836" s="2" t="inlineStr">
@@ -39623,7 +39623,7 @@
       </c>
       <c r="G837" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H837" s="2" t="inlineStr">
@@ -39670,7 +39670,7 @@
       </c>
       <c r="G838" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H838" s="2" t="inlineStr">
@@ -39717,7 +39717,7 @@
       </c>
       <c r="G839" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H839" s="2" t="inlineStr">
@@ -39764,7 +39764,7 @@
       </c>
       <c r="G840" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H840" s="2" t="inlineStr">
@@ -39811,7 +39811,7 @@
       </c>
       <c r="G841" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H841" s="2" t="inlineStr">
@@ -39858,7 +39858,7 @@
       </c>
       <c r="G842" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H842" s="2" t="inlineStr">
@@ -39905,7 +39905,7 @@
       </c>
       <c r="G843" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H843" s="2" t="inlineStr">
@@ -39952,7 +39952,7 @@
       </c>
       <c r="G844" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H844" s="2" t="inlineStr">
@@ -39999,7 +39999,7 @@
       </c>
       <c r="G845" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H845" s="2" t="inlineStr">
@@ -40046,7 +40046,7 @@
       </c>
       <c r="G846" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H846" s="2" t="inlineStr">
@@ -40093,7 +40093,7 @@
       </c>
       <c r="G847" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H847" s="2" t="inlineStr">
@@ -40140,7 +40140,7 @@
       </c>
       <c r="G848" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H848" s="2" t="inlineStr">
@@ -40187,7 +40187,7 @@
       </c>
       <c r="G849" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H849" s="2" t="inlineStr">
@@ -40197,7 +40197,7 @@
       </c>
       <c r="I849" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40234,7 +40234,7 @@
       </c>
       <c r="G850" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H850" s="2" t="inlineStr">
@@ -40244,7 +40244,7 @@
       </c>
       <c r="I850" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40281,7 +40281,7 @@
       </c>
       <c r="G851" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H851" s="2" t="inlineStr">
@@ -40291,7 +40291,7 @@
       </c>
       <c r="I851" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40328,7 +40328,7 @@
       </c>
       <c r="G852" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H852" s="2" t="inlineStr">
@@ -40338,7 +40338,7 @@
       </c>
       <c r="I852" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40375,7 +40375,7 @@
       </c>
       <c r="G853" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H853" s="2" t="inlineStr">
@@ -40422,7 +40422,7 @@
       </c>
       <c r="G854" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H854" s="2" t="inlineStr">
@@ -40432,7 +40432,7 @@
       </c>
       <c r="I854" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40469,7 +40469,7 @@
       </c>
       <c r="G855" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H855" s="2" t="inlineStr">
@@ -40479,7 +40479,7 @@
       </c>
       <c r="I855" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40516,7 +40516,7 @@
       </c>
       <c r="G856" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H856" s="2" t="inlineStr">
@@ -40526,7 +40526,7 @@
       </c>
       <c r="I856" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40563,7 +40563,7 @@
       </c>
       <c r="G857" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H857" s="2" t="inlineStr">
@@ -40573,7 +40573,7 @@
       </c>
       <c r="I857" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40610,7 +40610,7 @@
       </c>
       <c r="G858" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H858" s="2" t="inlineStr">
@@ -40620,7 +40620,7 @@
       </c>
       <c r="I858" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40657,7 +40657,7 @@
       </c>
       <c r="G859" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H859" s="2" t="inlineStr">
@@ -40667,7 +40667,7 @@
       </c>
       <c r="I859" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40704,7 +40704,7 @@
       </c>
       <c r="G860" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H860" s="2" t="inlineStr">
@@ -40714,7 +40714,7 @@
       </c>
       <c r="I860" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40751,7 +40751,7 @@
       </c>
       <c r="G861" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H861" s="2" t="inlineStr">
@@ -40761,7 +40761,7 @@
       </c>
       <c r="I861" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40798,7 +40798,7 @@
       </c>
       <c r="G862" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H862" s="2" t="inlineStr">
@@ -40808,7 +40808,7 @@
       </c>
       <c r="I862" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40845,7 +40845,7 @@
       </c>
       <c r="G863" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H863" s="2" t="inlineStr">
@@ -40855,7 +40855,7 @@
       </c>
       <c r="I863" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40892,7 +40892,7 @@
       </c>
       <c r="G864" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H864" s="2" t="inlineStr">
@@ -40902,7 +40902,7 @@
       </c>
       <c r="I864" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40939,7 +40939,7 @@
       </c>
       <c r="G865" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H865" s="2" t="inlineStr">
@@ -40949,7 +40949,7 @@
       </c>
       <c r="I865" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -40986,7 +40986,7 @@
       </c>
       <c r="G866" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H866" s="2" t="inlineStr">
@@ -40996,7 +40996,7 @@
       </c>
       <c r="I866" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -41033,7 +41033,7 @@
       </c>
       <c r="G867" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H867" s="2" t="inlineStr">
@@ -41043,7 +41043,7 @@
       </c>
       <c r="I867" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -41080,7 +41080,7 @@
       </c>
       <c r="G868" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H868" s="2" t="inlineStr">
@@ -41090,7 +41090,7 @@
       </c>
       <c r="I868" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -41127,7 +41127,7 @@
       </c>
       <c r="G869" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:00</t>
         </is>
       </c>
       <c r="H869" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 18:02:45
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -52080,7 +52080,7 @@
       </c>
       <c r="G1104" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1104" s="2" t="inlineStr">
@@ -52127,7 +52127,7 @@
       </c>
       <c r="G1105" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1105" s="2" t="inlineStr">
@@ -52174,7 +52174,7 @@
       </c>
       <c r="G1106" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1106" s="2" t="inlineStr">
@@ -52221,7 +52221,7 @@
       </c>
       <c r="G1107" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1107" s="2" t="inlineStr">
@@ -52268,7 +52268,7 @@
       </c>
       <c r="G1108" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1108" s="2" t="inlineStr">
@@ -52315,7 +52315,7 @@
       </c>
       <c r="G1109" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1109" s="2" t="inlineStr">
@@ -52362,7 +52362,7 @@
       </c>
       <c r="G1110" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1110" s="2" t="inlineStr">
@@ -52409,7 +52409,7 @@
       </c>
       <c r="G1111" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1111" s="2" t="inlineStr">
@@ -52456,7 +52456,7 @@
       </c>
       <c r="G1112" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1112" s="2" t="inlineStr">
@@ -52503,7 +52503,7 @@
       </c>
       <c r="G1113" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1113" s="2" t="inlineStr">
@@ -52550,7 +52550,7 @@
       </c>
       <c r="G1114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1114" s="2" t="inlineStr">
@@ -52597,7 +52597,7 @@
       </c>
       <c r="G1115" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1115" s="2" t="inlineStr">
@@ -52644,7 +52644,7 @@
       </c>
       <c r="G1116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
       <c r="H1116" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 18:12:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9265,7 +9265,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
@@ -9312,7 +9312,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -9359,7 +9359,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -9406,7 +9406,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -9453,7 +9453,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -9782,7 +9782,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -52090,7 +52090,7 @@
       </c>
       <c r="I1104" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52137,7 +52137,7 @@
       </c>
       <c r="I1105" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52184,7 +52184,7 @@
       </c>
       <c r="I1106" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52231,7 +52231,7 @@
       </c>
       <c r="I1107" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52278,7 +52278,7 @@
       </c>
       <c r="I1108" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52325,7 +52325,7 @@
       </c>
       <c r="I1109" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52372,7 +52372,7 @@
       </c>
       <c r="I1110" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52419,7 +52419,7 @@
       </c>
       <c r="I1111" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52466,7 +52466,7 @@
       </c>
       <c r="I1112" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52513,7 +52513,7 @@
       </c>
       <c r="I1113" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52560,7 +52560,7 @@
       </c>
       <c r="I1114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52607,7 +52607,7 @@
       </c>
       <c r="I1115" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>
@@ -52654,7 +52654,7 @@
       </c>
       <c r="I1116" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 18:22:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9275,7 +9275,7 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9463,7 +9463,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9557,7 +9557,7 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9604,7 +9604,7 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9651,7 +9651,7 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9745,7 +9745,7 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>
@@ -9792,7 +9792,7 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 23:13:11
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -51563,7 +51563,7 @@
       </c>
       <c r="G1093" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 17:36</t>
         </is>
       </c>
       <c r="H1093" s="2" t="inlineStr">
@@ -51798,7 +51798,7 @@
       </c>
       <c r="G1098" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1098" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-09 23:23:26
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -51573,7 +51573,7 @@
       </c>
       <c r="I1093" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 17:36</t>
         </is>
       </c>
     </row>
@@ -51808,7 +51808,7 @@
       </c>
       <c r="I1098" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 19:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 02:43:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$I$1648</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$I$1649</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1648"/>
+  <dimension ref="A1:I1649"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -76204,42 +76204,42 @@
     <row r="1618">
       <c r="A1618" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>560246</t>
         </is>
       </c>
       <c r="B1618" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1618" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8735</t>
         </is>
       </c>
       <c r="D1618" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000013410997</t>
         </is>
       </c>
       <c r="E1618" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="F1618" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>10/07/2026 02:29</t>
         </is>
       </c>
       <c r="G1618" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H1618" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 02:29</t>
         </is>
       </c>
       <c r="I1618" s="2" t="inlineStr">
@@ -76251,7 +76251,7 @@
     <row r="1619">
       <c r="A1619" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B1619" s="2" t="inlineStr">
@@ -76261,12 +76261,12 @@
       </c>
       <c r="C1619" s="2" t="inlineStr">
         <is>
-          <t>A0830</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D1619" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211269</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E1619" s="2" t="inlineStr">
@@ -76276,22 +76276,22 @@
       </c>
       <c r="F1619" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="G1619" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
       <c r="H1619" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I1619" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -76308,12 +76308,12 @@
       </c>
       <c r="C1620" s="2" t="inlineStr">
         <is>
-          <t>A0222</t>
+          <t>A0830</t>
         </is>
       </c>
       <c r="D1620" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211277</t>
+          <t>00019200000013211269</t>
         </is>
       </c>
       <c r="E1620" s="2" t="inlineStr">
@@ -76355,12 +76355,12 @@
       </c>
       <c r="C1621" s="2" t="inlineStr">
         <is>
-          <t>A8417</t>
+          <t>A0222</t>
         </is>
       </c>
       <c r="D1621" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211285</t>
+          <t>00019200000013211277</t>
         </is>
       </c>
       <c r="E1621" s="2" t="inlineStr">
@@ -76392,7 +76392,7 @@
     <row r="1622">
       <c r="A1622" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1622" s="2" t="inlineStr">
@@ -76402,12 +76402,12 @@
       </c>
       <c r="C1622" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A8417</t>
         </is>
       </c>
       <c r="D1622" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000013211285</t>
         </is>
       </c>
       <c r="E1622" s="2" t="inlineStr">
@@ -76417,22 +76417,22 @@
       </c>
       <c r="F1622" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="G1622" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
       <c r="H1622" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="I1622" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -76449,12 +76449,12 @@
       </c>
       <c r="C1623" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D1623" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E1623" s="2" t="inlineStr">
@@ -76496,12 +76496,12 @@
       </c>
       <c r="C1624" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D1624" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E1624" s="2" t="inlineStr">
@@ -76543,12 +76543,12 @@
       </c>
       <c r="C1625" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D1625" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E1625" s="2" t="inlineStr">
@@ -76590,12 +76590,12 @@
       </c>
       <c r="C1626" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D1626" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E1626" s="2" t="inlineStr">
@@ -76637,12 +76637,12 @@
       </c>
       <c r="C1627" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D1627" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E1627" s="2" t="inlineStr">
@@ -76684,12 +76684,12 @@
       </c>
       <c r="C1628" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D1628" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E1628" s="2" t="inlineStr">
@@ -76731,12 +76731,12 @@
       </c>
       <c r="C1629" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D1629" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E1629" s="2" t="inlineStr">
@@ -76778,12 +76778,12 @@
       </c>
       <c r="C1630" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D1630" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E1630" s="2" t="inlineStr">
@@ -76825,12 +76825,12 @@
       </c>
       <c r="C1631" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D1631" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E1631" s="2" t="inlineStr">
@@ -76872,12 +76872,12 @@
       </c>
       <c r="C1632" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D1632" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E1632" s="2" t="inlineStr">
@@ -76919,12 +76919,12 @@
       </c>
       <c r="C1633" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D1633" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E1633" s="2" t="inlineStr">
@@ -76966,12 +76966,12 @@
       </c>
       <c r="C1634" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D1634" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E1634" s="2" t="inlineStr">
@@ -77013,12 +77013,12 @@
       </c>
       <c r="C1635" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D1635" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E1635" s="2" t="inlineStr">
@@ -77060,12 +77060,12 @@
       </c>
       <c r="C1636" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D1636" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E1636" s="2" t="inlineStr">
@@ -77097,7 +77097,7 @@
     <row r="1637">
       <c r="A1637" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1637" s="2" t="inlineStr">
@@ -77107,12 +77107,12 @@
       </c>
       <c r="C1637" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D1637" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E1637" s="2" t="inlineStr">
@@ -77122,12 +77122,12 @@
       </c>
       <c r="F1637" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="G1637" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
       <c r="H1637" s="2" t="inlineStr">
@@ -77154,12 +77154,12 @@
       </c>
       <c r="C1638" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D1638" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E1638" s="2" t="inlineStr">
@@ -77201,12 +77201,12 @@
       </c>
       <c r="C1639" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D1639" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E1639" s="2" t="inlineStr">
@@ -77248,12 +77248,12 @@
       </c>
       <c r="C1640" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D1640" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E1640" s="2" t="inlineStr">
@@ -77295,12 +77295,12 @@
       </c>
       <c r="C1641" s="2" t="inlineStr">
         <is>
-          <t>A8196</t>
+          <t>A6598</t>
         </is>
       </c>
       <c r="D1641" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728802</t>
+          <t>00019200000012728756</t>
         </is>
       </c>
       <c r="E1641" s="2" t="inlineStr">
@@ -77332,7 +77332,7 @@
     <row r="1642">
       <c r="A1642" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556236</t>
         </is>
       </c>
       <c r="B1642" s="2" t="inlineStr">
@@ -77342,12 +77342,12 @@
       </c>
       <c r="C1642" s="2" t="inlineStr">
         <is>
-          <t>A6374</t>
+          <t>A8196</t>
         </is>
       </c>
       <c r="D1642" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419200</t>
+          <t>00019200000012728802</t>
         </is>
       </c>
       <c r="E1642" s="2" t="inlineStr">
@@ -77357,22 +77357,22 @@
       </c>
       <c r="F1642" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>09/06/2026 02:06</t>
         </is>
       </c>
       <c r="G1642" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
       <c r="H1642" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I1642" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -77389,12 +77389,12 @@
       </c>
       <c r="C1643" s="2" t="inlineStr">
         <is>
-          <t>A4452</t>
+          <t>A6374</t>
         </is>
       </c>
       <c r="D1643" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419218</t>
+          <t>00019200000013419200</t>
         </is>
       </c>
       <c r="E1643" s="2" t="inlineStr">
@@ -77436,12 +77436,12 @@
       </c>
       <c r="C1644" s="2" t="inlineStr">
         <is>
-          <t>A2241</t>
+          <t>A4452</t>
         </is>
       </c>
       <c r="D1644" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419340</t>
+          <t>00019200000013419218</t>
         </is>
       </c>
       <c r="E1644" s="2" t="inlineStr">
@@ -77483,12 +77483,12 @@
       </c>
       <c r="C1645" s="2" t="inlineStr">
         <is>
-          <t>A9562</t>
+          <t>A2241</t>
         </is>
       </c>
       <c r="D1645" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419358</t>
+          <t>00019200000013419340</t>
         </is>
       </c>
       <c r="E1645" s="2" t="inlineStr">
@@ -77520,7 +77520,7 @@
     <row r="1646">
       <c r="A1646" s="2" t="inlineStr">
         <is>
-          <t>559946</t>
+          <t>559781</t>
         </is>
       </c>
       <c r="B1646" s="2" t="inlineStr">
@@ -77530,12 +77530,12 @@
       </c>
       <c r="C1646" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A9562</t>
         </is>
       </c>
       <c r="D1646" s="2" t="inlineStr">
         <is>
-          <t>00019200000013414380</t>
+          <t>00019200000013419358</t>
         </is>
       </c>
       <c r="E1646" s="2" t="inlineStr">
@@ -77545,22 +77545,22 @@
       </c>
       <c r="F1646" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 00:41</t>
+          <t>07/07/2026 01:13</t>
         </is>
       </c>
       <c r="G1646" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="H1646" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 00:41</t>
+          <t>07/07/2026 01:13</t>
         </is>
       </c>
       <c r="I1646" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -77577,12 +77577,12 @@
       </c>
       <c r="C1647" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D1647" s="2" t="inlineStr">
         <is>
-          <t>00019200000013414399</t>
+          <t>00019200000013414380</t>
         </is>
       </c>
       <c r="E1647" s="2" t="inlineStr">
@@ -77614,52 +77614,99 @@
     <row r="1648">
       <c r="A1648" s="2" t="inlineStr">
         <is>
+          <t>559946</t>
+        </is>
+      </c>
+      <c r="B1648" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1648" s="2" t="inlineStr">
+        <is>
+          <t>A9207</t>
+        </is>
+      </c>
+      <c r="D1648" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013414399</t>
+        </is>
+      </c>
+      <c r="E1648" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="F1648" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 00:41</t>
+        </is>
+      </c>
+      <c r="G1648" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1648" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 00:41</t>
+        </is>
+      </c>
+      <c r="I1648" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="2" t="inlineStr">
+        <is>
           <t>559975</t>
         </is>
       </c>
-      <c r="B1648" s="2" t="inlineStr">
+      <c r="B1649" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="C1648" s="2" t="inlineStr">
+      <c r="C1649" s="2" t="inlineStr">
         <is>
           <t>TA0880</t>
         </is>
       </c>
-      <c r="D1648" s="2" t="inlineStr">
+      <c r="D1649" s="2" t="inlineStr">
         <is>
           <t>00019200000013419242</t>
         </is>
       </c>
-      <c r="E1648" s="2" t="inlineStr">
-        <is>
-          <t>MultiModal</t>
-        </is>
-      </c>
-      <c r="F1648" s="2" t="inlineStr">
+      <c r="E1649" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="F1649" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="G1648" s="2" t="inlineStr">
+      <c r="G1649" s="2" t="inlineStr">
         <is>
           <t>08/07/2026 18:00</t>
         </is>
       </c>
-      <c r="H1648" s="2" t="inlineStr">
+      <c r="H1649" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="I1648" s="2" t="inlineStr">
+      <c r="I1649" s="2" t="inlineStr">
         <is>
           <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1648"/>
+  <autoFilter ref="A1:I1649"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 03:53:13
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analítico" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$I$1649</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analítico'!$A$1:$I$1650</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1649"/>
+  <dimension ref="A1:I1650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -76204,7 +76204,7 @@
     <row r="1618">
       <c r="A1618" s="2" t="inlineStr">
         <is>
-          <t>560246</t>
+          <t>560241</t>
         </is>
       </c>
       <c r="B1618" s="2" t="inlineStr">
@@ -76214,12 +76214,12 @@
       </c>
       <c r="C1618" s="2" t="inlineStr">
         <is>
-          <t>A8735</t>
+          <t>TA0978</t>
         </is>
       </c>
       <c r="D1618" s="2" t="inlineStr">
         <is>
-          <t>00019200000013410997</t>
+          <t>00019200000013410431</t>
         </is>
       </c>
       <c r="E1618" s="2" t="inlineStr">
@@ -76229,7 +76229,7 @@
       </c>
       <c r="F1618" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 02:29</t>
+          <t>10/07/2026 03:41</t>
         </is>
       </c>
       <c r="G1618" s="2" t="inlineStr">
@@ -76239,7 +76239,7 @@
       </c>
       <c r="H1618" s="2" t="inlineStr">
         <is>
-          <t>10/07/2026 02:29</t>
+          <t>10/07/2026 03:41</t>
         </is>
       </c>
       <c r="I1618" s="2" t="inlineStr">
@@ -76251,42 +76251,42 @@
     <row r="1619">
       <c r="A1619" s="2" t="inlineStr">
         <is>
-          <t>555916</t>
+          <t>560246</t>
         </is>
       </c>
       <c r="B1619" s="2" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C1619" s="2" t="inlineStr">
         <is>
-          <t>A4580</t>
+          <t>A8735</t>
         </is>
       </c>
       <c r="D1619" s="2" t="inlineStr">
         <is>
-          <t>00019200000012721859</t>
+          <t>00019200000013410997</t>
         </is>
       </c>
       <c r="E1619" s="2" t="inlineStr">
         <is>
-          <t>MultiModal</t>
+          <t>Rodoviário</t>
         </is>
       </c>
       <c r="F1619" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026 22:21</t>
+          <t>10/07/2026 02:29</t>
         </is>
       </c>
       <c r="G1619" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:00</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H1619" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 02:29</t>
         </is>
       </c>
       <c r="I1619" s="2" t="inlineStr">
@@ -76298,7 +76298,7 @@
     <row r="1620">
       <c r="A1620" s="2" t="inlineStr">
         <is>
-          <t>556137</t>
+          <t>555916</t>
         </is>
       </c>
       <c r="B1620" s="2" t="inlineStr">
@@ -76308,12 +76308,12 @@
       </c>
       <c r="C1620" s="2" t="inlineStr">
         <is>
-          <t>A0830</t>
+          <t>A4580</t>
         </is>
       </c>
       <c r="D1620" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211269</t>
+          <t>00019200000012721859</t>
         </is>
       </c>
       <c r="E1620" s="2" t="inlineStr">
@@ -76323,22 +76323,22 @@
       </c>
       <c r="F1620" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>01/06/2026 22:21</t>
         </is>
       </c>
       <c r="G1620" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>03/06/2026 14:00</t>
         </is>
       </c>
       <c r="H1620" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026 06:03</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I1620" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026 11:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -76355,12 +76355,12 @@
       </c>
       <c r="C1621" s="2" t="inlineStr">
         <is>
-          <t>A0222</t>
+          <t>A0830</t>
         </is>
       </c>
       <c r="D1621" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211277</t>
+          <t>00019200000013211269</t>
         </is>
       </c>
       <c r="E1621" s="2" t="inlineStr">
@@ -76402,12 +76402,12 @@
       </c>
       <c r="C1622" s="2" t="inlineStr">
         <is>
-          <t>A8417</t>
+          <t>A0222</t>
         </is>
       </c>
       <c r="D1622" s="2" t="inlineStr">
         <is>
-          <t>00019200000013211285</t>
+          <t>00019200000013211277</t>
         </is>
       </c>
       <c r="E1622" s="2" t="inlineStr">
@@ -76439,7 +76439,7 @@
     <row r="1623">
       <c r="A1623" s="2" t="inlineStr">
         <is>
-          <t>556163</t>
+          <t>556137</t>
         </is>
       </c>
       <c r="B1623" s="2" t="inlineStr">
@@ -76449,12 +76449,12 @@
       </c>
       <c r="C1623" s="2" t="inlineStr">
         <is>
-          <t>A6892</t>
+          <t>A8417</t>
         </is>
       </c>
       <c r="D1623" s="2" t="inlineStr">
         <is>
-          <t>00019200000012729990</t>
+          <t>00019200000013211285</t>
         </is>
       </c>
       <c r="E1623" s="2" t="inlineStr">
@@ -76464,22 +76464,22 @@
       </c>
       <c r="F1623" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026 05:01</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="G1623" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 14:40</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
       <c r="H1623" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22/06/2026 06:03</t>
         </is>
       </c>
       <c r="I1623" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23/06/2026 11:00</t>
         </is>
       </c>
     </row>
@@ -76496,12 +76496,12 @@
       </c>
       <c r="C1624" s="2" t="inlineStr">
         <is>
-          <t>A9466</t>
+          <t>A6892</t>
         </is>
       </c>
       <c r="D1624" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730017</t>
+          <t>00019200000012729990</t>
         </is>
       </c>
       <c r="E1624" s="2" t="inlineStr">
@@ -76543,12 +76543,12 @@
       </c>
       <c r="C1625" s="2" t="inlineStr">
         <is>
-          <t>TA0682</t>
+          <t>A9466</t>
         </is>
       </c>
       <c r="D1625" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730025</t>
+          <t>00019200000012730017</t>
         </is>
       </c>
       <c r="E1625" s="2" t="inlineStr">
@@ -76590,12 +76590,12 @@
       </c>
       <c r="C1626" s="2" t="inlineStr">
         <is>
-          <t>A1433</t>
+          <t>TA0682</t>
         </is>
       </c>
       <c r="D1626" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730033</t>
+          <t>00019200000012730025</t>
         </is>
       </c>
       <c r="E1626" s="2" t="inlineStr">
@@ -76637,12 +76637,12 @@
       </c>
       <c r="C1627" s="2" t="inlineStr">
         <is>
-          <t>TA0977</t>
+          <t>A1433</t>
         </is>
       </c>
       <c r="D1627" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730041</t>
+          <t>00019200000012730033</t>
         </is>
       </c>
       <c r="E1627" s="2" t="inlineStr">
@@ -76684,12 +76684,12 @@
       </c>
       <c r="C1628" s="2" t="inlineStr">
         <is>
-          <t>A6225</t>
+          <t>TA0977</t>
         </is>
       </c>
       <c r="D1628" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730050</t>
+          <t>00019200000012730041</t>
         </is>
       </c>
       <c r="E1628" s="2" t="inlineStr">
@@ -76731,12 +76731,12 @@
       </c>
       <c r="C1629" s="2" t="inlineStr">
         <is>
-          <t>A3875</t>
+          <t>A6225</t>
         </is>
       </c>
       <c r="D1629" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730068</t>
+          <t>00019200000012730050</t>
         </is>
       </c>
       <c r="E1629" s="2" t="inlineStr">
@@ -76778,12 +76778,12 @@
       </c>
       <c r="C1630" s="2" t="inlineStr">
         <is>
-          <t>A9643</t>
+          <t>A3875</t>
         </is>
       </c>
       <c r="D1630" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730076</t>
+          <t>00019200000012730068</t>
         </is>
       </c>
       <c r="E1630" s="2" t="inlineStr">
@@ -76825,12 +76825,12 @@
       </c>
       <c r="C1631" s="2" t="inlineStr">
         <is>
-          <t>A6758</t>
+          <t>A9643</t>
         </is>
       </c>
       <c r="D1631" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730084</t>
+          <t>00019200000012730076</t>
         </is>
       </c>
       <c r="E1631" s="2" t="inlineStr">
@@ -76872,12 +76872,12 @@
       </c>
       <c r="C1632" s="2" t="inlineStr">
         <is>
-          <t>A9095</t>
+          <t>A6758</t>
         </is>
       </c>
       <c r="D1632" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730092</t>
+          <t>00019200000012730084</t>
         </is>
       </c>
       <c r="E1632" s="2" t="inlineStr">
@@ -76919,12 +76919,12 @@
       </c>
       <c r="C1633" s="2" t="inlineStr">
         <is>
-          <t>A7630</t>
+          <t>A9095</t>
         </is>
       </c>
       <c r="D1633" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730106</t>
+          <t>00019200000012730092</t>
         </is>
       </c>
       <c r="E1633" s="2" t="inlineStr">
@@ -76966,12 +76966,12 @@
       </c>
       <c r="C1634" s="2" t="inlineStr">
         <is>
-          <t>A2166</t>
+          <t>A7630</t>
         </is>
       </c>
       <c r="D1634" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730114</t>
+          <t>00019200000012730106</t>
         </is>
       </c>
       <c r="E1634" s="2" t="inlineStr">
@@ -77013,12 +77013,12 @@
       </c>
       <c r="C1635" s="2" t="inlineStr">
         <is>
-          <t>A7031</t>
+          <t>A2166</t>
         </is>
       </c>
       <c r="D1635" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730122</t>
+          <t>00019200000012730114</t>
         </is>
       </c>
       <c r="E1635" s="2" t="inlineStr">
@@ -77060,12 +77060,12 @@
       </c>
       <c r="C1636" s="2" t="inlineStr">
         <is>
-          <t>A8477</t>
+          <t>A7031</t>
         </is>
       </c>
       <c r="D1636" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730769</t>
+          <t>00019200000012730122</t>
         </is>
       </c>
       <c r="E1636" s="2" t="inlineStr">
@@ -77107,12 +77107,12 @@
       </c>
       <c r="C1637" s="2" t="inlineStr">
         <is>
-          <t>A3086</t>
+          <t>A8477</t>
         </is>
       </c>
       <c r="D1637" s="2" t="inlineStr">
         <is>
-          <t>00019200000012730980</t>
+          <t>00019200000012730769</t>
         </is>
       </c>
       <c r="E1637" s="2" t="inlineStr">
@@ -77144,7 +77144,7 @@
     <row r="1638">
       <c r="A1638" s="2" t="inlineStr">
         <is>
-          <t>556236</t>
+          <t>556163</t>
         </is>
       </c>
       <c r="B1638" s="2" t="inlineStr">
@@ -77154,12 +77154,12 @@
       </c>
       <c r="C1638" s="2" t="inlineStr">
         <is>
-          <t>A6151</t>
+          <t>A3086</t>
         </is>
       </c>
       <c r="D1638" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728721</t>
+          <t>00019200000012730980</t>
         </is>
       </c>
       <c r="E1638" s="2" t="inlineStr">
@@ -77169,12 +77169,12 @@
       </c>
       <c r="F1638" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026 02:06</t>
+          <t>06/06/2026 05:01</t>
         </is>
       </c>
       <c r="G1638" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026 11:00</t>
+          <t>09/06/2026 14:40</t>
         </is>
       </c>
       <c r="H1638" s="2" t="inlineStr">
@@ -77201,12 +77201,12 @@
       </c>
       <c r="C1639" s="2" t="inlineStr">
         <is>
-          <t>A9532</t>
+          <t>A6151</t>
         </is>
       </c>
       <c r="D1639" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728730</t>
+          <t>00019200000012728721</t>
         </is>
       </c>
       <c r="E1639" s="2" t="inlineStr">
@@ -77248,12 +77248,12 @@
       </c>
       <c r="C1640" s="2" t="inlineStr">
         <is>
-          <t>A5035</t>
+          <t>A9532</t>
         </is>
       </c>
       <c r="D1640" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728748</t>
+          <t>00019200000012728730</t>
         </is>
       </c>
       <c r="E1640" s="2" t="inlineStr">
@@ -77295,12 +77295,12 @@
       </c>
       <c r="C1641" s="2" t="inlineStr">
         <is>
-          <t>A6598</t>
+          <t>A5035</t>
         </is>
       </c>
       <c r="D1641" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728756</t>
+          <t>00019200000012728748</t>
         </is>
       </c>
       <c r="E1641" s="2" t="inlineStr">
@@ -77342,12 +77342,12 @@
       </c>
       <c r="C1642" s="2" t="inlineStr">
         <is>
-          <t>A8196</t>
+          <t>A6598</t>
         </is>
       </c>
       <c r="D1642" s="2" t="inlineStr">
         <is>
-          <t>00019200000012728802</t>
+          <t>00019200000012728756</t>
         </is>
       </c>
       <c r="E1642" s="2" t="inlineStr">
@@ -77379,7 +77379,7 @@
     <row r="1643">
       <c r="A1643" s="2" t="inlineStr">
         <is>
-          <t>559781</t>
+          <t>556236</t>
         </is>
       </c>
       <c r="B1643" s="2" t="inlineStr">
@@ -77389,12 +77389,12 @@
       </c>
       <c r="C1643" s="2" t="inlineStr">
         <is>
-          <t>A6374</t>
+          <t>A8196</t>
         </is>
       </c>
       <c r="D1643" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419200</t>
+          <t>00019200000012728802</t>
         </is>
       </c>
       <c r="E1643" s="2" t="inlineStr">
@@ -77404,22 +77404,22 @@
       </c>
       <c r="F1643" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>09/06/2026 02:06</t>
         </is>
       </c>
       <c r="G1643" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>10/06/2026 11:00</t>
         </is>
       </c>
       <c r="H1643" s="2" t="inlineStr">
         <is>
-          <t>07/07/2026 01:13</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I1643" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 18:00</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -77436,12 +77436,12 @@
       </c>
       <c r="C1644" s="2" t="inlineStr">
         <is>
-          <t>A4452</t>
+          <t>A6374</t>
         </is>
       </c>
       <c r="D1644" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419218</t>
+          <t>00019200000013419200</t>
         </is>
       </c>
       <c r="E1644" s="2" t="inlineStr">
@@ -77483,12 +77483,12 @@
       </c>
       <c r="C1645" s="2" t="inlineStr">
         <is>
-          <t>A2241</t>
+          <t>A4452</t>
         </is>
       </c>
       <c r="D1645" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419340</t>
+          <t>00019200000013419218</t>
         </is>
       </c>
       <c r="E1645" s="2" t="inlineStr">
@@ -77530,12 +77530,12 @@
       </c>
       <c r="C1646" s="2" t="inlineStr">
         <is>
-          <t>A9562</t>
+          <t>A2241</t>
         </is>
       </c>
       <c r="D1646" s="2" t="inlineStr">
         <is>
-          <t>00019200000013419358</t>
+          <t>00019200000013419340</t>
         </is>
       </c>
       <c r="E1646" s="2" t="inlineStr">
@@ -77567,7 +77567,7 @@
     <row r="1647">
       <c r="A1647" s="2" t="inlineStr">
         <is>
-          <t>559946</t>
+          <t>559781</t>
         </is>
       </c>
       <c r="B1647" s="2" t="inlineStr">
@@ -77577,12 +77577,12 @@
       </c>
       <c r="C1647" s="2" t="inlineStr">
         <is>
-          <t>A9230</t>
+          <t>A9562</t>
         </is>
       </c>
       <c r="D1647" s="2" t="inlineStr">
         <is>
-          <t>00019200000013414380</t>
+          <t>00019200000013419358</t>
         </is>
       </c>
       <c r="E1647" s="2" t="inlineStr">
@@ -77592,22 +77592,22 @@
       </c>
       <c r="F1647" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 00:41</t>
+          <t>07/07/2026 01:13</t>
         </is>
       </c>
       <c r="G1647" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="H1647" s="2" t="inlineStr">
         <is>
-          <t>08/07/2026 00:41</t>
+          <t>07/07/2026 01:13</t>
         </is>
       </c>
       <c r="I1647" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -77624,12 +77624,12 @@
       </c>
       <c r="C1648" s="2" t="inlineStr">
         <is>
-          <t>A9207</t>
+          <t>A9230</t>
         </is>
       </c>
       <c r="D1648" s="2" t="inlineStr">
         <is>
-          <t>00019200000013414399</t>
+          <t>00019200000013414380</t>
         </is>
       </c>
       <c r="E1648" s="2" t="inlineStr">
@@ -77661,52 +77661,99 @@
     <row r="1649">
       <c r="A1649" s="2" t="inlineStr">
         <is>
+          <t>559946</t>
+        </is>
+      </c>
+      <c r="B1649" s="2" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C1649" s="2" t="inlineStr">
+        <is>
+          <t>A9207</t>
+        </is>
+      </c>
+      <c r="D1649" s="2" t="inlineStr">
+        <is>
+          <t>00019200000013414399</t>
+        </is>
+      </c>
+      <c r="E1649" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="F1649" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 00:41</t>
+        </is>
+      </c>
+      <c r="G1649" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1649" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 00:41</t>
+        </is>
+      </c>
+      <c r="I1649" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="2" t="inlineStr">
+        <is>
           <t>559975</t>
         </is>
       </c>
-      <c r="B1649" s="2" t="inlineStr">
+      <c r="B1650" s="2" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="C1649" s="2" t="inlineStr">
+      <c r="C1650" s="2" t="inlineStr">
         <is>
           <t>TA0880</t>
         </is>
       </c>
-      <c r="D1649" s="2" t="inlineStr">
+      <c r="D1650" s="2" t="inlineStr">
         <is>
           <t>00019200000013419242</t>
         </is>
       </c>
-      <c r="E1649" s="2" t="inlineStr">
-        <is>
-          <t>MultiModal</t>
-        </is>
-      </c>
-      <c r="F1649" s="2" t="inlineStr">
+      <c r="E1650" s="2" t="inlineStr">
+        <is>
+          <t>MultiModal</t>
+        </is>
+      </c>
+      <c r="F1650" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="G1649" s="2" t="inlineStr">
+      <c r="G1650" s="2" t="inlineStr">
         <is>
           <t>08/07/2026 18:00</t>
         </is>
       </c>
-      <c r="H1649" s="2" t="inlineStr">
+      <c r="H1650" s="2" t="inlineStr">
         <is>
           <t>07/07/2026 00:59</t>
         </is>
       </c>
-      <c r="I1649" s="2" t="inlineStr">
+      <c r="I1650" s="2" t="inlineStr">
         <is>
           <t>08/07/2026 18:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1649"/>
+  <autoFilter ref="A1:I1650"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 08:34:10
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -77644,7 +77644,7 @@
       </c>
       <c r="G1648" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 18:00</t>
         </is>
       </c>
       <c r="H1648" s="2" t="inlineStr">
@@ -77691,7 +77691,7 @@
       </c>
       <c r="G1649" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 18:00</t>
         </is>
       </c>
       <c r="H1649" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 08:43:44
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -77654,7 +77654,7 @@
       </c>
       <c r="I1648" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 18:00</t>
         </is>
       </c>
     </row>
@@ -77701,7 +77701,7 @@
       </c>
       <c r="I1649" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 18:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 09:06:37
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -73884,7 +73884,7 @@
       </c>
       <c r="G1568" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1568" s="2" t="inlineStr">
@@ -73931,7 +73931,7 @@
       </c>
       <c r="G1569" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1569" s="2" t="inlineStr">
@@ -73978,7 +73978,7 @@
       </c>
       <c r="G1570" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1570" s="2" t="inlineStr">
@@ -74025,7 +74025,7 @@
       </c>
       <c r="G1571" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1571" s="2" t="inlineStr">
@@ -74072,7 +74072,7 @@
       </c>
       <c r="G1572" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1572" s="2" t="inlineStr">
@@ -74119,7 +74119,7 @@
       </c>
       <c r="G1573" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1573" s="2" t="inlineStr">
@@ -74166,7 +74166,7 @@
       </c>
       <c r="G1574" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1574" s="2" t="inlineStr">
@@ -74213,7 +74213,7 @@
       </c>
       <c r="G1575" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1575" s="2" t="inlineStr">
@@ -74260,7 +74260,7 @@
       </c>
       <c r="G1576" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1576" s="2" t="inlineStr">
@@ -74307,7 +74307,7 @@
       </c>
       <c r="G1577" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1577" s="2" t="inlineStr">
@@ -74354,7 +74354,7 @@
       </c>
       <c r="G1578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1578" s="2" t="inlineStr">
@@ -74401,7 +74401,7 @@
       </c>
       <c r="G1579" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1579" s="2" t="inlineStr">
@@ -74448,7 +74448,7 @@
       </c>
       <c r="G1580" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1580" s="2" t="inlineStr">
@@ -74495,7 +74495,7 @@
       </c>
       <c r="G1581" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1581" s="2" t="inlineStr">
@@ -74542,7 +74542,7 @@
       </c>
       <c r="G1582" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1582" s="2" t="inlineStr">
@@ -74589,7 +74589,7 @@
       </c>
       <c r="G1583" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1583" s="2" t="inlineStr">
@@ -74636,7 +74636,7 @@
       </c>
       <c r="G1584" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1584" s="2" t="inlineStr">
@@ -74683,7 +74683,7 @@
       </c>
       <c r="G1585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1585" s="2" t="inlineStr">
@@ -74730,7 +74730,7 @@
       </c>
       <c r="G1586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1586" s="2" t="inlineStr">
@@ -74777,7 +74777,7 @@
       </c>
       <c r="G1587" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1587" s="2" t="inlineStr">
@@ -74824,7 +74824,7 @@
       </c>
       <c r="G1588" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1588" s="2" t="inlineStr">
@@ -74871,7 +74871,7 @@
       </c>
       <c r="G1589" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1589" s="2" t="inlineStr">
@@ -74918,7 +74918,7 @@
       </c>
       <c r="G1590" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1590" s="2" t="inlineStr">
@@ -74965,7 +74965,7 @@
       </c>
       <c r="G1591" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
       <c r="H1591" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 09:15:22
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -73894,7 +73894,7 @@
       </c>
       <c r="I1568" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -73941,7 +73941,7 @@
       </c>
       <c r="I1569" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -73988,7 +73988,7 @@
       </c>
       <c r="I1570" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74035,7 +74035,7 @@
       </c>
       <c r="I1571" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74082,7 +74082,7 @@
       </c>
       <c r="I1572" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74129,7 +74129,7 @@
       </c>
       <c r="I1573" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74176,7 +74176,7 @@
       </c>
       <c r="I1574" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74223,7 +74223,7 @@
       </c>
       <c r="I1575" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74270,7 +74270,7 @@
       </c>
       <c r="I1576" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74317,7 +74317,7 @@
       </c>
       <c r="I1577" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74364,7 +74364,7 @@
       </c>
       <c r="I1578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74411,7 +74411,7 @@
       </c>
       <c r="I1579" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74458,7 +74458,7 @@
       </c>
       <c r="I1580" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74505,7 +74505,7 @@
       </c>
       <c r="I1581" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74552,7 +74552,7 @@
       </c>
       <c r="I1582" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74599,7 +74599,7 @@
       </c>
       <c r="I1583" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74646,7 +74646,7 @@
       </c>
       <c r="I1584" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74693,7 +74693,7 @@
       </c>
       <c r="I1585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74740,7 +74740,7 @@
       </c>
       <c r="I1586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74787,7 +74787,7 @@
       </c>
       <c r="I1587" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74834,7 +74834,7 @@
       </c>
       <c r="I1588" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74881,7 +74881,7 @@
       </c>
       <c r="I1589" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74928,7 +74928,7 @@
       </c>
       <c r="I1590" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -74975,7 +74975,7 @@
       </c>
       <c r="I1591" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 10:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 10:14:14
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -71393,7 +71393,7 @@
       </c>
       <c r="G1515" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 09:59</t>
         </is>
       </c>
       <c r="H1515" s="2" t="inlineStr">
@@ -71403,7 +71403,7 @@
       </c>
       <c r="I1515" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 09:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 10:24:38
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -27450,7 +27450,7 @@
       </c>
       <c r="G578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 16:00</t>
         </is>
       </c>
       <c r="H578" s="2" t="inlineStr">
@@ -27460,7 +27460,7 @@
       </c>
       <c r="I578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 16:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 10:35:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -8325,7 +8325,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr">
@@ -8560,7 +8560,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 10:45:46
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -8335,7 +8335,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8382,7 +8382,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8523,7 +8523,7 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8570,7 +8570,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -8617,7 +8617,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 13:10</t>
         </is>
       </c>
     </row>
@@ -27732,7 +27732,7 @@
       </c>
       <c r="G584" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:29</t>
         </is>
       </c>
       <c r="H584" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 11:15:34
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -27638,7 +27638,7 @@
       </c>
       <c r="G582" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:02</t>
         </is>
       </c>
       <c r="H582" s="2" t="inlineStr">
@@ -27826,7 +27826,7 @@
       </c>
       <c r="G586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:03</t>
         </is>
       </c>
       <c r="H586" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 11:25:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -16268,7 +16268,7 @@
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
       <c r="H340" s="2" t="inlineStr">
@@ -16278,7 +16278,7 @@
       </c>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
     </row>
@@ -16315,7 +16315,7 @@
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
       <c r="H341" s="2" t="inlineStr">
@@ -16325,7 +16325,7 @@
       </c>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
     </row>
@@ -16362,7 +16362,7 @@
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
       <c r="H342" s="2" t="inlineStr">
@@ -16372,7 +16372,7 @@
       </c>
       <c r="I342" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
     </row>
@@ -16409,7 +16409,7 @@
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
       <c r="H343" s="2" t="inlineStr">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
     </row>
@@ -16456,7 +16456,7 @@
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
       <c r="H344" s="2" t="inlineStr">
@@ -16466,7 +16466,7 @@
       </c>
       <c r="I344" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:10</t>
         </is>
       </c>
     </row>
@@ -16503,7 +16503,7 @@
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
       <c r="H345" s="2" t="inlineStr">
@@ -16513,7 +16513,7 @@
       </c>
       <c r="I345" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
     </row>
@@ -16550,7 +16550,7 @@
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
       <c r="H346" s="2" t="inlineStr">
@@ -16560,7 +16560,7 @@
       </c>
       <c r="I346" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
     </row>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
       <c r="H347" s="2" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="I347" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:24</t>
         </is>
       </c>
     </row>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="I582" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:02</t>
         </is>
       </c>
     </row>
@@ -27836,7 +27836,7 @@
       </c>
       <c r="I586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:03</t>
         </is>
       </c>
     </row>
@@ -41221,7 +41221,7 @@
       </c>
       <c r="G871" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H871" s="2" t="inlineStr">
@@ -41268,7 +41268,7 @@
       </c>
       <c r="G872" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H872" s="2" t="inlineStr">
@@ -41315,7 +41315,7 @@
       </c>
       <c r="G873" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H873" s="2" t="inlineStr">
@@ -41362,7 +41362,7 @@
       </c>
       <c r="G874" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H874" s="2" t="inlineStr">
@@ -41409,7 +41409,7 @@
       </c>
       <c r="G875" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H875" s="2" t="inlineStr">
@@ -41456,7 +41456,7 @@
       </c>
       <c r="G876" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H876" s="2" t="inlineStr">
@@ -41503,7 +41503,7 @@
       </c>
       <c r="G877" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H877" s="2" t="inlineStr">
@@ -41550,7 +41550,7 @@
       </c>
       <c r="G878" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H878" s="2" t="inlineStr">
@@ -41597,7 +41597,7 @@
       </c>
       <c r="G879" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
       <c r="H879" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 11:45:26
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -41231,7 +41231,7 @@
       </c>
       <c r="I871" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41278,7 +41278,7 @@
       </c>
       <c r="I872" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41325,7 +41325,7 @@
       </c>
       <c r="I873" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41372,7 +41372,7 @@
       </c>
       <c r="I874" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41419,7 +41419,7 @@
       </c>
       <c r="I875" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41466,7 +41466,7 @@
       </c>
       <c r="I876" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41513,7 +41513,7 @@
       </c>
       <c r="I877" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41560,7 +41560,7 @@
       </c>
       <c r="I878" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>
@@ -41607,7 +41607,7 @@
       </c>
       <c r="I879" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 12:05:35
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -11568,7 +11568,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:37</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr">
@@ -33372,7 +33372,7 @@
       </c>
       <c r="G704" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 16:00</t>
         </is>
       </c>
       <c r="H704" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 12:14:39
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -11578,7 +11578,7 @@
       </c>
       <c r="I240" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:37</t>
         </is>
       </c>
     </row>
@@ -33382,7 +33382,7 @@
       </c>
       <c r="I704" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 16:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 13:24:41
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -28024,7 +28024,7 @@
       </c>
       <c r="I590" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -46485,7 +46485,7 @@
       </c>
       <c r="G983" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:57</t>
         </is>
       </c>
       <c r="H983" s="2" t="inlineStr">
@@ -46495,7 +46495,7 @@
       </c>
       <c r="I983" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:57</t>
         </is>
       </c>
     </row>
@@ -50482,7 +50482,7 @@
       </c>
       <c r="G1070" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1070" s="2" t="inlineStr">
@@ -50492,7 +50492,7 @@
       </c>
       <c r="I1070" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50529,7 +50529,7 @@
       </c>
       <c r="G1071" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1071" s="2" t="inlineStr">
@@ -50539,7 +50539,7 @@
       </c>
       <c r="I1071" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50576,7 +50576,7 @@
       </c>
       <c r="G1072" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1072" s="2" t="inlineStr">
@@ -50586,7 +50586,7 @@
       </c>
       <c r="I1072" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50623,7 +50623,7 @@
       </c>
       <c r="G1073" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1073" s="2" t="inlineStr">
@@ -50633,7 +50633,7 @@
       </c>
       <c r="I1073" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50670,7 +50670,7 @@
       </c>
       <c r="G1074" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1074" s="2" t="inlineStr">
@@ -50680,7 +50680,7 @@
       </c>
       <c r="I1074" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50717,7 +50717,7 @@
       </c>
       <c r="G1075" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1075" s="2" t="inlineStr">
@@ -50727,7 +50727,7 @@
       </c>
       <c r="I1075" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50764,7 +50764,7 @@
       </c>
       <c r="G1076" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1076" s="2" t="inlineStr">
@@ -50774,7 +50774,7 @@
       </c>
       <c r="I1076" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -50811,7 +50811,7 @@
       </c>
       <c r="G1077" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
       <c r="H1077" s="2" t="inlineStr">
@@ -50821,7 +50821,7 @@
       </c>
       <c r="I1077" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:30</t>
         </is>
       </c>
     </row>
@@ -76281,7 +76281,7 @@
       </c>
       <c r="G1619" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:50</t>
         </is>
       </c>
       <c r="H1619" s="2" t="inlineStr">
@@ -76291,7 +76291,7 @@
       </c>
       <c r="I1619" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 13:44:24
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -32667,7 +32667,7 @@
       </c>
       <c r="G689" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H689" s="2" t="inlineStr">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="G690" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H690" s="2" t="inlineStr">
@@ -32761,7 +32761,7 @@
       </c>
       <c r="G691" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H691" s="2" t="inlineStr">
@@ -32808,7 +32808,7 @@
       </c>
       <c r="G692" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H692" s="2" t="inlineStr">
@@ -32855,7 +32855,7 @@
       </c>
       <c r="G693" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H693" s="2" t="inlineStr">
@@ -32902,7 +32902,7 @@
       </c>
       <c r="G694" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H694" s="2" t="inlineStr">
@@ -32949,7 +32949,7 @@
       </c>
       <c r="G695" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H695" s="2" t="inlineStr">
@@ -32996,7 +32996,7 @@
       </c>
       <c r="G696" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H696" s="2" t="inlineStr">
@@ -33043,7 +33043,7 @@
       </c>
       <c r="G697" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H697" s="2" t="inlineStr">
@@ -33090,7 +33090,7 @@
       </c>
       <c r="G698" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H698" s="2" t="inlineStr">
@@ -33137,7 +33137,7 @@
       </c>
       <c r="G699" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H699" s="2" t="inlineStr">
@@ -33184,7 +33184,7 @@
       </c>
       <c r="G700" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H700" s="2" t="inlineStr">
@@ -33231,7 +33231,7 @@
       </c>
       <c r="G701" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H701" s="2" t="inlineStr">
@@ -33278,7 +33278,7 @@
       </c>
       <c r="G702" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H702" s="2" t="inlineStr">
@@ -33325,7 +33325,7 @@
       </c>
       <c r="G703" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
       <c r="H703" s="2" t="inlineStr">
@@ -39304,7 +39304,7 @@
       </c>
       <c r="I830" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39351,7 +39351,7 @@
       </c>
       <c r="I831" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39398,7 +39398,7 @@
       </c>
       <c r="I832" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39445,7 +39445,7 @@
       </c>
       <c r="I833" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39539,7 +39539,7 @@
       </c>
       <c r="I835" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39586,7 +39586,7 @@
       </c>
       <c r="I836" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39633,7 +39633,7 @@
       </c>
       <c r="I837" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39680,7 +39680,7 @@
       </c>
       <c r="I838" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39727,7 +39727,7 @@
       </c>
       <c r="I839" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39774,7 +39774,7 @@
       </c>
       <c r="I840" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39821,7 +39821,7 @@
       </c>
       <c r="I841" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39868,7 +39868,7 @@
       </c>
       <c r="I842" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39915,7 +39915,7 @@
       </c>
       <c r="I843" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -39962,7 +39962,7 @@
       </c>
       <c r="I844" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40009,7 +40009,7 @@
       </c>
       <c r="I845" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40056,7 +40056,7 @@
       </c>
       <c r="I846" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40103,7 +40103,7 @@
       </c>
       <c r="I847" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40150,7 +40150,7 @@
       </c>
       <c r="I848" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40197,7 +40197,7 @@
       </c>
       <c r="I849" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -40432,7 +40432,7 @@
       </c>
       <c r="I854" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>
@@ -41184,7 +41184,7 @@
       </c>
       <c r="I870" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 13:54:19
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -32677,7 +32677,7 @@
       </c>
       <c r="I689" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32724,7 +32724,7 @@
       </c>
       <c r="I690" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32771,7 +32771,7 @@
       </c>
       <c r="I691" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32818,7 +32818,7 @@
       </c>
       <c r="I692" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32865,7 +32865,7 @@
       </c>
       <c r="I693" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32912,7 +32912,7 @@
       </c>
       <c r="I694" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -32959,7 +32959,7 @@
       </c>
       <c r="I695" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33006,7 +33006,7 @@
       </c>
       <c r="I696" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33053,7 +33053,7 @@
       </c>
       <c r="I697" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33100,7 +33100,7 @@
       </c>
       <c r="I698" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33147,7 +33147,7 @@
       </c>
       <c r="I699" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33194,7 +33194,7 @@
       </c>
       <c r="I700" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33241,7 +33241,7 @@
       </c>
       <c r="I701" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33288,7 +33288,7 @@
       </c>
       <c r="I702" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -33335,7 +33335,7 @@
       </c>
       <c r="I703" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>09/07/2026 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 14:24:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -23412,7 +23412,7 @@
       </c>
       <c r="G492" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:17</t>
         </is>
       </c>
       <c r="H492" s="2" t="inlineStr">
@@ -23459,7 +23459,7 @@
       </c>
       <c r="G493" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:17</t>
         </is>
       </c>
       <c r="H493" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 14:44:25
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -23422,7 +23422,7 @@
       </c>
       <c r="I492" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:17</t>
         </is>
       </c>
     </row>
@@ -23469,7 +23469,7 @@
       </c>
       <c r="I493" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 14:54:16
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -18665,7 +18665,7 @@
       </c>
       <c r="G391" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H391" s="2" t="inlineStr">
@@ -18675,7 +18675,7 @@
       </c>
       <c r="I391" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18712,7 +18712,7 @@
       </c>
       <c r="G392" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H392" s="2" t="inlineStr">
@@ -18722,7 +18722,7 @@
       </c>
       <c r="I392" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18759,7 +18759,7 @@
       </c>
       <c r="G393" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H393" s="2" t="inlineStr">
@@ -18769,7 +18769,7 @@
       </c>
       <c r="I393" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18806,7 +18806,7 @@
       </c>
       <c r="G394" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H394" s="2" t="inlineStr">
@@ -18816,7 +18816,7 @@
       </c>
       <c r="I394" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18853,7 +18853,7 @@
       </c>
       <c r="G395" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H395" s="2" t="inlineStr">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="I395" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18900,7 +18900,7 @@
       </c>
       <c r="G396" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H396" s="2" t="inlineStr">
@@ -18910,7 +18910,7 @@
       </c>
       <c r="I396" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18947,7 +18947,7 @@
       </c>
       <c r="G397" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H397" s="2" t="inlineStr">
@@ -18957,7 +18957,7 @@
       </c>
       <c r="I397" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -18994,7 +18994,7 @@
       </c>
       <c r="G398" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H398" s="2" t="inlineStr">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="I398" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -19041,7 +19041,7 @@
       </c>
       <c r="G399" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H399" s="2" t="inlineStr">
@@ -19051,7 +19051,7 @@
       </c>
       <c r="I399" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -19088,7 +19088,7 @@
       </c>
       <c r="G400" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H400" s="2" t="inlineStr">
@@ -19098,7 +19098,7 @@
       </c>
       <c r="I400" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -19135,7 +19135,7 @@
       </c>
       <c r="G401" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H401" s="2" t="inlineStr">
@@ -19145,7 +19145,7 @@
       </c>
       <c r="I401" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="G495" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:45</t>
         </is>
       </c>
       <c r="H495" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 15:24:57
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -46532,7 +46532,7 @@
       </c>
       <c r="G984" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:08</t>
         </is>
       </c>
       <c r="H984" s="2" t="inlineStr">
@@ -46542,7 +46542,7 @@
       </c>
       <c r="I984" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 16:06:29
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9829,7 +9829,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -9876,7 +9876,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
@@ -9923,7 +9923,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -9970,7 +9970,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -23271,7 +23271,7 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
@@ -23318,7 +23318,7 @@
       </c>
       <c r="G490" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
       <c r="H490" s="2" t="inlineStr">
@@ -23365,7 +23365,7 @@
       </c>
       <c r="G491" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
       <c r="H491" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 16:16:20
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -10017,7 +10017,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:06</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:06</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
@@ -50435,7 +50435,7 @@
       </c>
       <c r="G1069" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
       <c r="H1069" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 16:25:29
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -9839,7 +9839,7 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
     </row>
@@ -9886,7 +9886,7 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
     </row>
@@ -9933,7 +9933,7 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 11:35</t>
         </is>
       </c>
     </row>
@@ -10027,7 +10027,7 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:06</t>
         </is>
       </c>
     </row>
@@ -10074,7 +10074,7 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:06</t>
         </is>
       </c>
     </row>
@@ -12226,7 +12226,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr">
@@ -12273,7 +12273,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr">
@@ -12320,7 +12320,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr">
@@ -12367,7 +12367,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr">
@@ -12414,7 +12414,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
@@ -12461,7 +12461,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
@@ -12555,7 +12555,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr">
@@ -12696,7 +12696,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr">
@@ -12790,7 +12790,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
@@ -12884,7 +12884,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
@@ -12931,7 +12931,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr">
@@ -12978,7 +12978,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr">
@@ -13025,7 +13025,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr">
@@ -13260,7 +13260,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr">
@@ -13354,7 +13354,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr">
@@ -13448,7 +13448,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr">
@@ -13542,7 +13542,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr">
@@ -13552,7 +13552,7 @@
       </c>
       <c r="I282" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -13589,7 +13589,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr">
@@ -13599,7 +13599,7 @@
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -13636,7 +13636,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr">
@@ -13683,7 +13683,7 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr">
@@ -13693,7 +13693,7 @@
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -13730,7 +13730,7 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr">
@@ -13777,7 +13777,7 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="I288" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -13871,7 +13871,7 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H289" s="2" t="inlineStr">
@@ -13918,7 +13918,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr">
@@ -13928,7 +13928,7 @@
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13965,7 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr">
@@ -13975,7 +13975,7 @@
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14012,7 +14012,7 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14059,7 +14059,7 @@
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H293" s="2" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14106,7 +14106,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H295" s="2" t="inlineStr">
@@ -14163,7 +14163,7 @@
       </c>
       <c r="I295" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14200,7 +14200,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr">
@@ -14210,7 +14210,7 @@
       </c>
       <c r="I296" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14247,7 +14247,7 @@
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H297" s="2" t="inlineStr">
@@ -14257,7 +14257,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14294,7 +14294,7 @@
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H298" s="2" t="inlineStr">
@@ -14341,7 +14341,7 @@
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H299" s="2" t="inlineStr">
@@ -14351,7 +14351,7 @@
       </c>
       <c r="I299" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14388,7 +14388,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
@@ -14398,7 +14398,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr">
@@ -14482,7 +14482,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H302" s="2" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="I302" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14529,7 +14529,7 @@
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H303" s="2" t="inlineStr">
@@ -14576,7 +14576,7 @@
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H304" s="2" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H305" s="2" t="inlineStr">
@@ -14670,7 +14670,7 @@
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H306" s="2" t="inlineStr">
@@ -14680,7 +14680,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14717,7 +14717,7 @@
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H307" s="2" t="inlineStr">
@@ -14727,7 +14727,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14764,7 +14764,7 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
@@ -14774,7 +14774,7 @@
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14811,7 +14811,7 @@
       </c>
       <c r="G309" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H309" s="2" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -14858,7 +14858,7 @@
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:00</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
@@ -16644,7 +16644,7 @@
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 16:10</t>
         </is>
       </c>
       <c r="H348" s="2" t="inlineStr">
@@ -16654,7 +16654,7 @@
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 16:10</t>
         </is>
       </c>
     </row>
@@ -23281,7 +23281,7 @@
       </c>
       <c r="I489" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
     </row>
@@ -23328,7 +23328,7 @@
       </c>
       <c r="I490" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
     </row>
@@ -23375,7 +23375,7 @@
       </c>
       <c r="I491" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:51</t>
         </is>
       </c>
     </row>
@@ -50445,7 +50445,7 @@
       </c>
       <c r="I1069" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 17:54:44
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -52879,7 +52879,7 @@
       </c>
       <c r="G1121" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:33</t>
         </is>
       </c>
       <c r="H1121" s="2" t="inlineStr">
@@ -52889,7 +52889,7 @@
       </c>
       <c r="I1121" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 12:33</t>
         </is>
       </c>
     </row>
@@ -52926,7 +52926,7 @@
       </c>
       <c r="G1122" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1122" s="2" t="inlineStr">
@@ -52973,7 +52973,7 @@
       </c>
       <c r="G1123" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1123" s="2" t="inlineStr">
@@ -53020,7 +53020,7 @@
       </c>
       <c r="G1124" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1124" s="2" t="inlineStr">
@@ -53067,7 +53067,7 @@
       </c>
       <c r="G1125" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1125" s="2" t="inlineStr">
@@ -53114,7 +53114,7 @@
       </c>
       <c r="G1126" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1126" s="2" t="inlineStr">
@@ -53161,7 +53161,7 @@
       </c>
       <c r="G1127" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1127" s="2" t="inlineStr">
@@ -53208,7 +53208,7 @@
       </c>
       <c r="G1128" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1128" s="2" t="inlineStr">
@@ -53255,7 +53255,7 @@
       </c>
       <c r="G1129" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1129" s="2" t="inlineStr">
@@ -53302,7 +53302,7 @@
       </c>
       <c r="G1130" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1130" s="2" t="inlineStr">
@@ -53349,7 +53349,7 @@
       </c>
       <c r="G1131" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1131" s="2" t="inlineStr">
@@ -53396,7 +53396,7 @@
       </c>
       <c r="G1132" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1132" s="2" t="inlineStr">
@@ -53443,7 +53443,7 @@
       </c>
       <c r="G1133" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1133" s="2" t="inlineStr">
@@ -53490,7 +53490,7 @@
       </c>
       <c r="G1134" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1134" s="2" t="inlineStr">
@@ -53537,7 +53537,7 @@
       </c>
       <c r="G1135" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1135" s="2" t="inlineStr">
@@ -53584,7 +53584,7 @@
       </c>
       <c r="G1136" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1136" s="2" t="inlineStr">
@@ -53631,7 +53631,7 @@
       </c>
       <c r="G1137" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1137" s="2" t="inlineStr">
@@ -53678,7 +53678,7 @@
       </c>
       <c r="G1138" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
       <c r="H1138" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 18:15:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -52936,7 +52936,7 @@
       </c>
       <c r="I1122" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -52983,7 +52983,7 @@
       </c>
       <c r="I1123" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53030,7 +53030,7 @@
       </c>
       <c r="I1124" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53077,7 +53077,7 @@
       </c>
       <c r="I1125" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53124,7 +53124,7 @@
       </c>
       <c r="I1126" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53171,7 +53171,7 @@
       </c>
       <c r="I1127" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53218,7 +53218,7 @@
       </c>
       <c r="I1128" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53265,7 +53265,7 @@
       </c>
       <c r="I1129" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53312,7 +53312,7 @@
       </c>
       <c r="I1130" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53359,7 +53359,7 @@
       </c>
       <c r="I1131" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53406,7 +53406,7 @@
       </c>
       <c r="I1132" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53453,7 +53453,7 @@
       </c>
       <c r="I1133" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53500,7 +53500,7 @@
       </c>
       <c r="I1134" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53547,7 +53547,7 @@
       </c>
       <c r="I1135" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53594,7 +53594,7 @@
       </c>
       <c r="I1136" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53641,7 +53641,7 @@
       </c>
       <c r="I1137" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -53688,7 +53688,7 @@
       </c>
       <c r="I1138" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 13:30</t>
         </is>
       </c>
     </row>
@@ -54101,7 +54101,7 @@
       </c>
       <c r="G1147" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 16:56</t>
         </is>
       </c>
       <c r="H1147" s="2" t="inlineStr">
@@ -54111,7 +54111,7 @@
       </c>
       <c r="I1147" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 16:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 18:34:26
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -44981,7 +44981,7 @@
       </c>
       <c r="G951" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
       <c r="H951" s="2" t="inlineStr">
@@ -45028,7 +45028,7 @@
       </c>
       <c r="G952" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
       <c r="H952" s="2" t="inlineStr">
@@ -45075,7 +45075,7 @@
       </c>
       <c r="G953" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
       <c r="H953" s="2" t="inlineStr">
@@ -45122,7 +45122,7 @@
       </c>
       <c r="G954" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
       <c r="H954" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 18:44:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -44991,7 +44991,7 @@
       </c>
       <c r="I951" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
     </row>
@@ -45038,7 +45038,7 @@
       </c>
       <c r="I952" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
     </row>
@@ -45085,7 +45085,7 @@
       </c>
       <c r="I953" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
     </row>
@@ -45132,7 +45132,7 @@
       </c>
       <c r="I954" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 14:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 20:15:27
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -75012,7 +75012,7 @@
       </c>
       <c r="G1592" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1592" s="2" t="inlineStr">
@@ -75059,7 +75059,7 @@
       </c>
       <c r="G1593" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1593" s="2" t="inlineStr">
@@ -75106,7 +75106,7 @@
       </c>
       <c r="G1594" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1594" s="2" t="inlineStr">
@@ -75153,7 +75153,7 @@
       </c>
       <c r="G1595" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1595" s="2" t="inlineStr">
@@ -75200,7 +75200,7 @@
       </c>
       <c r="G1596" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1596" s="2" t="inlineStr">
@@ -75247,7 +75247,7 @@
       </c>
       <c r="G1597" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1597" s="2" t="inlineStr">
@@ -75294,7 +75294,7 @@
       </c>
       <c r="G1598" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1598" s="2" t="inlineStr">
@@ -75341,7 +75341,7 @@
       </c>
       <c r="G1599" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1599" s="2" t="inlineStr">
@@ -75388,7 +75388,7 @@
       </c>
       <c r="G1600" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1600" s="2" t="inlineStr">
@@ -75435,7 +75435,7 @@
       </c>
       <c r="G1601" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1601" s="2" t="inlineStr">
@@ -75482,7 +75482,7 @@
       </c>
       <c r="G1602" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1602" s="2" t="inlineStr">
@@ -75529,7 +75529,7 @@
       </c>
       <c r="G1603" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1603" s="2" t="inlineStr">
@@ -75576,7 +75576,7 @@
       </c>
       <c r="G1604" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1604" s="2" t="inlineStr">
@@ -75623,7 +75623,7 @@
       </c>
       <c r="G1605" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
       <c r="H1605" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 20:25:00
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -75022,7 +75022,7 @@
       </c>
       <c r="I1592" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75069,7 +75069,7 @@
       </c>
       <c r="I1593" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75116,7 +75116,7 @@
       </c>
       <c r="I1594" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75163,7 +75163,7 @@
       </c>
       <c r="I1595" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75210,7 +75210,7 @@
       </c>
       <c r="I1596" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75257,7 +75257,7 @@
       </c>
       <c r="I1597" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75304,7 +75304,7 @@
       </c>
       <c r="I1598" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75351,7 +75351,7 @@
       </c>
       <c r="I1599" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75398,7 +75398,7 @@
       </c>
       <c r="I1600" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75445,7 +75445,7 @@
       </c>
       <c r="I1601" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75492,7 +75492,7 @@
       </c>
       <c r="I1602" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75539,7 +75539,7 @@
       </c>
       <c r="I1603" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75586,7 +75586,7 @@
       </c>
       <c r="I1604" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>
@@ -75633,7 +75633,7 @@
       </c>
       <c r="I1605" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 15:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 21:25:03
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -53725,7 +53725,7 @@
       </c>
       <c r="G1139" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1139" s="2" t="inlineStr">
@@ -53772,7 +53772,7 @@
       </c>
       <c r="G1140" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1140" s="2" t="inlineStr">
@@ -53819,7 +53819,7 @@
       </c>
       <c r="G1141" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1141" s="2" t="inlineStr">
@@ -53866,7 +53866,7 @@
       </c>
       <c r="G1142" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1142" s="2" t="inlineStr">
@@ -53913,7 +53913,7 @@
       </c>
       <c r="G1143" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1143" s="2" t="inlineStr">
@@ -53960,7 +53960,7 @@
       </c>
       <c r="G1144" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1144" s="2" t="inlineStr">
@@ -54007,7 +54007,7 @@
       </c>
       <c r="G1145" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
       <c r="H1145" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 21:44:35
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -53735,7 +53735,7 @@
       </c>
       <c r="I1139" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -53782,7 +53782,7 @@
       </c>
       <c r="I1140" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -53829,7 +53829,7 @@
       </c>
       <c r="I1141" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -53876,7 +53876,7 @@
       </c>
       <c r="I1142" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -53923,7 +53923,7 @@
       </c>
       <c r="I1143" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -53970,7 +53970,7 @@
       </c>
       <c r="I1144" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -54017,7 +54017,7 @@
       </c>
       <c r="I1145" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 19:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 23:04:53
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -51281,7 +51281,7 @@
       </c>
       <c r="G1087" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1087" s="2" t="inlineStr">
@@ -51328,7 +51328,7 @@
       </c>
       <c r="G1088" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1088" s="2" t="inlineStr">
@@ -51375,7 +51375,7 @@
       </c>
       <c r="G1089" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1089" s="2" t="inlineStr">
@@ -51422,7 +51422,7 @@
       </c>
       <c r="G1090" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1090" s="2" t="inlineStr">
@@ -51469,7 +51469,7 @@
       </c>
       <c r="G1091" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1091" s="2" t="inlineStr">
@@ -51516,7 +51516,7 @@
       </c>
       <c r="G1092" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1092" s="2" t="inlineStr">
@@ -51563,7 +51563,7 @@
       </c>
       <c r="G1093" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
       <c r="H1093" s="2" t="inlineStr">
@@ -51610,7 +51610,7 @@
       </c>
       <c r="G1094" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
       <c r="H1094" s="2" t="inlineStr">
@@ -51657,7 +51657,7 @@
       </c>
       <c r="G1095" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
       <c r="H1095" s="2" t="inlineStr">
@@ -51704,7 +51704,7 @@
       </c>
       <c r="G1096" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
       <c r="H1096" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-10 23:14:19
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -51291,7 +51291,7 @@
       </c>
       <c r="I1087" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51338,7 +51338,7 @@
       </c>
       <c r="I1088" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51385,7 +51385,7 @@
       </c>
       <c r="I1089" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51432,7 +51432,7 @@
       </c>
       <c r="I1090" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51479,7 +51479,7 @@
       </c>
       <c r="I1091" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51526,7 +51526,7 @@
       </c>
       <c r="I1092" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51573,7 +51573,7 @@
       </c>
       <c r="I1093" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:57</t>
         </is>
       </c>
     </row>
@@ -51620,7 +51620,7 @@
       </c>
       <c r="I1094" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
     </row>
@@ -51667,7 +51667,7 @@
       </c>
       <c r="I1095" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
     </row>
@@ -51714,7 +51714,7 @@
       </c>
       <c r="I1096" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 18:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-11 11:45:18
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -27779,7 +27779,7 @@
       </c>
       <c r="G585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/07/2026 11:28</t>
         </is>
       </c>
       <c r="H585" s="2" t="inlineStr">
@@ -27789,7 +27789,7 @@
       </c>
       <c r="I585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/07/2026 11:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-12 21:46:55
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3359,7 +3359,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>A4763</t>
+        </is>
+      </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
           <t>00019200000013208128</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-12 22:27:31
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3316,7 +3316,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>A3712</t>
+        </is>
+      </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
           <t>00019200000013208110</t>
@@ -3492,7 +3496,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>A4045</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
           <t>00019200000013208152</t>
@@ -3625,7 +3633,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr"/>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>TA1026</t>
+        </is>
+      </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
           <t>00019200000013404830</t>
@@ -4372,7 +4384,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>A9130</t>
+        </is>
+      </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
           <t>00019200000013406213</t>
@@ -5241,7 +5257,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr"/>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>A3131</t>
+        </is>
+      </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
           <t>00019200000013417401</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-12 22:37:12
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -3911,7 +3911,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>A3373</t>
+        </is>
+      </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
           <t>00019200000013404903</t>
@@ -4298,7 +4302,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>A7559</t>
+        </is>
+      </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
           <t>00019200000013404997</t>
@@ -5026,7 +5034,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr"/>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>A5178</t>
+        </is>
+      </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
           <t>00019200000013410350</t>
@@ -5304,7 +5316,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr"/>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>A5654</t>
+        </is>
+      </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
           <t>00019200000013417410</t>
@@ -5347,7 +5363,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr"/>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>TA0370</t>
+        </is>
+      </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
           <t>00019200000013417428</t>
@@ -5390,7 +5410,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr"/>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>A4214</t>
+        </is>
+      </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
           <t>00019200000013417436</t>
@@ -5433,7 +5457,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr"/>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>A2316</t>
+        </is>
+      </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
           <t>00019200000013417444</t>
@@ -5476,7 +5504,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>A2518</t>
+        </is>
+      </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
           <t>00019200000013417452</t>
@@ -5519,7 +5551,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr"/>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>A6207</t>
+        </is>
+      </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
           <t>00019200000013417460</t>
@@ -5605,7 +5641,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C113" s="2" t="inlineStr"/>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>A5182</t>
+        </is>
+      </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
           <t>00019200000013417517</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-12 22:47:07
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5598,7 +5598,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr"/>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>TA0092</t>
+        </is>
+      </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
           <t>00019200000013417479</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 00:17:27
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -50020,7 +50020,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1058" s="2" t="inlineStr"/>
+      <c r="C1058" s="2" t="inlineStr">
+        <is>
+          <t>TA0207</t>
+        </is>
+      </c>
       <c r="D1058" s="2" t="inlineStr">
         <is>
           <t>00019200000013415034</t>
@@ -50920,7 +50924,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1078" s="2" t="inlineStr"/>
+      <c r="C1078" s="2" t="inlineStr">
+        <is>
+          <t>A8808</t>
+        </is>
+      </c>
       <c r="D1078" s="2" t="inlineStr">
         <is>
           <t>00019200000013415239</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 00:27:04
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -50196,7 +50196,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1062" s="2" t="inlineStr"/>
+      <c r="C1062" s="2" t="inlineStr">
+        <is>
+          <t>A9066</t>
+        </is>
+      </c>
       <c r="D1062" s="2" t="inlineStr">
         <is>
           <t>00019200000013415077</t>
@@ -50239,7 +50243,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1063" s="2" t="inlineStr"/>
+      <c r="C1063" s="2" t="inlineStr">
+        <is>
+          <t>A5087</t>
+        </is>
+      </c>
       <c r="D1063" s="2" t="inlineStr">
         <is>
           <t>00019200000013415085</t>
@@ -50282,7 +50290,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1064" s="2" t="inlineStr"/>
+      <c r="C1064" s="2" t="inlineStr">
+        <is>
+          <t>A2955</t>
+        </is>
+      </c>
       <c r="D1064" s="2" t="inlineStr">
         <is>
           <t>00019200000013415093</t>
@@ -51057,7 +51069,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1081" s="2" t="inlineStr"/>
+      <c r="C1081" s="2" t="inlineStr">
+        <is>
+          <t>A4752</t>
+        </is>
+      </c>
       <c r="D1081" s="2" t="inlineStr">
         <is>
           <t>00019200000013415530</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 01:37:27
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -51994,7 +51994,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1100" s="2" t="inlineStr"/>
+      <c r="C1100" s="2" t="inlineStr">
+        <is>
+          <t>TA0322</t>
+        </is>
+      </c>
       <c r="D1100" s="2" t="inlineStr">
         <is>
           <t>00019200000013415042</t>
@@ -52037,7 +52041,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1101" s="2" t="inlineStr"/>
+      <c r="C1101" s="2" t="inlineStr">
+        <is>
+          <t>A3253</t>
+        </is>
+      </c>
       <c r="D1101" s="2" t="inlineStr">
         <is>
           <t>00019200000013415050</t>
@@ -52080,7 +52088,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1102" s="2" t="inlineStr"/>
+      <c r="C1102" s="2" t="inlineStr">
+        <is>
+          <t>A4590</t>
+        </is>
+      </c>
       <c r="D1102" s="2" t="inlineStr">
         <is>
           <t>00019200000013415069</t>
@@ -52910,7 +52922,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1120" s="2" t="inlineStr"/>
+      <c r="C1120" s="2" t="inlineStr">
+        <is>
+          <t>A9483</t>
+        </is>
+      </c>
       <c r="D1120" s="2" t="inlineStr">
         <is>
           <t>00019200000013415247</t>
@@ -52953,7 +52969,11 @@
           <t>PI</t>
         </is>
       </c>
-      <c r="C1121" s="2" t="inlineStr"/>
+      <c r="C1121" s="2" t="inlineStr">
+        <is>
+          <t>TA1219</t>
+        </is>
+      </c>
       <c r="D1121" s="2" t="inlineStr">
         <is>
           <t>00019200000013415255</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 02:57:09
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -5337,7 +5337,11 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr"/>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>A6242</t>
+        </is>
+      </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
           <t>00019200000013404970</t>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 04:46:58
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -26138,7 +26138,7 @@
       </c>
       <c r="H547" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I547" s="2" t="inlineStr">
@@ -26185,7 +26185,7 @@
       </c>
       <c r="H548" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I548" s="2" t="inlineStr">
@@ -26232,7 +26232,7 @@
       </c>
       <c r="H549" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I549" s="2" t="inlineStr">
@@ -26279,7 +26279,7 @@
       </c>
       <c r="H550" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I550" s="2" t="inlineStr">
@@ -26326,7 +26326,7 @@
       </c>
       <c r="H551" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I551" s="2" t="inlineStr">
@@ -26608,7 +26608,7 @@
       </c>
       <c r="H557" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I557" s="2" t="inlineStr">
@@ -26655,7 +26655,7 @@
       </c>
       <c r="H558" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I558" s="2" t="inlineStr">
@@ -26890,7 +26890,7 @@
       </c>
       <c r="H563" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I563" s="2" t="inlineStr">
@@ -27172,7 +27172,7 @@
       </c>
       <c r="H569" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I569" s="2" t="inlineStr">
@@ -27266,7 +27266,7 @@
       </c>
       <c r="H571" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I571" s="2" t="inlineStr">
@@ -27360,7 +27360,7 @@
       </c>
       <c r="H573" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I573" s="2" t="inlineStr">
@@ -27454,7 +27454,7 @@
       </c>
       <c r="H575" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I575" s="2" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="H578" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I578" s="2" t="inlineStr">
@@ -27877,7 +27877,7 @@
       </c>
       <c r="H584" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I584" s="2" t="inlineStr">
@@ -27924,7 +27924,7 @@
       </c>
       <c r="H585" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I585" s="2" t="inlineStr">
@@ -27971,7 +27971,7 @@
       </c>
       <c r="H586" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I586" s="2" t="inlineStr">
@@ -28065,7 +28065,7 @@
       </c>
       <c r="H588" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I588" s="2" t="inlineStr">
@@ -28112,7 +28112,7 @@
       </c>
       <c r="H589" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I589" s="2" t="inlineStr">
@@ -28159,7 +28159,7 @@
       </c>
       <c r="H590" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I590" s="2" t="inlineStr">
@@ -28206,7 +28206,7 @@
       </c>
       <c r="H591" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I591" s="2" t="inlineStr">
@@ -28253,7 +28253,7 @@
       </c>
       <c r="H592" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I592" s="2" t="inlineStr">
@@ -28300,7 +28300,7 @@
       </c>
       <c r="H593" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 04:28</t>
         </is>
       </c>
       <c r="I593" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 07:37:08
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -58649,7 +58649,7 @@
       </c>
       <c r="G1239" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1239" s="2" t="inlineStr">
@@ -58692,7 +58692,7 @@
       </c>
       <c r="G1240" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1240" s="2" t="inlineStr">
@@ -58735,7 +58735,7 @@
       </c>
       <c r="G1241" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1241" s="2" t="inlineStr">
@@ -58778,7 +58778,7 @@
       </c>
       <c r="G1242" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1242" s="2" t="inlineStr">
@@ -58821,7 +58821,7 @@
       </c>
       <c r="G1243" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1243" s="2" t="inlineStr">
@@ -58868,7 +58868,7 @@
       </c>
       <c r="G1244" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1244" s="2" t="inlineStr">
@@ -58915,7 +58915,7 @@
       </c>
       <c r="G1245" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1245" s="2" t="inlineStr">
@@ -58958,7 +58958,7 @@
       </c>
       <c r="G1246" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1246" s="2" t="inlineStr">
@@ -59001,7 +59001,7 @@
       </c>
       <c r="G1247" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1247" s="2" t="inlineStr">
@@ -59044,7 +59044,7 @@
       </c>
       <c r="G1248" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1248" s="2" t="inlineStr">
@@ -59087,7 +59087,7 @@
       </c>
       <c r="G1249" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1249" s="2" t="inlineStr">
@@ -59134,7 +59134,7 @@
       </c>
       <c r="G1250" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1250" s="2" t="inlineStr">
@@ -59181,7 +59181,7 @@
       </c>
       <c r="G1251" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1251" s="2" t="inlineStr">
@@ -59228,7 +59228,7 @@
       </c>
       <c r="G1252" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1252" s="2" t="inlineStr">
@@ -59275,7 +59275,7 @@
       </c>
       <c r="G1253" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1253" s="2" t="inlineStr">
@@ -59322,7 +59322,7 @@
       </c>
       <c r="G1254" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1254" s="2" t="inlineStr">
@@ -59369,7 +59369,7 @@
       </c>
       <c r="G1255" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1255" s="2" t="inlineStr">
@@ -59416,7 +59416,7 @@
       </c>
       <c r="G1256" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1256" s="2" t="inlineStr">
@@ -59459,7 +59459,7 @@
       </c>
       <c r="G1257" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1257" s="2" t="inlineStr">
@@ -59502,7 +59502,7 @@
       </c>
       <c r="G1258" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1258" s="2" t="inlineStr">
@@ -59545,7 +59545,7 @@
       </c>
       <c r="G1259" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1259" s="2" t="inlineStr">
@@ -59592,7 +59592,7 @@
       </c>
       <c r="G1260" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1260" s="2" t="inlineStr">
@@ -59639,7 +59639,7 @@
       </c>
       <c r="G1261" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1261" s="2" t="inlineStr">
@@ -59686,7 +59686,7 @@
       </c>
       <c r="G1262" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1262" s="2" t="inlineStr">
@@ -59733,7 +59733,7 @@
       </c>
       <c r="G1263" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1263" s="2" t="inlineStr">
@@ -59780,7 +59780,7 @@
       </c>
       <c r="G1264" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1264" s="2" t="inlineStr">
@@ -59827,7 +59827,7 @@
       </c>
       <c r="G1265" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1265" s="2" t="inlineStr">
@@ -59874,7 +59874,7 @@
       </c>
       <c r="G1266" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1266" s="2" t="inlineStr">
@@ -59921,7 +59921,7 @@
       </c>
       <c r="G1267" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1267" s="2" t="inlineStr">
@@ -59968,7 +59968,7 @@
       </c>
       <c r="G1268" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1268" s="2" t="inlineStr">
@@ -60015,7 +60015,7 @@
       </c>
       <c r="G1269" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1269" s="2" t="inlineStr">
@@ -60062,7 +60062,7 @@
       </c>
       <c r="G1270" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1270" s="2" t="inlineStr">
@@ -60109,7 +60109,7 @@
       </c>
       <c r="G1271" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1271" s="2" t="inlineStr">
@@ -60156,7 +60156,7 @@
       </c>
       <c r="G1272" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1272" s="2" t="inlineStr">
@@ -60203,7 +60203,7 @@
       </c>
       <c r="G1273" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1273" s="2" t="inlineStr">
@@ -73515,7 +73515,7 @@
       </c>
       <c r="G1561" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1561" s="2" t="inlineStr">
@@ -73562,7 +73562,7 @@
       </c>
       <c r="G1562" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1562" s="2" t="inlineStr">
@@ -73609,7 +73609,7 @@
       </c>
       <c r="G1563" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1563" s="2" t="inlineStr">
@@ -73656,7 +73656,7 @@
       </c>
       <c r="G1564" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1564" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 07:47:12
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -58878,7 +58878,7 @@
       </c>
       <c r="I1244" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -58925,7 +58925,7 @@
       </c>
       <c r="I1245" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59602,7 +59602,7 @@
       </c>
       <c r="I1260" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59649,7 +59649,7 @@
       </c>
       <c r="I1261" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59696,7 +59696,7 @@
       </c>
       <c r="I1262" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59743,7 +59743,7 @@
       </c>
       <c r="I1263" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59790,7 +59790,7 @@
       </c>
       <c r="I1264" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59837,7 +59837,7 @@
       </c>
       <c r="I1265" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59884,7 +59884,7 @@
       </c>
       <c r="I1266" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59931,7 +59931,7 @@
       </c>
       <c r="I1267" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -59978,7 +59978,7 @@
       </c>
       <c r="I1268" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -60025,7 +60025,7 @@
       </c>
       <c r="I1269" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -73525,7 +73525,7 @@
       </c>
       <c r="I1561" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -73572,7 +73572,7 @@
       </c>
       <c r="I1562" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -73619,7 +73619,7 @@
       </c>
       <c r="I1563" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -73666,7 +73666,7 @@
       </c>
       <c r="I1564" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 08:38:02
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -88186,7 +88186,7 @@
       </c>
       <c r="G1874" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1874" s="2" t="inlineStr">
@@ -88233,7 +88233,7 @@
       </c>
       <c r="G1875" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1875" s="2" t="inlineStr">
@@ -88280,7 +88280,7 @@
       </c>
       <c r="G1876" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1876" s="2" t="inlineStr">
@@ -88327,7 +88327,7 @@
       </c>
       <c r="G1877" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1877" s="2" t="inlineStr">
@@ -88374,7 +88374,7 @@
       </c>
       <c r="G1878" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1878" s="2" t="inlineStr">
@@ -88421,7 +88421,7 @@
       </c>
       <c r="G1879" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H1879" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 08:48:01
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -1609,7 +1609,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11/07/2026 15:00</t>
         </is>
       </c>
     </row>
@@ -88196,7 +88196,7 @@
       </c>
       <c r="I1874" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -88243,7 +88243,7 @@
       </c>
       <c r="I1875" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -88290,7 +88290,7 @@
       </c>
       <c r="I1876" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -88337,7 +88337,7 @@
       </c>
       <c r="I1877" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -88384,7 +88384,7 @@
       </c>
       <c r="I1878" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>
@@ -88431,7 +88431,7 @@
       </c>
       <c r="I1879" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 09:09:08
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -33790,7 +33790,7 @@
       </c>
       <c r="G710" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
       <c r="H710" s="2" t="inlineStr">
@@ -33837,7 +33837,7 @@
       </c>
       <c r="G711" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
       <c r="H711" s="2" t="inlineStr">
@@ -33884,7 +33884,7 @@
       </c>
       <c r="G712" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
       <c r="H712" s="2" t="inlineStr">
@@ -33931,7 +33931,7 @@
       </c>
       <c r="G713" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
       <c r="H713" s="2" t="inlineStr">
@@ -33978,7 +33978,7 @@
       </c>
       <c r="G714" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
       <c r="H714" s="2" t="inlineStr">
@@ -34025,7 +34025,7 @@
       </c>
       <c r="G715" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 08:00</t>
         </is>
       </c>
       <c r="H715" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 09:18:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -33800,7 +33800,7 @@
       </c>
       <c r="I710" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -33847,7 +33847,7 @@
       </c>
       <c r="I711" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -33894,7 +33894,7 @@
       </c>
       <c r="I712" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -33941,7 +33941,7 @@
       </c>
       <c r="I713" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -33988,7 +33988,7 @@
       </c>
       <c r="I714" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 10:00</t>
         </is>
       </c>
     </row>
@@ -34035,7 +34035,7 @@
       </c>
       <c r="I715" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 08:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 12:11:28
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -4325,7 +4325,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/07/2026 17:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza dashboards Aura - 2026-07-13 13:29:30
</commit_message>
<xml_diff>
--- a/relatorio_analitico_vtcbox.xlsx
+++ b/relatorio_analitico_vtcbox.xlsx
@@ -55514,7 +55514,7 @@
       </c>
       <c r="I1172" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55561,7 +55561,7 @@
       </c>
       <c r="I1173" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55608,7 +55608,7 @@
       </c>
       <c r="I1174" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55655,7 +55655,7 @@
       </c>
       <c r="I1175" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55702,7 +55702,7 @@
       </c>
       <c r="I1176" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55749,7 +55749,7 @@
       </c>
       <c r="I1177" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55796,7 +55796,7 @@
       </c>
       <c r="I1178" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55843,7 +55843,7 @@
       </c>
       <c r="I1179" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55890,7 +55890,7 @@
       </c>
       <c r="I1180" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55937,7 +55937,7 @@
       </c>
       <c r="I1181" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -55984,7 +55984,7 @@
       </c>
       <c r="I1182" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13/07/2026 13:00</t>
         </is>
       </c>
     </row>

</xml_diff>